<commit_message>
Clarify context budgeting and refresh all live sample reports
</commit_message>
<xml_diff>
--- a/reports/claims_context_managed/report.xlsx
+++ b/reports/claims_context_managed/report.xlsx
@@ -165,7 +165,7 @@
     <t>Run ID</t>
   </si>
   <si>
-    <t>01a0cc56-1873-7b63-b513-657d1eef7154</t>
+    <t>01a0ccdf-b7b4-7282-a01f-e7dd9f070b7d</t>
   </si>
   <si>
     <t>Recording</t>
@@ -183,7 +183,7 @@
     <t>FX fetched at</t>
   </si>
   <si>
-    <t>2026-09-23T03:35:56.284466Z</t>
+    <t>2026-09-23T06:06:28.037095Z</t>
   </si>
   <si>
     <t>UTC</t>
@@ -306,7 +306,7 @@
     <t>gpt-5.6-luna</t>
   </si>
   <si>
-    <t>01a0cc56-187b-7450-ad6e-21c96db9718a</t>
+    <t>01a0ccdf-b7bb-7643-9f73-5583342bd8b2</t>
   </si>
   <si>
     <t>Fresh input</t>
@@ -357,8 +357,8 @@
     <t xml:space="preserve">    Output content</t>
   </si>
   <si>
-    <t>[{"id": "rs_0845e0b9ad7ff9fc006ab3493e6b7487d288af70c2a616db12", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs0k-fqX2q8DHlb0ME0Q0fMJGVmPQ_qEEZS1gnrfn6rFBgS2IsO-NdrNLlvGzdG_QwDvfV_Ep4sN0Dpr0FRne2X-DUe-m1f69kIIX-pSBRwhK4t_pCdxyL2Nh9nlIh1YScIFYyTsEK3F1K6jt_-0goHzrKrS7kbrEaxgmPzGpB4y2AjqsydJD3Ymw0swtEHE7KpoLOAaYXldkjITKPqAKOgUydbrKWY6PcANFn6Le_4Sews8J8EfKAskzFrv3ARDzYE6_DWePDIfsPVX8MExHpOalx2zs27tNMQPBLPw9j8E4t6P55s7Lj6R2yBTvK1zieZ_72IjiMiSbEZj2tru59sGBnmzXK8zZclaor8mdlJonvoa73u0NlvdvJvdUHedpLdRQLEv8AIShrNymoGf9LzMawCtyjJrXxgV5XOw_3RLzyYmjCT2WDFrzdYXTwE6RVwkLLuWBJtVPiHFsBoYNosatbVGCfKbwSvrIG9VUdHKpUDRgCf497Cls4_fy7XA6tLGtnSaKmlUF5dx9NSfv_StiKhWv7uzTdA6-4xHuNlIkndlGcGqLbLWYLilhYymVGsh93-al6WyXDQYJJNHn1OXJt8WavwpDbjS9qhYVVLqgm4c77ZU0IbzcFH0MyUu3Wvw5E6lj9lWYIQiy4DeWBVTFxj67BtT7XflV68hXWhE3UWNFWXa0yiK-kt5liLHHgAow0slTmlFGnUIP0GDhEJ8gqLezGC3ZDKOHFa0pcCBkq-fBe6b4vNQHHlDbd4BCeIPqXXaTkoS_TkroqYoUO6QZUUcfRpCqZcg3uD762EkVK2--uzYLLkOBFECAf7DAQ87TeSleMMyZ6scupb_lVeVp_R1EB1oD8KiWt5Roj-eyDmMeah9EmtPf3jnzCc2J67KlRZJQogD1dEDTUrFc295pQr-84srfituXnI0KUp0blIxqWh9xc5ILHXuUR_4_UCvfJJjbyb88RhK9JdNKLzwaHcgfDePZs0OWuq6iJnXs2ngNEGgjwalR98uIMI5rx8tJGWxthaD0AZPeJp-CGZykA5TV7_BmLQu68HyuNkkQjns1CaQgjE7DN-Qb_re8dt_peMtfwE7dFNxxU8ufviONHzqxyfhpCSd9-CtMUUCC_3GZAZSOIDpiMh3xOr607qp47pqYxLMr73vaYQBp6S3mwDDOZxdCAApaEDkhHXw-SoeAZ9lv4Hxbmxz0dAfwSv9N"}, {"type": "function_call", "name": "read_policy", "arguments": "{}", "call_id": "call_XUipt02G1LDasiRER2p424ec", "id": "fc_0845e0b9ad7ff9fc006ab3493e972887d2af12d65aea0ebd1e", "index": 1}]
-{"name": "read_policy", "args": {}, "id": "call_XUipt02G1LDasiRER2p424ec", "type": "tool_call"}</t>
+    <t>[{"id": "rs_08acf24a3e239f6a006ab36c795cb087d28ebbb1d47994f32f", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x5_Wgphp9Sf8NFOLXYsJNwFrOGSvHpwsXSNNJrZbRlaAdLrEIv2LZc7i3SZshIgBijJJPSCWpWKgvmqyjAB3-y4Bg0ZPyuHNtAcM_8iEjFKxvq0ZoUyq0fyPRacA8au8U4Na_TujB9F93P5gz0vbBPiRTtbsKx8OToiBd2id6X5vKBSOYYj4HAQqdy_GieOrYoFZcUAOghheMqZCQv8LYiGxh1KHnZKAFfg0oyopHuWw7W79VDqhoIcXF3JdEU1l3Bh3vLFVTAFAvNeeGXsA_nTWbeYOJ-opbm6Pl2BrNjBQRorbv8MJv-3pzGu0IG8CnCVEM-ja7BCwm-0lh5n5xpYLSHb-Zb11OccCrrts9I3aFpTVcbS8P8GKKjpVr5ySUKijGaY_VZIb7_dDtAiBbiuY4PI3SFl4KsaFtwKfeLj5do8Wx49KM7OlFHQrWMpbWcYsq5smhis-Loc3u05QeLqAJbxv-K37r3O_rrNHA_Xh77QSq75XdwpGsBWObENsaC4w7M4SCZVnZAiPhS4eixcQiRmcC1aqEpSjADyUZPVXnV8HYBQnKPpr_A71TXqfbOxjvNsrHHx3xYfy_ihIXIKGhRqHTFKd9EqZjA4GTS7CtFbJelrlur9jMOyb30CV2VAsZQL9gMA1d3lEhnTl_QsvH8b_l8OCaZOLGBY7wYVQlOEMG465esivFJndemdcVqe0LzW2_NKmS7lOHzqmiORe0rMZmlr1ZOQBTpAQClpghkdO6XpL4tOlSlB157f6G_eUyQy1MB8GACtlNYKfvCCNjzPQZHgRbd3iGHf6GABuMDnmPOx-S3Y1595G5mq4nrMXq2HQJGShD7hn1JfERyQDLK6F-g3FR8muhl57akKzZcqW0I4_lhw3swc6-p0A4oU9TAlTTOriJFXRmk2V2gNvNwXtCW2WtjmqhnPpdTgQZYN3lMqQZKKAMezRuuOJ-af_uAn1a4o4JTumnZSqj_HJvXjX2ln9fIrG8Uz1LVREi8qaaJKG6srgCda-WQnUcn_aWgU5zcPYwDQIA_dJobLTEp_u8TWcMeZrd8PTm77BJJHMW4i2WnAF_xFWb3xwBA5KpoylSeq7IT-b63ZKpFV-gtbSwxR_us3NS26IgnzJDy9TtfLfYK1h9Acpb1b8-3lD24Mb9-Xf2FUR2IIMrscjyVSUSCBhOR9xZxQVyCCDdprRg7x5E_PAkJB0vdmRET"}, {"type": "function_call", "name": "read_policy", "arguments": "{}", "call_id": "call_KpG3hBdlMxiECjhYb4CXiCnZ", "id": "fc_08acf24a3e239f6a006ab36c79963087d28b6769ea89a88da9", "index": 1}]
+{"name": "read_policy", "args": {}, "id": "call_KpG3hBdlMxiECjhYb4CXiCnZ", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Call total</t>
@@ -370,7 +370,7 @@
     <t>Tool · read_policy</t>
   </si>
   <si>
-    <t>01a0cc56-1dab-7da2-8312-b16f074b8a76</t>
+    <t>01a0ccdf-bc28-74a1-9d0f-67b8c1faddaa</t>
   </si>
   <si>
     <t xml:space="preserve">    Arguments</t>
@@ -388,7 +388,7 @@
     <t>R2</t>
   </si>
   <si>
-    <t>01a0cc56-1daf-7261-b469-e39f85795d01</t>
+    <t>01a0ccdf-bc2b-72c0-88f0-5490bade1f97</t>
   </si>
   <si>
     <t>Conversation history · cache read</t>
@@ -397,7 +397,7 @@
     <t xml:space="preserve">    Tool result</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "Policy POL-001 has a **CAD 150 deductible** for accidental laptop damage.", "phase": "final_answer", "index": 0, "id": "msg_0845e0b9ad7ff9fc006ab3493f7d8887d292cab85da7025e32"}]</t>
+    <t>[{"type": "text", "text": "Policy POL-001 applies a **CAD 150 deductible** to accidental laptop damage.", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c7a8ae487d2a2bed20de84b96d9"}]</t>
   </si>
   <si>
     <t>Turn 2</t>
@@ -406,20 +406,20 @@
     <t>R3</t>
   </si>
   <si>
-    <t>01a0cc56-217d-70c0-8d7a-fc2a6c3b8206</t>
+    <t>01a0ccdf-bfdf-7370-a947-75db376a8377</t>
   </si>
   <si>
     <t>What happened in claim CLM-001, and what is its status?</t>
   </si>
   <si>
-    <t>[{"id": "rs_0845e0b9ad7ff9fc006ab349410b1087d28c1447f6e57e1c28", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs0lBNTEfcdLf4nsExQtpQ6UHRNyUC8tJSW4c04ShL_DqlvbikP3NjehCYawKSoDTUDdSuipkzfxHJc_BU7xJEAT2zFXeuIKRHOJMrq00HSfVGjge-Sn9CoiY75Hh12EWQ9o9-XQEGM1uFxsrmEh5JFpsSK3ljhATe4Lk2WWtxK16aC9vgdZLbtDousyQutIgLJONlTMtnPECH71pF5MzI8T3YQvsgxlTwiCKeLRsMWSn1QfEMD08F5Cy7zX_oNQ1AiiBsaHTbFV-hOYHFLL3YiOr_VKrxNpmsTUVXrN0Fs3QlDJL8XeX1POS9w_WQTVdkCMEiRlzJbr_DBiZevhUh1aTTm1eQ2XbEOcYxXGEdkY-IzxfhE8e4kYvrcs2Hl8deHlVgi3xpbL6cmOzpZx-o1LkXEu41Lmu2d738oQtzIApf-ojdMi5foatjURUfvT34ZFjwEOWydHygEK02pBuJMFr0zszGUUsRNXBpoBfMKKcoDR6OArjgEEOOMj1BWIZUPaNkJ8zPSGAraeRXGsYzD1_dxUYFl9AsonzTA82CzBLZeYxSMoU9l0pmIZGjdBDis6jmsei8U2sQ0HJYxCs7GrrGw682rOdQmC9VNIvIH4YU1qSPv9xCD172sZjDvY2M-hCtQAoYmG3WQawHR47xiyji3EESbWoS2PegTjB5zEDd_W-0C17tqe05SM7GRejCpwHiZkY6TSXnMWcYzLsHA2DqS2zPqbJNO8tYe78j_mxpCpQYFBBis1CqGBmEIO_h9nZ1IiZeWBeSVmfnx49e1ngDmDn3oQg-FzSOo3bmTyh44RmckZqTMViDUmssmhj10IbIDaz5mUKJmqBYyCscg9lPuhT2THL86HTl5KPm5hLZDuFdEGZlc2dsSeF7n7GSuwNI8H96fts5gc3oJrANWcAOzWi8PucI41BspGrSxUotHIGP1CtpPDbJOZoSZPtM9sLeFtDNWXYDn9bsnyFMOYCK9WMLQdk7Lm935twiLm-LVzlnZIPzlwFQ4ZSHlYxFp7002rk7TMHK1_vhOWGJATEAcW2Bpn_hLHtOSRPS5OShTLVjMqyjVYhPRUTEfu5AXs00fQkbnO2BS6MTx23pGa5oQW12578CUTYCLzd_Ajf24zsXSZqFRmYvnadf-R-sCFZPxiCG6GUEr3CCGutvdVI5oEqIxP9uQjnShIuvzo796OWQDOwNgjh0OPWmeYUdouE"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_J1dQcfiaSTomTKu6AEjdZ7e2", "id": "fc_0845e0b9ad7ff9fc006ab34941261487d29582261ff0ebf3a4", "index": 1}]
-{"name": "read_claim", "args": {}, "id": "call_J1dQcfiaSTomTKu6AEjdZ7e2", "type": "tool_call"}</t>
+    <t>[{"id": "rs_08acf24a3e239f6a006ab36c7b6b1c87d298298a6c599f981d", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x7y1_D29XwcxpNBCWtwTjbHl126ixQ1Vy0A_gmMEggm99GUqg7KwDS7Xpkev-Uup9_LRQ_-WQP9avAuzN89L2vMWtLdvDrZvZiowgpwN5eAfizhKpLgjc3vVU1ThawGCO0eX6DIKDM9nOh4is8Dyt2AkM7Ux1UcTLvm1UgW2iJdXG1PyurLpied_NYuaSEzh3gtlhx5w1YBzdwMGBRVgyA0aS8T8IYIQsOo-oP1dODeGCyMoH88acRxYkUCIqgfyqTpczzaPmqdvOKsyiMjo3uTq_vdCaDJgrpxFijwxXixXO5tGzP5BPCr92Pg0Ap2VUJ7dKNWVwli-0VSkQbZyFXC0XCuG-sydsYvcTo_dJcB3z7HzRE9P1Ade4GPfMtBoq3earqeK1aafwu2798jo1ILDwx-uDh0ADwqSQzcwb5fdcrkRaEqoEI2ElxW2n4nfKoskbkFTejjCW46yIsNdC3YC3cqgaqmoAq7kOoTMYt1XuOtVMz8rXzKG0JVNGoW9HDe_cmBFg5dX7o-XVdvvS0FmkE56YQQJNRwcWiObNegnoH_uuSopRG9Wl3q4rnZOrZDFGTyFOKTs0MwBFpLAsu3Dfrak3BUfCL12aG0Uou2RXajjQT3O4UmIorpS6tBYq94m7NpAlK_t4hYEmvvpZaotxBV1AMT00RlS4pOf4D1ioFbnW8PF1XNEL5EG1Z3AkoFBzeBjkuJHZgynw2cLtlZyCMh74-ZlYE4LI7bdwLLfiuhrfwhPUIWwe3xtd0QV9_zpxBDCCfulN4GPz7oE6CdTNbfk88UOBo1_hI46zZM-MGTuDckg0GjKO4y8zJ4lIgsUAfN8ishSxhie4zc0mlnAiy2WzA2ktluANdt4uNk84hXyGghThjuOS8HentlSMnCBnUxakBXYKZ0exgIDUZewT0_1DDGIxUcOijy3XyqtcFC9yBuq2nypj2qT9zFld8J7vHnjTDiNs7Y_tGVGZhGiqxw16Pw4Rv_pjT5NIOSQBQx4HDJLMcwjaxlumHHPyZNu6rDsFIPs8LFioOulPF6_kVcNf46GVHL68ZGj8lrbktNs0-_0jjTvfQ8RSmJlVrx90vvKSYKb3UkqBNj1h_d0_2VAzH7_qEDGGBoqfhTbg1QL-NuNe3a45gOs1HYuv_WFgbsJwlhax7oQl91IWudRhdGwsIp7pPZKNCgY39IuD4jI-IR3Ju9Mu372ceADvM"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_78AYLUwYWh6NWaqvO8hpsVMS", "id": "fc_08acf24a3e239f6a006ab36c7bced487d2b2a1a89aa0a6b9ac", "index": 1}]
+{"name": "read_claim", "args": {}, "id": "call_78AYLUwYWh6NWaqvO8hpsVMS", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Tool · read_claim</t>
   </si>
   <si>
-    <t>01a0cc56-2774-7091-bc9e-a071006d24fc</t>
+    <t>01a0ccdf-c7a7-7571-982f-202ee708c675</t>
   </si>
   <si>
     <t>{"claim_id": "CLM-001", "revision": 1, "description": "A laptop was stolen from a parked car.", "status": "pending"}</t>
@@ -428,10 +428,10 @@
     <t>R4</t>
   </si>
   <si>
-    <t>01a0cc56-2777-7c40-9613-b1f1b808c3de</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "Claim CLM-001 concerns **a laptop stolen from a parked car**. Its status is **pending**.", "phase": "final_answer", "index": 0, "id": "msg_0845e0b9ad7ff9fc006ab34942267c87d2a9fc08e8719e54f3"}]</t>
+    <t>01a0ccdf-c7aa-7073-9062-c33e52e5abcc</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "Claim CLM-001 concerns **a laptop stolen from a parked car**. Its status is **pending**.", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c7d6c7c87d2a3a592be1fba4fe9"}]</t>
   </si>
   <si>
     <t>Turn 3</t>
@@ -440,20 +440,20 @@
     <t>R5</t>
   </si>
   <si>
-    <t>01a0cc56-2c1d-7981-9d77-dee15d4e046d</t>
+    <t>01a0ccdf-cbc9-71c2-bf15-0ce6b5568029</t>
   </si>
   <si>
     <t>Correct the claim: the laptop was not stolen. Its screen cracked when it fell from a desk at home. Replace the description with 'The laptop screen cracked when it fell from a desk at home.' and change the status to approved.</t>
   </si>
   <si>
-    <t>[{"id": "rs_0845e0b9ad7ff9fc006ab34943387c87d2a7c04407216396d2", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs0lDovynfsRUfATQPk5MwOP6Q1a5st00oE4e6eIB7j7XLvSdnN8dqOhgc3dkybQGF2SkzzgG41e-FjFzk5Zsf0hP0-YzkFP7kIoMAedw44lfPEXBJCaBsQOm4WWTJAyZxLa_kFU-1n-NdlAcOpOLGtGuGA3X9NvuH1s1rDp-EXDf8X7PxM36Ud4y_K9hWFZCW_d2Ud_a_DmkkKeYMcYN4V6D0P-0np4tJFRBxKEzFpgld-l0g7UGVAuq6Gz4CXYxIqqX5s6kJzxd84NT4WZbDkynYv9-r8pLpNThqwA0Mvd0fMcDa0PKoXgyVA1TtDj_TSyXEGOqlIKVXSbB47MCODpzDH35DUVb8owNzDciW2jmreFxoN5Dc-WcruU1a176R2BqhJptaQsLEexSBWaindcn3jiyMydqiSgC-ajKIAZHSwCCG3RTpZqGyr8YKmBHgUIiN4MJOMLaES97D7W_4mAnfsinGRoeyhoc4v0VKkalRAsBtr6KpZLT2p8d0BXX6rZWYckQblVPYu_dDSapOGb4mL5yytD7vnyyB0qe8QBNxawU0B33B3DW925Ojx-f10HhOlZM0Q33GjcAfgP9PX04u8WVhuq1o8WBl8YFLY8ERxPNV_sfYOzMsYKootJCJfeADltXDC5V7rSYFK4euzq5RQQa1UrrOiGKyN0pH-mO-VIAZofarzpYzO4aXrG78PJHwlYz-gV5ok5Lr5GyraqcuMCBJcpcYO0J9P1qYLIgO_L9VZTrKVTnPL1iLPk_NI78UcgxikJU_cZW4sdhbC_hkpyBeNBlCD1MEhsU57qJ_HVLNjQY988udQcn5Nxle9XPKGF6IJhkcR5yXq-9MF2NwfVFZ_D08CbYZf7EtDJmtvc-MaAd1siz5mGMZ-MoMoVXotbPYKUUDnJeq2RJ3B-T28cxMY7OKvhqtTTak7Mrnkr3aT8L_KT96XfcQRA2QfSLuBl1htzVesMIdhxOwV1yYG5L1DA5Mv-LvkWVrpFWnOLEZgMVTFXKSwTExXRPScEq7qywWr0nCiBi5aSEyiVmucVRfOWWO7gX0WlOpl3hPWnRrzg44muwur2QmrwHKDq7jNLjYfjS3jQeOvKhy0z3cpayUwhsIWfKtoGpuPSPr7o8UzkVhc3ToJ6OHjwZYNxAxF3UOiq1LdP3NQWLKToLwmeIQpuoV_xbzjHeIG_k88xAdbmapjE1k7zajALAOnsH"}, {"type": "function_call", "name": "edit_claim", "arguments": "{\"expected_revision\":1,\"description\":\"The laptop screen cracked when it fell from a desk at home.\",\"status\":\"approved\"}", "call_id": "call_N7YRgMtLrDmZpNilLwOcY7Fm", "id": "fc_0845e0b9ad7ff9fc006ab34943681887d2b8d04d34f5245077", "index": 1}]
-{"name": "edit_claim", "args": {"expected_revision": 1, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}, "id": "call_N7YRgMtLrDmZpNilLwOcY7Fm", "type": "tool_call"}</t>
+    <t>[{"id": "rs_08acf24a3e239f6a006ab36c7eca4887d2b43c97c61c8f7a94", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x_jYNbPJ18Vz45kZQLd0QPFXPKxTnH0RqCGG4eb9Ir4lwm3Z1gwvhHt-L_bONsAHnc0-nwLsaD8MGIONU8kuaVa9_cVHlG77yoo0XjeU8xwhJz6-019Y4TUMBheHwGT4PL-JeHvVDeMrKxmAC4PxYSqjvCnjdSGcDfEsrx7_bZxG6j8L4tjvIUEg5alFHbg5i5Cwssirjt_Kx-Zs59D6Sv09C7WEjEYoEt7pwQZtRQUWzjMYo6Ha-PShe3Bm18-2sUnHKC4_ilSKhF1euFW4ngCEAdK7e-NzgK5z1Cc6ZsgR08VZdDpsg2x8lpX0_sgxs-4lx7jcq_q_bmSpdNzMf4hykh0UUVo0rneMqNNkk8cRLFGauha69TC333MA7YcGOcvHHqvSWwDw5jTPNBQs38Ce-GDSbZePt4le9qwU60_L53xH6baWrc6c4o2ACOIWZl6U7hB7nYOti3pwWCQEXvJJ26s-QrqYApgaKPqIoKDe48GcHwyYxh364To-3yM7Omp-LFbxVy0pFvkGxbOsbqdFWkQpDe9_XCDUizpT4MT_wH9hd_CwV972cSB5Z2rXrpxlyiO_d3Um0iAcjOw4t0Q_AxN-Yfg9hY9BiDl-RVkZFSMDCdtczcf61ozbC-hUz78P4hFxts9ShXrg0Cii2MVaigtI9NJaHyG9HKNO0oJfx47KvgNIgNRwntMoWF4gvdyKbekpXY-bx_kN6vq0fDayWJtEmeaGO1YeyYl_bGFWlzMKdBX4rLstK0UlUX8N-40lGkxAB7Ql2ITfrHmQJHwj6v5G1skKuIgLvpkmlDX-n26trlATBqr1py6OcoHxx9fhMFjFOA4bOKNCAjFEzhn5GDyGOnyH3VShOgubn3BBAGnGgz7Z_bvrJmRRaer1s9vyy9RLgHpG6RblCZYDk-GpHeq2JTJF1vUAaYPYXkLioIxwMocNbcNZ8nTC2KHbHwhQq4A_AWwaZAl5inh9SwaT5xB1EMuNCdRdhge2h6PhvN7MzUbt1K_2UkyScN2PvsDe5Ak84rCxsPEKzV9f83m768HugqTwSkygp6X7xUAv51f7JVAFUmVXpWlm4pc4eHqA5dhMmKjvVtE0KlLd2cIPsfFxCrnby4ysuN6fSxroK9jYqQt608-N7dw9GmQLpxb6dGaO4avTqCxzGZC3jsL9XM0mIC3FFFWhrB8k4T1DSe94FGHxXK0pPd97E9_Ce3fFVjoFl43XOqQmvvnSzK8zEV5jyFTit3JCB_g_Sl02TqBbfbY9u8FYyD9zMmb3tR"}, {"type": "function_call", "name": "edit_claim", "arguments": "{\"expected_revision\":1,\"description\":\"The laptop screen cracked when it fell from a desk at home.\",\"status\":\"approved\"}", "call_id": "call_dYUixnYLB2nLVku0kx5CQMiT", "id": "fc_08acf24a3e239f6a006ab36c7f120087d2b40371b1dfbf91da", "index": 1}]
+{"name": "edit_claim", "args": {"expected_revision": 1, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}, "id": "call_dYUixnYLB2nLVku0kx5CQMiT", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Tool · edit_claim</t>
   </si>
   <si>
-    <t>01a0cc56-3056-7ae3-9a71-ff6d3f8d6e80</t>
+    <t>01a0ccdf-d312-79a2-aa4d-ed292e67dfc9</t>
   </si>
   <si>
     <t>{'expected_revision': 1, 'description': 'The laptop screen cracked when it fell from a desk at home.', 'status': 'approved'}</t>
@@ -465,10 +465,10 @@
     <t>R6</t>
   </si>
   <si>
-    <t>01a0cc56-3059-7f32-9aa1-e9ef8816a456</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "Claim CLM-001 was updated:\n\n- **Description:** The laptop screen cracked when it fell from a desk at home.\n- **Status:** Approved", "phase": "final_answer", "index": 0, "id": "msg_0845e0b9ad7ff9fc006ab34944691487d2877481e37c81ea6d"}]</t>
+    <t>01a0ccdf-d315-75f0-9854-d36f955026cf</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "Claim CLM-001 has been updated:\n\n- **Description:** The laptop screen cracked when it fell from a desk at home.\n- **Status:** Approved", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c81184087d28244d716be6b3c6c"}]</t>
   </si>
   <si>
     <t>Turn 4</t>
@@ -477,13 +477,13 @@
     <t>R7</t>
   </si>
   <si>
-    <t>01a0cc56-3529-7fa3-aff5-4e8792088317</t>
+    <t>01a0ccdf-da76-70c3-baf0-d4bbf09f4104</t>
   </si>
   <si>
     <t>What is the policy's coverage limit?</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "The policy\u2019s coverage limit is **CAD 2,000**.", "phase": "final_answer", "index": 0, "id": "msg_04b0a37d493a2c8b006ab34945aac087d2a332f425fd659e8e"}]</t>
+    <t>[{"type": "text", "text": "The policy\u2019s coverage limit is **CAD 2,000**.", "phase": "final_answer", "index": 0, "id": "msg_0a7a88b94261cb0d006ab36c82409087d284ba98eae380acdb"}]</t>
   </si>
   <si>
     <t>Turn 5</t>
@@ -492,17 +492,17 @@
     <t>R8</t>
   </si>
   <si>
-    <t>01a0cc56-39f3-7961-8e17-8e393b66a443</t>
+    <t>01a0ccdf-de67-7a20-be6e-34860eeda2e5</t>
   </si>
   <si>
     <t>What happened to the laptop, where did it happen, and what is the current claim status?</t>
   </si>
   <si>
-    <t>[{"id": "rs_04b0a37d493a2c8b006ab34946dca487d29845e3da104944d7", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs0lHZtgKgaC5wWomLUrnT_dsxxIw6HILy38OOnipTtGyDRNeeOgkUgB2xnpUkt5eu4qq31hmjNLnxIu_HVJN4-pN5lYVyB2HYhlzstOAiWd3S-geuLrXm5Qtsc52t-EGfxoy50DohTMVzUI3kwPgRg4fDpQWBQEhboAApQ5tvuGAjZpcXebstTylrLZzOu-sPCs-FASwchCus3uziSMBWK0HvMGSZHsYpsvMCxt235iydBo-QAvhrkKSA2qv0UWixsrKwFpesugVyzEeSCy5oubPzFjxpnqDwwu3B7z3Ld4GNtx1hvM4D2AzPIjS2rYX6lcf9_Ee1G1V07v3naQv8Iix6705-IPaRJ7MkDgKoB8oKNElyeMsU6eGaSpN_ln01EEv0F-id4xf7IptfSMyzLzWZA4s2hGxrs7laSTuljySqYYl-ndIYliaBT4Kk12V8knRR1E_yNATmkduY5d9tpaCKKy5mWVESNoD_llsemPaMuQk0BCQvx7KdvwXBXGo3gnE2laNfQGkeRjOKBsmAWV1hZS8XmKawVjwd07NyAW2GnhbEXD7KWlNWF6_hfZ9E_MfnFQqaAq9jXii5ZVedPj9EfTXtQRB3ltitPhfpB8yTOQp5eDZIFI8sujBF--Bnpi88uEECE8wmhWhX6aadlnAU-AHTNHqfICfIHw9u4XtJ9LYMV6vgbG7defSd2C7IInpMsV8f2j2eDutdNsBZM-MJ5U_2-SzDQgnBwEG_vq_1C8IQO2wXpq8utcxrx_fvcTYAcEdjWBY7P0YbNTLiHiASTQmG4R2UuqV2zPs2jKcQN1kJyuxkTvOPjPNsuD0Ea3lP28ZgF7M-_H2x0sOk4tNq0H19NAoKg5x6zPgWWYi2ZycZfhb3y0LWrgumayuGk2UliYlj6zT58O6EKSKlKOcNZoThau-71tp32m4ZOURPtr6xZihiZmNDb73Gdh5HH0ELZjCRcObIiR1uBdZjRsyq1oLFom9TP_57ko2GJ0jxPb9oggLTMeHA8c70sKqgKiXndhvLt37z71qfOXlXJwzbqneXip5Hnleeie7EXuxnAvGcyniQLUuo9fbftGv3N7dlWkGGJNTCXh1HK9FASrq2RQMvjyQ4NyVoQifORDlOLwRmKxGtzyaFmkLnV2NJIOcbF1IKs0d9S_rIGv7uQG22XLJFhGK_eUWU9xx39HhwebAk8X3bUdOm5Irt1PIr32-"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_ulIkPB8qIzqRCxTVUQMRsoER", "id": "fc_04b0a37d493a2c8b006ab3494715ec87d297e4eb45bfb7d030", "index": 1}]
-{"name": "read_claim", "args": {}, "id": "call_ulIkPB8qIzqRCxTVUQMRsoER", "type": "tool_call"}</t>
-  </si>
-  <si>
-    <t>01a0cc56-3e74-7c72-855a-c5bfc76cf28b</t>
+    <t>[{"id": "rs_0a7a88b94261cb0d006ab36c8384ac87d2b7524d5f9aac208c", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2yD6ofmZyNuFeQTyE7ubOTNJI5qhtc5nxT8ndpiI_kGGq0bVD6lkx_D7_HsrwSmikfdjfVu7b8aA9dFSHGD2ZgxD9YmgsJHrQtj9vn5QfWnkywtSzz-hr20ct2JvtCiNQbLbDuiAy5a7z37RYlWaMT4rJTUUwbUyiYYYD-uJyafLF9ROWcnpmTEnyf7i6v7lLqtRMvPd76VmHz4471Wbk2CjPB85fiHGEZ8ou3lgY5QyxMpZ48qwlLx-nu9q6eU_vo9DMNjJHfebw2oCRq_0HTDnBNUfLBoRby2YeWqPII81ZkFMuJ1vbuW5dSURrio-GIUho6zRatQO50Yevy7id4t0n1cGVdTlbawUIMek9PsVB9y59H3US6Iin06_YzdX4yQE-zr2Xg4wbKH2TnGPgQcu51H0FhFsEY_WR643hm2imtiyuHO8jjsDOl-UjNEnFs2kfV1CHhT5iGTnX95D7vwGEhTasq-cqQvDW2FnhC-FeEm9-14REJjmjk6Dn5ipJTYKZhOv9eqYdn1-V5BYdQblBUEdcAoZVUn6EfCn6N7BwOBccZ60F5k6-OLIbOX_If_Yxf6AQ9pgzKL2mHVx_peiExCMIOTUs-nSfxIlWhxzZpIu274LlMpesMzT3FvCp1YiECQRNBLLNLcZb7gA41borQcSWgnRjEZktoeeM1JPcboA2chUhNFtE9SOsEaoysImWMSOHQZImnBW5zmQPINXJGuPDOWhj-gYHRQJZlzKy_uW5U1QZIcIOLzMFVByfL8MXDuMgCUmXzFMSEZHF_irZXrLMwoNGF-IFw9D7Akk8F73zciM1BVFyNYK-j5pWssYIz6Sf9_bZYCqCQxY1bFuzqjDg-THC1g7ULJTfItp3V4tqWB1tRd24jRGrM1Yoax30HFgyHDCQIYVCrvLN-pCzjlhKrn7ANlwlTlGsrwQlmPlBPdIM5FP52U9WwBw3Fi44CVp_RtqdEUelj-_J3vrJKVzQ6wro58FqoEnZlBp1T0uk0Tyt6yRoACUzqpAnGnik2dMaarNMFpIQm9KxFmpxOuKb_a0EA1oUPb5GX19J823LBV0NnNHn9XdeyQzIf5kcNen59uy0nBXoXrcfvJAPHPXm-IHm4C0ZihLbJecqGDVGg_ceDQrUMJ9w70MtVHDcB3NFnEiPrv7Q10QBXHKcWULk7ow-T_2qXMH5KE-CfOyEUO_VE8WoCgf7V54AYfenTo58O_gKFPv3-ATI8CuQ=="}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_6v6G40JtLb7Fq5mINTNLOHLt", "id": "fc_0a7a88b94261cb0d006ab36c83cf0087d2bd4191ab7bca5748", "index": 1}]
+{"name": "read_claim", "args": {}, "id": "call_6v6G40JtLb7Fq5mINTNLOHLt", "type": "tool_call"}</t>
+  </si>
+  <si>
+    <t>01a0ccdf-e44b-7c72-8be8-fcd41c8e6f83</t>
   </si>
   <si>
     <t>{"claim_id": "CLM-001", "revision": 2, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}</t>
@@ -511,10 +511,10 @@
     <t>R9</t>
   </si>
   <si>
-    <t>01a0cc56-3e77-7293-8d72-38bc2c780c0a</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "The laptop screen cracked when it fell from a desk at home. The current claim status is **approved**.", "phase": "final_answer", "index": 0, "id": "msg_04b0a37d493a2c8b006ab34947f7ec87d29615e7022d56c808"}]</t>
+    <t>01a0ccdf-e44e-77e0-82ae-e05dc49996a7</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "The laptop fell from a desk, cracking the screen. It happened at home, and the claim status is **approved**.", "phase": "final_answer", "index": 0, "id": "msg_0a7a88b94261cb0d006ab36c84d70887d2aeabbb838a44a091"}]</t>
   </si>
   <si>
     <t>LangGraph</t>
@@ -535,7 +535,7 @@
     <t>Execute the claim_turn workflow operation and pass its result to the next graph step.</t>
   </si>
   <si>
-    <t>01a0cc56-1877-7c30-962c-dd451c04cc12</t>
+    <t>01a0ccdf-b7b7-77a2-a96e-7839f65fff4c</t>
   </si>
   <si>
     <t xml:space="preserve">        claims_agent</t>
@@ -544,7 +544,7 @@
     <t>Execute the claims_agent workflow operation and pass its result to the next graph step.</t>
   </si>
   <si>
-    <t>01a0cc56-1878-76e3-9ec5-2672643609f3</t>
+    <t>01a0ccdf-b7b7-77a2-a96e-784c0d8754fd</t>
   </si>
   <si>
     <t xml:space="preserve">            model</t>
@@ -553,7 +553,7 @@
     <t>Prepare the current conversation, run model middleware, and invoke the chat model.</t>
   </si>
   <si>
-    <t>01a0cc56-1879-7502-8c98-3d8bc6e066d1</t>
+    <t>01a0ccdf-b7b9-7062-a7c6-d364f127b6ab</t>
   </si>
   <si>
     <t xml:space="preserve">                ChatOpenAI</t>
@@ -574,7 +574,7 @@
     <t>Execute tool calls requested by the preceding model response and return their observations.</t>
   </si>
   <si>
-    <t>01a0cc56-1da9-7a31-91d7-ae587099c7d8</t>
+    <t>01a0ccdf-bc26-7252-9a98-6502ab914746</t>
   </si>
   <si>
     <t>No model charge</t>
@@ -589,22 +589,22 @@
     <t>Read fictional policy POL-001, including coverage, deductible, and limit.</t>
   </si>
   <si>
-    <t>01a0cc56-1dae-7990-9c98-bd8a0048e62d</t>
-  </si>
-  <si>
-    <t>01a0cc56-2173-76a3-ac73-a7932fafb011</t>
-  </si>
-  <si>
-    <t>01a0cc56-2176-7b43-b317-51ae929d9433</t>
-  </si>
-  <si>
-    <t>01a0cc56-2177-78a3-acf1-bc41932f9ea3</t>
-  </si>
-  <si>
-    <t>01a0cc56-217a-7b41-88f2-1892d89a51b3</t>
-  </si>
-  <si>
-    <t>01a0cc56-2773-7513-82d4-5bb7888b04b7</t>
+    <t>01a0ccdf-bc2a-7980-8aa7-0ef6b62afdc4</t>
+  </si>
+  <si>
+    <t>01a0ccdf-bfd9-7152-a32a-74292c4115ce</t>
+  </si>
+  <si>
+    <t>01a0ccdf-bfdb-7810-b785-3d8e5ba6a36c</t>
+  </si>
+  <si>
+    <t>01a0ccdf-bfdc-7e23-b958-1055eeda5a65</t>
+  </si>
+  <si>
+    <t>01a0ccdf-bfdd-7b21-8f48-d304d91a70bf</t>
+  </si>
+  <si>
+    <t>01a0ccdf-c7a4-7810-8512-e9429a148fc1</t>
   </si>
   <si>
     <t xml:space="preserve">                read_claim</t>
@@ -613,22 +613,22 @@
     <t>Read the complete current claim, including its authoritative revision.</t>
   </si>
   <si>
-    <t>01a0cc56-2776-7ac3-8f6e-cb38b7f24492</t>
-  </si>
-  <si>
-    <t>01a0cc56-2c1a-7262-af00-f2b576b34013</t>
-  </si>
-  <si>
-    <t>01a0cc56-2c1b-7742-bc1f-8f31b603c02b</t>
-  </si>
-  <si>
-    <t>01a0cc56-2c1b-7742-bc1f-8f49a3961e63</t>
-  </si>
-  <si>
-    <t>01a0cc56-2c1c-7d00-9186-65f1e01c9b8d</t>
-  </si>
-  <si>
-    <t>01a0cc56-3054-7301-bd14-1ce523412385</t>
+    <t>01a0ccdf-c7a9-7a03-bd18-acfaca02907d</t>
+  </si>
+  <si>
+    <t>01a0ccdf-cbc5-7813-bdba-4cf361a6843f</t>
+  </si>
+  <si>
+    <t>01a0ccdf-cbc6-75f0-beca-a188817832f3</t>
+  </si>
+  <si>
+    <t>01a0ccdf-cbc6-75f0-beca-a19bb9970575</t>
+  </si>
+  <si>
+    <t>01a0ccdf-cbc8-7cf2-b0ef-aa10f2c7df29</t>
+  </si>
+  <si>
+    <t>01a0ccdf-d312-79a2-aa4d-ed1d69c37f03</t>
   </si>
   <si>
     <t xml:space="preserve">                edit_claim</t>
@@ -640,37 +640,37 @@
             revision, not the resulting claim contents.</t>
   </si>
   <si>
-    <t>01a0cc56-3058-7b13-a0a5-8b94915cdb5e</t>
-  </si>
-  <si>
-    <t>01a0cc56-3525-7d11-9ae2-f2cd556305af</t>
-  </si>
-  <si>
-    <t>01a0cc56-3527-7862-83c9-4aef39456d87</t>
-  </si>
-  <si>
-    <t>01a0cc56-3527-7862-83c9-4aff2e5246a0</t>
-  </si>
-  <si>
-    <t>01a0cc56-3528-76e1-aa81-76ff4b2380a1</t>
-  </si>
-  <si>
-    <t>01a0cc56-39ef-7883-ac44-79501d4c2a87</t>
-  </si>
-  <si>
-    <t>01a0cc56-39f1-75f0-ab6f-1ca619b75af7</t>
-  </si>
-  <si>
-    <t>01a0cc56-39f1-75f0-ab6f-1cbadabb0b50</t>
-  </si>
-  <si>
-    <t>01a0cc56-39f2-7340-a064-8a554f14ef30</t>
-  </si>
-  <si>
-    <t>01a0cc56-3e74-7c72-855a-c5a5f931f067</t>
-  </si>
-  <si>
-    <t>01a0cc56-3e76-7da0-856b-718d88667c92</t>
+    <t>01a0ccdf-d314-7191-9d92-37de4cab918a</t>
+  </si>
+  <si>
+    <t>01a0ccdf-da71-7361-8cc6-97222da230c4</t>
+  </si>
+  <si>
+    <t>01a0ccdf-da72-7b10-b712-2fa8dfc703c5</t>
+  </si>
+  <si>
+    <t>01a0ccdf-da73-7f33-9d8b-dfe284f7d757</t>
+  </si>
+  <si>
+    <t>01a0ccdf-da74-72f3-89f8-1b68f70e4db9</t>
+  </si>
+  <si>
+    <t>01a0ccdf-de62-7ca0-be24-4f844499f0f7</t>
+  </si>
+  <si>
+    <t>01a0ccdf-de64-78c2-bdc5-2da0940d0b00</t>
+  </si>
+  <si>
+    <t>01a0ccdf-de65-78d3-aecd-aff853e37e7f</t>
+  </si>
+  <si>
+    <t>01a0ccdf-de66-7101-92d9-726494fcf04f</t>
+  </si>
+  <si>
+    <t>01a0ccdf-e449-7531-952a-5a46174e70f1</t>
+  </si>
+  <si>
+    <t>01a0ccdf-e44d-7cc3-924f-35f1043e3acb</t>
   </si>
 </sst>
 </file>
@@ -1138,19 +1138,19 @@
       </c>
       <c r="E2" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32,'Turns'!E46,'Turns'!E61,'Turns'!E75,'Turns'!E90,'Turns'!E104,'Turns'!E118,'Turns'!E133)=9,SUM('Turns'!E17,'Turns'!E32,'Turns'!E46,'Turns'!E61,'Turns'!E75,'Turns'!E90,'Turns'!E104,'Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00104248215</v>
+        <v>0.00106516377</v>
       </c>
       <c r="F2" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32,'Turns'!F46,'Turns'!F61,'Turns'!F75,'Turns'!F90,'Turns'!F104,'Turns'!F118,'Turns'!F133)=9,SUM('Turns'!F17,'Turns'!F32,'Turns'!F46,'Turns'!F61,'Turns'!F75,'Turns'!F90,'Turns'!F104,'Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.001195</v>
+        <v>0.001221</v>
       </c>
       <c r="G2" s="5">
         <f>IF(ISNUMBER(E2),ROUND(E2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>104.0</v>
+        <v>107.0</v>
       </c>
       <c r="H2" s="5">
         <f>IF(ISNUMBER(F2),ROUND(F2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>120.0</v>
+        <v>122.0</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -1162,11 +1162,11 @@
       </c>
       <c r="E3" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.00017883585</v>
+        <v>0.000181278486</v>
       </c>
       <c r="F3" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.000205</v>
+        <v>0.0002078</v>
       </c>
       <c r="G3" s="5">
         <f>IF(ISNUMBER(E3),ROUND(E3*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1299,7 +1299,7 @@
         <v>105</v>
       </c>
       <c r="D11" s="4">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="24" customHeight="1">
@@ -1313,15 +1313,15 @@
         <v>106</v>
       </c>
       <c r="D12" s="5">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E12" s="2">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER('Reference data'!$B$3)),F12*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="F12" s="2">
         <f>IF(D12=0,0,IF(ISNUMBER('Reference data'!F17),D12*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="G12" s="5">
         <f>IF(ISNUMBER(E12),ROUND(E12*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1410,11 +1410,11 @@
       </c>
       <c r="E17" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E12,'Turns'!E13)=3,SUM('Turns'!E5,'Turns'!E12,'Turns'!E13),"Unknown")</f>
-        <v>8.5143312e-05</v>
+        <v>8.7237e-05</v>
       </c>
       <c r="F17" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F12,'Turns'!F13)=3,SUM('Turns'!F5,'Turns'!F12,'Turns'!F13),"Unknown")</f>
-        <v>9.76e-05</v>
+        <v>0.0001</v>
       </c>
       <c r="G17" s="5">
         <f>IF(ISNUMBER(E17),ROUND(E17*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1475,7 +1475,7 @@
         <v>94</v>
       </c>
       <c r="D21" s="4">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="J21" s="4" t="s">
         <v>95</v>
@@ -1525,15 +1525,15 @@
         <v>97</v>
       </c>
       <c r="D23" s="5">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="E23" s="2">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER('Reference data'!$B$3)),F23*'Reference data'!$B$3,"Unknown")</f>
-        <v>7.1708814e-05</v>
+        <v>7.2057762e-05</v>
       </c>
       <c r="F23" s="2">
         <f>IF(D23=0,0,IF(ISNUMBER('Reference data'!B17),D23*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>8.22e-05</v>
+        <v>8.26e-05</v>
       </c>
       <c r="G23" s="5">
         <f>IF(ISNUMBER(E23),ROUND(E23*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1672,11 +1672,11 @@
       </c>
       <c r="E32" s="2">
         <f>IF(COUNT('Turns'!E22,'Turns'!E23,'Turns'!E28)=3,SUM('Turns'!E22,'Turns'!E23,'Turns'!E28),"Unknown")</f>
-        <v>9.3692538e-05</v>
+        <v>9.4041486e-05</v>
       </c>
       <c r="F32" s="2">
         <f>IF(COUNT('Turns'!F22,'Turns'!F23,'Turns'!F28)=3,SUM('Turns'!F22,'Turns'!F23,'Turns'!F28),"Unknown")</f>
-        <v>0.0001074</v>
+        <v>0.0001078</v>
       </c>
       <c r="G32" s="5">
         <f>IF(ISNUMBER(E32),ROUND(E32*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1699,11 +1699,11 @@
       </c>
       <c r="E33" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000223675668</v>
+        <v>0.000224373564</v>
       </c>
       <c r="F33" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002564</v>
+        <v>0.0002572</v>
       </c>
       <c r="G33" s="5">
         <f>IF(ISNUMBER(E33),ROUND(E33*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1725,7 +1725,7 @@
         <v>94</v>
       </c>
       <c r="D34" s="4">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>95</v>
@@ -1775,15 +1775,15 @@
         <v>97</v>
       </c>
       <c r="D36" s="5">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E36" s="2">
         <f>IF(AND(ISNUMBER(F36),ISNUMBER('Reference data'!$B$3)),F36*'Reference data'!$B$3,"Unknown")</f>
-        <v>7.9036722e-05</v>
+        <v>7.938567e-05</v>
       </c>
       <c r="F36" s="2">
         <f>IF(D36=0,0,IF(ISNUMBER('Reference data'!B17),D36*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>9.06e-05</v>
+        <v>9.1e-05</v>
       </c>
       <c r="G36" s="5">
         <f>IF(ISNUMBER(E36),ROUND(E36*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1952,11 +1952,11 @@
       </c>
       <c r="E46" s="2">
         <f>IF(COUNT('Turns'!E35,'Turns'!E36,'Turns'!E41,'Turns'!E42)=4,SUM('Turns'!E35,'Turns'!E36,'Turns'!E41,'Turns'!E42),"Unknown")</f>
-        <v>0.000104160978</v>
+        <v>0.000104509926</v>
       </c>
       <c r="F46" s="2">
         <f>IF(COUNT('Turns'!F35,'Turns'!F36,'Turns'!F41,'Turns'!F42)=4,SUM('Turns'!F35,'Turns'!F36,'Turns'!F41,'Turns'!F42),"Unknown")</f>
-        <v>0.0001194</v>
+        <v>0.0001198</v>
       </c>
       <c r="G46" s="5">
         <f>IF(ISNUMBER(E46),ROUND(E46*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2017,7 +2017,7 @@
         <v>94</v>
       </c>
       <c r="D50" s="4">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="J50" s="4" t="s">
         <v>95</v>
@@ -2067,15 +2067,15 @@
         <v>97</v>
       </c>
       <c r="D52" s="5">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="E52" s="2">
         <f>IF(AND(ISNUMBER(F52),ISNUMBER('Reference data'!$B$3)),F52*'Reference data'!$B$3,"Unknown")</f>
-        <v>9.1249902e-05</v>
+        <v>9.159885e-05</v>
       </c>
       <c r="F52" s="2">
         <f>IF(D52=0,0,IF(ISNUMBER('Reference data'!B17),D52*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001046</v>
+        <v>0.000105</v>
       </c>
       <c r="G52" s="5">
         <f>IF(ISNUMBER(E52),ROUND(E52*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="H52" s="5">
         <f>IF(ISNUMBER(F52),ROUND(F52*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>10.0</v>
+        <v>11.0</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="34" customHeight="1">
@@ -2214,11 +2214,11 @@
       </c>
       <c r="E61" s="2">
         <f>IF(COUNT('Turns'!E51,'Turns'!E52,'Turns'!E57)=3,SUM('Turns'!E51,'Turns'!E52,'Turns'!E57),"Unknown")</f>
-        <v>0.00011951469</v>
+        <v>0.000119863638</v>
       </c>
       <c r="F61" s="2">
         <f>IF(COUNT('Turns'!F51,'Turns'!F52,'Turns'!F57)=3,SUM('Turns'!F51,'Turns'!F52,'Turns'!F57),"Unknown")</f>
-        <v>0.000137</v>
+        <v>0.0001374</v>
       </c>
       <c r="G61" s="5">
         <f>IF(ISNUMBER(E61),ROUND(E61*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2241,19 +2241,19 @@
       </c>
       <c r="E62" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000313355304</v>
+        <v>0.000324870588</v>
       </c>
       <c r="F62" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003592</v>
+        <v>0.0003724</v>
       </c>
       <c r="G62" s="5">
         <f>IF(ISNUMBER(E62),ROUND(E62*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="H62" s="5">
         <f>IF(ISNUMBER(F62),ROUND(F62*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="63" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -2267,7 +2267,7 @@
         <v>94</v>
       </c>
       <c r="D63" s="4">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="J63" s="4" t="s">
         <v>95</v>
@@ -2317,15 +2317,15 @@
         <v>97</v>
       </c>
       <c r="D65" s="5">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E65" s="2">
         <f>IF(AND(ISNUMBER(F65),ISNUMBER('Reference data'!$B$3)),F65*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.000105207822</v>
+        <v>0.00010555677</v>
       </c>
       <c r="F65" s="2">
         <f>IF(D65=0,0,IF(ISNUMBER('Reference data'!B17),D65*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001206</v>
+        <v>0.000121</v>
       </c>
       <c r="G65" s="5">
         <f>IF(ISNUMBER(E65),ROUND(E65*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2383,7 +2383,7 @@
         <v>105</v>
       </c>
       <c r="D69" s="4">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="24" customHeight="1">
@@ -2397,23 +2397,23 @@
         <v>106</v>
       </c>
       <c r="D70" s="5">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E70" s="2">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER('Reference data'!$B$3)),F70*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="F70" s="2">
         <f>IF(D70=0,0,IF(ISNUMBER('Reference data'!F17),D70*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="G70" s="5">
         <f>IF(ISNUMBER(E70),ROUND(E70*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="H70" s="5">
         <f>IF(ISNUMBER(F70),ROUND(F70*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="71" spans="1:13" ht="24" customHeight="1">
@@ -2494,19 +2494,19 @@
       </c>
       <c r="E75" s="2">
         <f>IF(COUNT('Turns'!E64,'Turns'!E65,'Turns'!E70,'Turns'!E71)=4,SUM('Turns'!E64,'Turns'!E65,'Turns'!E70,'Turns'!E71),"Unknown")</f>
-        <v>0.00015964371</v>
+        <v>0.00016836741</v>
       </c>
       <c r="F75" s="2">
         <f>IF(COUNT('Turns'!F64,'Turns'!F65,'Turns'!F70,'Turns'!F71)=4,SUM('Turns'!F64,'Turns'!F65,'Turns'!F70,'Turns'!F71),"Unknown")</f>
-        <v>0.000183</v>
+        <v>0.000193</v>
       </c>
       <c r="G75" s="5">
         <f>IF(ISNUMBER(E75),ROUND(E75*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
       <c r="H75" s="5">
         <f>IF(ISNUMBER(F75),ROUND(F75*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="K75" s="4" t="s">
         <v>111</v>
@@ -2559,7 +2559,7 @@
         <v>94</v>
       </c>
       <c r="D79" s="4">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="J79" s="4" t="s">
         <v>95</v>
@@ -2609,15 +2609,15 @@
         <v>97</v>
       </c>
       <c r="D81" s="5">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="E81" s="2">
         <f>IF(AND(ISNUMBER(F81),ISNUMBER('Reference data'!$B$3)),F81*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.000118118898</v>
+        <v>0.000119863638</v>
       </c>
       <c r="F81" s="2">
         <f>IF(D81=0,0,IF(ISNUMBER('Reference data'!B17),D81*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001354</v>
+        <v>0.0001374</v>
       </c>
       <c r="G81" s="5">
         <f>IF(ISNUMBER(E81),ROUND(E81*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2675,7 +2675,7 @@
         <v>105</v>
       </c>
       <c r="D85" s="4">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="24" customHeight="1">
@@ -2689,15 +2689,15 @@
         <v>107</v>
       </c>
       <c r="D86" s="5">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E86" s="2">
         <f>IF(AND(ISNUMBER(F86),ISNUMBER('Reference data'!$B$3)),F86*'Reference data'!$B$3,"Unknown")</f>
-        <v>3.5592696e-05</v>
+        <v>3.663954e-05</v>
       </c>
       <c r="F86" s="2">
         <f>IF(D86=0,0,IF(ISNUMBER('Reference data'!E17),D86*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>4.08e-05</v>
+        <v>4.2e-05</v>
       </c>
       <c r="G86" s="5">
         <f>IF(ISNUMBER(E86),ROUND(E86*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2708,7 +2708,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="47" customHeight="1">
+    <row r="87" spans="1:13" ht="60" customHeight="1">
       <c r="A87" t="s">
         <v>143</v>
       </c>
@@ -2756,15 +2756,15 @@
       </c>
       <c r="E90" s="2">
         <f>IF(COUNT('Turns'!E80,'Turns'!E81,'Turns'!E86)=3,SUM('Turns'!E80,'Turns'!E81,'Turns'!E86),"Unknown")</f>
-        <v>0.000153711594</v>
+        <v>0.000156503178</v>
       </c>
       <c r="F90" s="2">
         <f>IF(COUNT('Turns'!F80,'Turns'!F81,'Turns'!F86)=3,SUM('Turns'!F80,'Turns'!F81,'Turns'!F86),"Unknown")</f>
-        <v>0.0001762</v>
+        <v>0.0001794</v>
       </c>
       <c r="G90" s="5">
         <f>IF(ISNUMBER(E90),ROUND(E90*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="H90" s="5">
         <f>IF(ISNUMBER(F90),ROUND(F90*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3047,19 +3047,19 @@
       </c>
       <c r="E105" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.000232748316</v>
+        <v>0.00024077412</v>
       </c>
       <c r="F105" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.0002668</v>
+        <v>0.000276</v>
       </c>
       <c r="G105" s="5">
         <f>IF(ISNUMBER(E105),ROUND(E105*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="H105" s="5">
         <f>IF(ISNUMBER(F105),ROUND(F105*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="106" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -3189,7 +3189,7 @@
         <v>105</v>
       </c>
       <c r="D112" s="4">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="113" spans="1:13" ht="24" customHeight="1">
@@ -3203,15 +3203,15 @@
         <v>106</v>
       </c>
       <c r="D113" s="5">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E113" s="2">
         <f>IF(AND(ISNUMBER(F113),ISNUMBER('Reference data'!$B$3)),F113*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="F113" s="2">
         <f>IF(D113=0,0,IF(ISNUMBER('Reference data'!F17),D113*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="G113" s="5">
         <f>IF(ISNUMBER(E113),ROUND(E113*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="H113" s="5">
         <f>IF(ISNUMBER(F113),ROUND(F113*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="114" spans="1:13" ht="24" customHeight="1">
@@ -3252,7 +3252,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="115" spans="1:13" ht="268" customHeight="1">
+    <row r="115" spans="1:13" ht="281" customHeight="1">
       <c r="A115" t="s">
         <v>152</v>
       </c>
@@ -3300,11 +3300,11 @@
       </c>
       <c r="E118" s="2">
         <f>IF(COUNT('Turns'!E107,'Turns'!E108,'Turns'!E113,'Turns'!E114)=4,SUM('Turns'!E107,'Turns'!E108,'Turns'!E113,'Turns'!E114),"Unknown")</f>
-        <v>0.000109744146</v>
+        <v>0.000113931522</v>
       </c>
       <c r="F118" s="2">
         <f>IF(COUNT('Turns'!F107,'Turns'!F108,'Turns'!F113,'Turns'!F114)=4,SUM('Turns'!F107,'Turns'!F108,'Turns'!F113,'Turns'!F114),"Unknown")</f>
-        <v>0.0001258</v>
+        <v>0.0001306</v>
       </c>
       <c r="G118" s="5">
         <f>IF(ISNUMBER(E118),ROUND(E118*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3365,7 +3365,7 @@
         <v>94</v>
       </c>
       <c r="D122" s="4">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="J122" s="4" t="s">
         <v>95</v>
@@ -3415,15 +3415,15 @@
         <v>97</v>
       </c>
       <c r="D124" s="5">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="E124" s="2">
         <f>IF(AND(ISNUMBER(F124),ISNUMBER('Reference data'!$B$3)),F124*'Reference data'!$B$3,"Unknown")</f>
-        <v>9.5786226e-05</v>
+        <v>9.6484122e-05</v>
       </c>
       <c r="F124" s="2">
         <f>IF(D124=0,0,IF(ISNUMBER('Reference data'!B17),D124*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001098</v>
+        <v>0.0001106</v>
       </c>
       <c r="G124" s="5">
         <f>IF(ISNUMBER(E124),ROUND(E124*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3481,7 +3481,7 @@
         <v>105</v>
       </c>
       <c r="D128" s="4">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="24" customHeight="1">
@@ -3495,15 +3495,15 @@
         <v>107</v>
       </c>
       <c r="D129" s="5">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E129" s="2">
         <f>IF(AND(ISNUMBER(F129),ISNUMBER('Reference data'!$B$3)),F129*'Reference data'!$B$3,"Unknown")</f>
-        <v>2.7217944e-05</v>
+        <v>3.0358476e-05</v>
       </c>
       <c r="F129" s="2">
         <f>IF(D129=0,0,IF(ISNUMBER('Reference data'!E17),D129*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>3.12e-05</v>
+        <v>3.48e-05</v>
       </c>
       <c r="G129" s="5">
         <f>IF(ISNUMBER(E129),ROUND(E129*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3562,19 +3562,19 @@
       </c>
       <c r="E133" s="2">
         <f>IF(COUNT('Turns'!E123,'Turns'!E124,'Turns'!E129)=3,SUM('Turns'!E123,'Turns'!E124,'Turns'!E129),"Unknown")</f>
-        <v>0.00012300417</v>
+        <v>0.000126842598</v>
       </c>
       <c r="F133" s="2">
         <f>IF(COUNT('Turns'!F123,'Turns'!F124,'Turns'!F129)=3,SUM('Turns'!F123,'Turns'!F124,'Turns'!F129),"Unknown")</f>
-        <v>0.000141</v>
+        <v>0.0001454</v>
       </c>
       <c r="G133" s="5">
         <f>IF(ISNUMBER(E133),ROUND(E133*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="H133" s="5">
         <f>IF(ISNUMBER(F133),ROUND(F133*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="K133" s="4" t="s">
         <v>111</v>
@@ -3724,15 +3724,15 @@
       </c>
       <c r="J2" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>743.0</v>
+        <v>745.0</v>
       </c>
       <c r="K2" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.000129634182</v>
+        <v>0.00012998313</v>
       </c>
       <c r="L2" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.0001486</v>
+        <v>0.000149</v>
       </c>
       <c r="M2" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3769,23 +3769,23 @@
       </c>
       <c r="V2" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="W2" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="X2" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="Y2" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.00017883585</v>
+        <v>0.000181278486</v>
       </c>
       <c r="Z2" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.000205</v>
+        <v>0.0002078</v>
       </c>
       <c r="AA2" s="5">
         <f>IF(ISNUMBER(Y2),ROUND(Y2*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3796,7 +3796,7 @@
         <v>21.0</v>
       </c>
       <c r="AD2" s="1">
-        <v>2277.454</v>
+        <v>2064.456</v>
       </c>
       <c r="AE2" s="1" t="s">
         <v>164</v>
@@ -3829,15 +3829,15 @@
       </c>
       <c r="J3" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>743.0</v>
+        <v>745.0</v>
       </c>
       <c r="K3" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.000129634182</v>
+        <v>0.00012998313</v>
       </c>
       <c r="L3" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.0001486</v>
+        <v>0.000149</v>
       </c>
       <c r="M3" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3874,23 +3874,23 @@
       </c>
       <c r="V3" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="W3" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="X3" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="Y3" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.00017883585</v>
+        <v>0.000181278486</v>
       </c>
       <c r="Z3" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.000205</v>
+        <v>0.0002078</v>
       </c>
       <c r="AA3" s="5">
         <f>IF(ISNUMBER(Y3),ROUND(Y3*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3901,7 +3901,7 @@
         <v>21.0</v>
       </c>
       <c r="AD3" s="1">
-        <v>2275.24</v>
+        <v>2062.321</v>
       </c>
       <c r="AE3" s="1" t="s">
         <v>164</v>
@@ -3934,15 +3934,15 @@
       </c>
       <c r="J4" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>743.0</v>
+        <v>745.0</v>
       </c>
       <c r="K4" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.000129634182</v>
+        <v>0.00012998313</v>
       </c>
       <c r="L4" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.0001486</v>
+        <v>0.000149</v>
       </c>
       <c r="M4" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3979,23 +3979,23 @@
       </c>
       <c r="V4" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="W4" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="X4" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="Y4" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.00017883585</v>
+        <v>0.000181278486</v>
       </c>
       <c r="Z4" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.000205</v>
+        <v>0.0002078</v>
       </c>
       <c r="AA4" s="5">
         <f>IF(ISNUMBER(Y4),ROUND(Y4*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4006,7 +4006,7 @@
         <v>21.0</v>
       </c>
       <c r="AD4" s="1">
-        <v>2273.82</v>
+        <v>2061.077</v>
       </c>
       <c r="AE4" s="1" t="s">
         <v>164</v>
@@ -4081,23 +4081,23 @@
       </c>
       <c r="V5" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="W5" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="X5" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="Y5" s="2">
         <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>8.5143312e-05</v>
+        <v>8.7237e-05</v>
       </c>
       <c r="Z5" s="2">
         <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>9.76e-05</v>
+        <v>0.0001</v>
       </c>
       <c r="AA5" s="5">
         <f>IF(ISNUMBER(Y5),ROUND(Y5*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4108,7 +4108,7 @@
         <v>10.0</v>
       </c>
       <c r="AD5" s="1">
-        <v>1326.524</v>
+        <v>1132.401</v>
       </c>
       <c r="AE5" s="1" t="s">
         <v>164</v>
@@ -4186,23 +4186,23 @@
       </c>
       <c r="V6" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>10.0</v>
+        <v>12.0</v>
       </c>
       <c r="W6" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.2562128e-05</v>
       </c>
       <c r="X6" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.44e-05</v>
       </c>
       <c r="Y6" s="2">
         <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>8.5143312e-05</v>
+        <v>8.7237e-05</v>
       </c>
       <c r="Z6" s="2">
         <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>9.76e-05</v>
+        <v>0.0001</v>
       </c>
       <c r="AA6" s="5">
         <f>IF(ISNUMBER(Y6),ROUND(Y6*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4216,7 +4216,7 @@
         <v>93</v>
       </c>
       <c r="AD6" s="1">
-        <v>1323.569</v>
+        <v>1129.267</v>
       </c>
       <c r="AE6" s="1" t="s">
         <v>177</v>
@@ -4248,7 +4248,7 @@
         <v>170</v>
       </c>
       <c r="AD7" s="1">
-        <v>3.816</v>
+        <v>3.23</v>
       </c>
       <c r="AE7" s="1" t="s">
         <v>181</v>
@@ -4280,7 +4280,7 @@
         <v>180</v>
       </c>
       <c r="AD8" s="1">
-        <v>0.854</v>
+        <v>0.491</v>
       </c>
       <c r="AE8" s="1" t="s">
         <v>181</v>
@@ -4313,15 +4313,15 @@
       </c>
       <c r="J9" s="2">
         <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>411.0</v>
+        <v>413.0</v>
       </c>
       <c r="K9" s="2">
         <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>7.1708814e-05</v>
+        <v>7.2057762e-05</v>
       </c>
       <c r="L9" s="2">
         <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>8.22e-05</v>
+        <v>8.26e-05</v>
       </c>
       <c r="M9" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -4367,11 +4367,11 @@
       </c>
       <c r="Y9" s="2">
         <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>9.3692538e-05</v>
+        <v>9.4041486e-05</v>
       </c>
       <c r="Z9" s="2">
         <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.0001074</v>
+        <v>0.0001078</v>
       </c>
       <c r="AA9" s="5">
         <f>IF(ISNUMBER(Y9),ROUND(Y9*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4382,7 +4382,7 @@
         <v>11.0</v>
       </c>
       <c r="AD9" s="1">
-        <v>938.926</v>
+        <v>921.4930000000001</v>
       </c>
       <c r="AE9" s="1" t="s">
         <v>164</v>
@@ -4405,7 +4405,7 @@
         <v>111</v>
       </c>
       <c r="F10" s="1">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>176</v>
@@ -4418,15 +4418,15 @@
       </c>
       <c r="J10" s="2">
         <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>411.0</v>
+        <v>413.0</v>
       </c>
       <c r="K10" s="2">
         <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>7.1708814e-05</v>
+        <v>7.2057762e-05</v>
       </c>
       <c r="L10" s="2">
         <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>8.22e-05</v>
+        <v>8.26e-05</v>
       </c>
       <c r="M10" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -4472,11 +4472,11 @@
       </c>
       <c r="Y10" s="2">
         <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>9.3692538e-05</v>
+        <v>9.4041486e-05</v>
       </c>
       <c r="Z10" s="2">
         <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.0001074</v>
+        <v>0.0001078</v>
       </c>
       <c r="AA10" s="5">
         <f>IF(ISNUMBER(Y10),ROUND(Y10*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4490,7 +4490,7 @@
         <v>118</v>
       </c>
       <c r="AD10" s="1">
-        <v>937.184</v>
+        <v>919.8680000000001</v>
       </c>
       <c r="AE10" s="1" t="s">
         <v>177</v>
@@ -4520,15 +4520,15 @@
       </c>
       <c r="J11" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>976.0</v>
+        <v>980.0</v>
       </c>
       <c r="K11" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.000170286624</v>
+        <v>0.00017098452</v>
       </c>
       <c r="L11" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.0001952</v>
+        <v>0.000196</v>
       </c>
       <c r="M11" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4577,11 +4577,11 @@
       </c>
       <c r="Y11" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000223675668</v>
+        <v>0.000224373564</v>
       </c>
       <c r="Z11" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002564</v>
+        <v>0.0002572</v>
       </c>
       <c r="AA11" s="5">
         <f>IF(ISNUMBER(Y11),ROUND(Y11*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4592,7 +4592,7 @@
         <v>26.0</v>
       </c>
       <c r="AD11" s="1">
-        <v>2706.443</v>
+        <v>3034.127</v>
       </c>
       <c r="AE11" s="1" t="s">
         <v>164</v>
@@ -4625,15 +4625,15 @@
       </c>
       <c r="J12" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>976.0</v>
+        <v>980.0</v>
       </c>
       <c r="K12" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.000170286624</v>
+        <v>0.00017098452</v>
       </c>
       <c r="L12" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.0001952</v>
+        <v>0.000196</v>
       </c>
       <c r="M12" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4682,11 +4682,11 @@
       </c>
       <c r="Y12" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000223675668</v>
+        <v>0.000224373564</v>
       </c>
       <c r="Z12" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002564</v>
+        <v>0.0002572</v>
       </c>
       <c r="AA12" s="5">
         <f>IF(ISNUMBER(Y12),ROUND(Y12*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4697,7 +4697,7 @@
         <v>26.0</v>
       </c>
       <c r="AD12" s="1">
-        <v>2703.009</v>
+        <v>3031.748</v>
       </c>
       <c r="AE12" s="1" t="s">
         <v>164</v>
@@ -4730,15 +4730,15 @@
       </c>
       <c r="J13" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>976.0</v>
+        <v>980.0</v>
       </c>
       <c r="K13" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.000170286624</v>
+        <v>0.00017098452</v>
       </c>
       <c r="L13" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.0001952</v>
+        <v>0.000196</v>
       </c>
       <c r="M13" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4787,11 +4787,11 @@
       </c>
       <c r="Y13" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000223675668</v>
+        <v>0.000224373564</v>
       </c>
       <c r="Z13" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002564</v>
+        <v>0.0002572</v>
       </c>
       <c r="AA13" s="5">
         <f>IF(ISNUMBER(Y13),ROUND(Y13*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4802,7 +4802,7 @@
         <v>26.0</v>
       </c>
       <c r="AD13" s="1">
-        <v>2701.045</v>
+        <v>3030.634</v>
       </c>
       <c r="AE13" s="1" t="s">
         <v>164</v>
@@ -4835,15 +4835,15 @@
       </c>
       <c r="J14" s="2">
         <f>IF(COUNT('Turns'!D36)=1,SUM('Turns'!D36),"Unknown")</f>
-        <v>453.0</v>
+        <v>455.0</v>
       </c>
       <c r="K14" s="2">
         <f>IF(COUNT('Turns'!E36)=1,SUM('Turns'!E36),"Unknown")</f>
-        <v>7.9036722e-05</v>
+        <v>7.938567e-05</v>
       </c>
       <c r="L14" s="2">
         <f>IF(COUNT('Turns'!F36)=1,SUM('Turns'!F36),"Unknown")</f>
-        <v>9.06e-05</v>
+        <v>9.1e-05</v>
       </c>
       <c r="M14" s="2">
         <f>IF(COUNT('Turns'!D35)=1,SUM('Turns'!D35),"Unknown")</f>
@@ -4892,11 +4892,11 @@
       </c>
       <c r="Y14" s="2">
         <f>IF(COUNT('Turns'!E46)=1,SUM('Turns'!E46),"Unknown")</f>
-        <v>0.000104160978</v>
+        <v>0.000104509926</v>
       </c>
       <c r="Z14" s="2">
         <f>IF(COUNT('Turns'!F46)=1,SUM('Turns'!F46),"Unknown")</f>
-        <v>0.0001194</v>
+        <v>0.0001198</v>
       </c>
       <c r="AA14" s="5">
         <f>IF(ISNUMBER(Y14),ROUND(Y14*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4907,7 +4907,7 @@
         <v>12.0</v>
       </c>
       <c r="AD14" s="1">
-        <v>1527.204</v>
+        <v>1989.086</v>
       </c>
       <c r="AE14" s="1" t="s">
         <v>164</v>
@@ -4930,7 +4930,7 @@
         <v>111</v>
       </c>
       <c r="F15" s="1">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>176</v>
@@ -4943,15 +4943,15 @@
       </c>
       <c r="J15" s="2">
         <f>IF(COUNT('Turns'!D36)=1,SUM('Turns'!D36),"Unknown")</f>
-        <v>453.0</v>
+        <v>455.0</v>
       </c>
       <c r="K15" s="2">
         <f>IF(COUNT('Turns'!E36)=1,SUM('Turns'!E36),"Unknown")</f>
-        <v>7.9036722e-05</v>
+        <v>7.938567e-05</v>
       </c>
       <c r="L15" s="2">
         <f>IF(COUNT('Turns'!F36)=1,SUM('Turns'!F36),"Unknown")</f>
-        <v>9.06e-05</v>
+        <v>9.1e-05</v>
       </c>
       <c r="M15" s="2">
         <f>IF(COUNT('Turns'!D35)=1,SUM('Turns'!D35),"Unknown")</f>
@@ -5000,11 +5000,11 @@
       </c>
       <c r="Y15" s="2">
         <f>IF(COUNT('Turns'!E46)=1,SUM('Turns'!E46),"Unknown")</f>
-        <v>0.000104160978</v>
+        <v>0.000104509926</v>
       </c>
       <c r="Z15" s="2">
         <f>IF(COUNT('Turns'!F46)=1,SUM('Turns'!F46),"Unknown")</f>
-        <v>0.0001194</v>
+        <v>0.0001198</v>
       </c>
       <c r="AA15" s="5">
         <f>IF(ISNUMBER(Y15),ROUND(Y15*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5018,7 +5018,7 @@
         <v>124</v>
       </c>
       <c r="AD15" s="1">
-        <v>1523.188</v>
+        <v>1986.238</v>
       </c>
       <c r="AE15" s="1" t="s">
         <v>177</v>
@@ -5050,7 +5050,7 @@
         <v>188</v>
       </c>
       <c r="AD16" s="1">
-        <v>2.515</v>
+        <v>3.446</v>
       </c>
       <c r="AE16" s="1" t="s">
         <v>181</v>
@@ -5082,7 +5082,7 @@
         <v>190</v>
       </c>
       <c r="AD17" s="1">
-        <v>0.587</v>
+        <v>0.825</v>
       </c>
       <c r="AE17" s="1" t="s">
         <v>181</v>
@@ -5115,15 +5115,15 @@
       </c>
       <c r="J18" s="2">
         <f>IF(COUNT('Turns'!D52)=1,SUM('Turns'!D52),"Unknown")</f>
-        <v>523.0</v>
+        <v>525.0</v>
       </c>
       <c r="K18" s="2">
         <f>IF(COUNT('Turns'!E52)=1,SUM('Turns'!E52),"Unknown")</f>
-        <v>9.1249902e-05</v>
+        <v>9.159885e-05</v>
       </c>
       <c r="L18" s="2">
         <f>IF(COUNT('Turns'!F52)=1,SUM('Turns'!F52),"Unknown")</f>
-        <v>0.0001046</v>
+        <v>0.000105</v>
       </c>
       <c r="M18" s="2">
         <f>IF(COUNT('Turns'!D51)=1,SUM('Turns'!D51),"Unknown")</f>
@@ -5169,11 +5169,11 @@
       </c>
       <c r="Y18" s="2">
         <f>IF(COUNT('Turns'!E61)=1,SUM('Turns'!E61),"Unknown")</f>
-        <v>0.00011951469</v>
+        <v>0.000119863638</v>
       </c>
       <c r="Z18" s="2">
         <f>IF(COUNT('Turns'!F61)=1,SUM('Turns'!F61),"Unknown")</f>
-        <v>0.000137</v>
+        <v>0.0001374</v>
       </c>
       <c r="AA18" s="5">
         <f>IF(ISNUMBER(Y18),ROUND(Y18*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5184,7 +5184,7 @@
         <v>14.0</v>
       </c>
       <c r="AD18" s="1">
-        <v>1164.534</v>
+        <v>1032.616</v>
       </c>
       <c r="AE18" s="1" t="s">
         <v>164</v>
@@ -5207,7 +5207,7 @@
         <v>111</v>
       </c>
       <c r="F19" s="1">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>176</v>
@@ -5220,15 +5220,15 @@
       </c>
       <c r="J19" s="2">
         <f>IF(COUNT('Turns'!D52)=1,SUM('Turns'!D52),"Unknown")</f>
-        <v>523.0</v>
+        <v>525.0</v>
       </c>
       <c r="K19" s="2">
         <f>IF(COUNT('Turns'!E52)=1,SUM('Turns'!E52),"Unknown")</f>
-        <v>9.1249902e-05</v>
+        <v>9.159885e-05</v>
       </c>
       <c r="L19" s="2">
         <f>IF(COUNT('Turns'!F52)=1,SUM('Turns'!F52),"Unknown")</f>
-        <v>0.0001046</v>
+        <v>0.000105</v>
       </c>
       <c r="M19" s="2">
         <f>IF(COUNT('Turns'!D51)=1,SUM('Turns'!D51),"Unknown")</f>
@@ -5274,11 +5274,11 @@
       </c>
       <c r="Y19" s="2">
         <f>IF(COUNT('Turns'!E61)=1,SUM('Turns'!E61),"Unknown")</f>
-        <v>0.00011951469</v>
+        <v>0.000119863638</v>
       </c>
       <c r="Z19" s="2">
         <f>IF(COUNT('Turns'!F61)=1,SUM('Turns'!F61),"Unknown")</f>
-        <v>0.000137</v>
+        <v>0.0001374</v>
       </c>
       <c r="AA19" s="5">
         <f>IF(ISNUMBER(Y19),ROUND(Y19*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5292,7 +5292,7 @@
         <v>131</v>
       </c>
       <c r="AD19" s="1">
-        <v>1162.538</v>
+        <v>1031.15</v>
       </c>
       <c r="AE19" s="1" t="s">
         <v>177</v>
@@ -5322,15 +5322,15 @@
       </c>
       <c r="J20" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1280.0</v>
+        <v>1292.0</v>
       </c>
       <c r="K20" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.00022332672</v>
+        <v>0.000225420408</v>
       </c>
       <c r="L20" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.000256</v>
+        <v>0.0002584</v>
       </c>
       <c r="M20" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5355,46 +5355,46 @@
       </c>
       <c r="S20" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>74.0</v>
+        <v>75.0</v>
       </c>
       <c r="T20" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.7466456e-05</v>
+        <v>7.85133e-05</v>
       </c>
       <c r="U20" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>8.88e-05</v>
+        <v>9e-05</v>
       </c>
       <c r="V20" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>12.0</v>
+        <v>20.0</v>
       </c>
       <c r="W20" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="X20" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="Y20" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000313355304</v>
+        <v>0.000324870588</v>
       </c>
       <c r="Z20" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003592</v>
+        <v>0.0003724</v>
       </c>
       <c r="AA20" s="5">
         <f>IF(ISNUMBER(Y20),ROUND(Y20*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="AB20" s="5">
         <f>IF(ISNUMBER(Z20),ROUND(Z20*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="AD20" s="1">
-        <v>2298.823</v>
+        <v>3736.47</v>
       </c>
       <c r="AE20" s="1" t="s">
         <v>164</v>
@@ -5427,15 +5427,15 @@
       </c>
       <c r="J21" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1280.0</v>
+        <v>1292.0</v>
       </c>
       <c r="K21" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.00022332672</v>
+        <v>0.000225420408</v>
       </c>
       <c r="L21" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.000256</v>
+        <v>0.0002584</v>
       </c>
       <c r="M21" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5460,46 +5460,46 @@
       </c>
       <c r="S21" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>74.0</v>
+        <v>75.0</v>
       </c>
       <c r="T21" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.7466456e-05</v>
+        <v>7.85133e-05</v>
       </c>
       <c r="U21" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>8.88e-05</v>
+        <v>9e-05</v>
       </c>
       <c r="V21" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>12.0</v>
+        <v>20.0</v>
       </c>
       <c r="W21" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="X21" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="Y21" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000313355304</v>
+        <v>0.000324870588</v>
       </c>
       <c r="Z21" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003592</v>
+        <v>0.0003724</v>
       </c>
       <c r="AA21" s="5">
         <f>IF(ISNUMBER(Y21),ROUND(Y21*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="AB21" s="5">
         <f>IF(ISNUMBER(Z21),ROUND(Z21*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="AD21" s="1">
-        <v>2296.696</v>
+        <v>3734.538</v>
       </c>
       <c r="AE21" s="1" t="s">
         <v>164</v>
@@ -5532,15 +5532,15 @@
       </c>
       <c r="J22" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1280.0</v>
+        <v>1292.0</v>
       </c>
       <c r="K22" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.00022332672</v>
+        <v>0.000225420408</v>
       </c>
       <c r="L22" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.000256</v>
+        <v>0.0002584</v>
       </c>
       <c r="M22" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5565,46 +5565,46 @@
       </c>
       <c r="S22" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>74.0</v>
+        <v>75.0</v>
       </c>
       <c r="T22" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.7466456e-05</v>
+        <v>7.85133e-05</v>
       </c>
       <c r="U22" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>8.88e-05</v>
+        <v>9e-05</v>
       </c>
       <c r="V22" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>12.0</v>
+        <v>20.0</v>
       </c>
       <c r="W22" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="X22" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="Y22" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000313355304</v>
+        <v>0.000324870588</v>
       </c>
       <c r="Z22" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003592</v>
+        <v>0.0003724</v>
       </c>
       <c r="AA22" s="5">
         <f>IF(ISNUMBER(Y22),ROUND(Y22*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>31.0</v>
+        <v>32.0</v>
       </c>
       <c r="AB22" s="5">
         <f>IF(ISNUMBER(Z22),ROUND(Z22*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>36.0</v>
+        <v>37.0</v>
       </c>
       <c r="AD22" s="1">
-        <v>2295.737</v>
+        <v>3732.928</v>
       </c>
       <c r="AE22" s="1" t="s">
         <v>164</v>
@@ -5637,15 +5637,15 @@
       </c>
       <c r="J23" s="2">
         <f>IF(COUNT('Turns'!D65)=1,SUM('Turns'!D65),"Unknown")</f>
-        <v>603.0</v>
+        <v>605.0</v>
       </c>
       <c r="K23" s="2">
         <f>IF(COUNT('Turns'!E65)=1,SUM('Turns'!E65),"Unknown")</f>
-        <v>0.000105207822</v>
+        <v>0.00010555677</v>
       </c>
       <c r="L23" s="2">
         <f>IF(COUNT('Turns'!F65)=1,SUM('Turns'!F65),"Unknown")</f>
-        <v>0.0001206</v>
+        <v>0.000121</v>
       </c>
       <c r="M23" s="2">
         <f>IF(COUNT('Turns'!D64)=1,SUM('Turns'!D64),"Unknown")</f>
@@ -5682,34 +5682,34 @@
       </c>
       <c r="V23" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>12.0</v>
+        <v>20.0</v>
       </c>
       <c r="W23" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="X23" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="Y23" s="2">
         <f>IF(COUNT('Turns'!E75)=1,SUM('Turns'!E75),"Unknown")</f>
-        <v>0.00015964371</v>
+        <v>0.00016836741</v>
       </c>
       <c r="Z23" s="2">
         <f>IF(COUNT('Turns'!F75)=1,SUM('Turns'!F75),"Unknown")</f>
-        <v>0.000183</v>
+        <v>0.000193</v>
       </c>
       <c r="AA23" s="5">
         <f>IF(ISNUMBER(Y23),ROUND(Y23*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
       <c r="AB23" s="5">
         <f>IF(ISNUMBER(Z23),ROUND(Z23*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="AD23" s="1">
-        <v>1079.269</v>
+        <v>1865.263</v>
       </c>
       <c r="AE23" s="1" t="s">
         <v>164</v>
@@ -5732,7 +5732,7 @@
         <v>111</v>
       </c>
       <c r="F24" s="1">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>176</v>
@@ -5745,15 +5745,15 @@
       </c>
       <c r="J24" s="2">
         <f>IF(COUNT('Turns'!D65)=1,SUM('Turns'!D65),"Unknown")</f>
-        <v>603.0</v>
+        <v>605.0</v>
       </c>
       <c r="K24" s="2">
         <f>IF(COUNT('Turns'!E65)=1,SUM('Turns'!E65),"Unknown")</f>
-        <v>0.000105207822</v>
+        <v>0.00010555677</v>
       </c>
       <c r="L24" s="2">
         <f>IF(COUNT('Turns'!F65)=1,SUM('Turns'!F65),"Unknown")</f>
-        <v>0.0001206</v>
+        <v>0.000121</v>
       </c>
       <c r="M24" s="2">
         <f>IF(COUNT('Turns'!D64)=1,SUM('Turns'!D64),"Unknown")</f>
@@ -5790,37 +5790,37 @@
       </c>
       <c r="V24" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>12.0</v>
+        <v>20.0</v>
       </c>
       <c r="W24" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>2.093688e-05</v>
       </c>
       <c r="X24" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>2.4e-05</v>
       </c>
       <c r="Y24" s="2">
         <f>IF(COUNT('Turns'!E75)=1,SUM('Turns'!E75),"Unknown")</f>
-        <v>0.00015964371</v>
+        <v>0.00016836741</v>
       </c>
       <c r="Z24" s="2">
         <f>IF(COUNT('Turns'!F75)=1,SUM('Turns'!F75),"Unknown")</f>
-        <v>0.000183</v>
+        <v>0.000193</v>
       </c>
       <c r="AA24" s="5">
         <f>IF(ISNUMBER(Y24),ROUND(Y24*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>16.0</v>
+        <v>17.0</v>
       </c>
       <c r="AB24" s="5">
         <f>IF(ISNUMBER(Z24),ROUND(Z24*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>18.0</v>
+        <v>19.0</v>
       </c>
       <c r="AC24" s="1" t="s">
         <v>135</v>
       </c>
       <c r="AD24" s="1">
-        <v>1077.505</v>
+        <v>1863.739</v>
       </c>
       <c r="AE24" s="1" t="s">
         <v>177</v>
@@ -5852,7 +5852,7 @@
         <v>196</v>
       </c>
       <c r="AD25" s="1">
-        <v>2.477</v>
+        <v>1.923</v>
       </c>
       <c r="AE25" s="1" t="s">
         <v>181</v>
@@ -5884,7 +5884,7 @@
         <v>198</v>
       </c>
       <c r="AD26" s="1">
-        <v>0.637</v>
+        <v>0.491</v>
       </c>
       <c r="AE26" s="1" t="s">
         <v>181</v>
@@ -5917,15 +5917,15 @@
       </c>
       <c r="J27" s="2">
         <f>IF(COUNT('Turns'!D81)=1,SUM('Turns'!D81),"Unknown")</f>
-        <v>677.0</v>
+        <v>687.0</v>
       </c>
       <c r="K27" s="2">
         <f>IF(COUNT('Turns'!E81)=1,SUM('Turns'!E81),"Unknown")</f>
-        <v>0.000118118898</v>
+        <v>0.000119863638</v>
       </c>
       <c r="L27" s="2">
         <f>IF(COUNT('Turns'!F81)=1,SUM('Turns'!F81),"Unknown")</f>
-        <v>0.0001354</v>
+        <v>0.0001374</v>
       </c>
       <c r="M27" s="2">
         <f>IF(COUNT('Turns'!D80)=1,SUM('Turns'!D80),"Unknown")</f>
@@ -5950,15 +5950,15 @@
       </c>
       <c r="S27" s="2">
         <f>IF(COUNT('Turns'!D86)=1,SUM('Turns'!D86),"Unknown")</f>
-        <v>34.0</v>
+        <v>35.0</v>
       </c>
       <c r="T27" s="2">
         <f>IF(COUNT('Turns'!E86)=1,SUM('Turns'!E86),"Unknown")</f>
-        <v>3.5592696e-05</v>
+        <v>3.663954e-05</v>
       </c>
       <c r="U27" s="2">
         <f>IF(COUNT('Turns'!F86)=1,SUM('Turns'!F86),"Unknown")</f>
-        <v>4.08e-05</v>
+        <v>4.2e-05</v>
       </c>
       <c r="V27" s="2">
         <v>0</v>
@@ -5971,22 +5971,22 @@
       </c>
       <c r="Y27" s="2">
         <f>IF(COUNT('Turns'!E90)=1,SUM('Turns'!E90),"Unknown")</f>
-        <v>0.000153711594</v>
+        <v>0.000156503178</v>
       </c>
       <c r="Z27" s="2">
         <f>IF(COUNT('Turns'!F90)=1,SUM('Turns'!F90),"Unknown")</f>
-        <v>0.0001762</v>
+        <v>0.0001794</v>
       </c>
       <c r="AA27" s="5">
         <f>IF(ISNUMBER(Y27),ROUND(Y27*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="AB27" s="5">
         <f>IF(ISNUMBER(Z27),ROUND(Z27*'Reference data'!$B$2,0),"Unknown")</f>
         <v>18.0</v>
       </c>
       <c r="AD27" s="1">
-        <v>1210.737</v>
+        <v>1854.326</v>
       </c>
       <c r="AE27" s="1" t="s">
         <v>164</v>
@@ -6009,7 +6009,7 @@
         <v>111</v>
       </c>
       <c r="F28" s="1">
-        <v>677</v>
+        <v>687</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>176</v>
@@ -6022,15 +6022,15 @@
       </c>
       <c r="J28" s="2">
         <f>IF(COUNT('Turns'!D81)=1,SUM('Turns'!D81),"Unknown")</f>
-        <v>677.0</v>
+        <v>687.0</v>
       </c>
       <c r="K28" s="2">
         <f>IF(COUNT('Turns'!E81)=1,SUM('Turns'!E81),"Unknown")</f>
-        <v>0.000118118898</v>
+        <v>0.000119863638</v>
       </c>
       <c r="L28" s="2">
         <f>IF(COUNT('Turns'!F81)=1,SUM('Turns'!F81),"Unknown")</f>
-        <v>0.0001354</v>
+        <v>0.0001374</v>
       </c>
       <c r="M28" s="2">
         <f>IF(COUNT('Turns'!D80)=1,SUM('Turns'!D80),"Unknown")</f>
@@ -6055,15 +6055,15 @@
       </c>
       <c r="S28" s="2">
         <f>IF(COUNT('Turns'!D86)=1,SUM('Turns'!D86),"Unknown")</f>
-        <v>34.0</v>
+        <v>35.0</v>
       </c>
       <c r="T28" s="2">
         <f>IF(COUNT('Turns'!E86)=1,SUM('Turns'!E86),"Unknown")</f>
-        <v>3.5592696e-05</v>
+        <v>3.663954e-05</v>
       </c>
       <c r="U28" s="2">
         <f>IF(COUNT('Turns'!F86)=1,SUM('Turns'!F86),"Unknown")</f>
-        <v>4.08e-05</v>
+        <v>4.2e-05</v>
       </c>
       <c r="V28" s="2">
         <v>0</v>
@@ -6076,15 +6076,15 @@
       </c>
       <c r="Y28" s="2">
         <f>IF(COUNT('Turns'!E90)=1,SUM('Turns'!E90),"Unknown")</f>
-        <v>0.000153711594</v>
+        <v>0.000156503178</v>
       </c>
       <c r="Z28" s="2">
         <f>IF(COUNT('Turns'!F90)=1,SUM('Turns'!F90),"Unknown")</f>
-        <v>0.0001762</v>
+        <v>0.0001794</v>
       </c>
       <c r="AA28" s="5">
         <f>IF(ISNUMBER(Y28),ROUND(Y28*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>15.0</v>
+        <v>16.0</v>
       </c>
       <c r="AB28" s="5">
         <f>IF(ISNUMBER(Z28),ROUND(Z28*'Reference data'!$B$2,0),"Unknown")</f>
@@ -6094,7 +6094,7 @@
         <v>143</v>
       </c>
       <c r="AD28" s="1">
-        <v>1209.171</v>
+        <v>1840.509</v>
       </c>
       <c r="AE28" s="1" t="s">
         <v>177</v>
@@ -6193,7 +6193,7 @@
         <v>11.0</v>
       </c>
       <c r="AD29" s="1">
-        <v>1208.469</v>
+        <v>990.8049999999999</v>
       </c>
       <c r="AE29" s="1" t="s">
         <v>164</v>
@@ -6295,7 +6295,7 @@
         <v>11.0</v>
       </c>
       <c r="AD30" s="1">
-        <v>1206.442</v>
+        <v>988.484</v>
       </c>
       <c r="AE30" s="1" t="s">
         <v>164</v>
@@ -6397,7 +6397,7 @@
         <v>11.0</v>
       </c>
       <c r="AD31" s="1">
-        <v>1204.25</v>
+        <v>987.3869999999999</v>
       </c>
       <c r="AE31" s="1" t="s">
         <v>164</v>
@@ -6499,7 +6499,7 @@
         <v>11.0</v>
       </c>
       <c r="AD32" s="1">
-        <v>1200.459</v>
+        <v>985.467</v>
       </c>
       <c r="AE32" s="1" t="s">
         <v>164</v>
@@ -6607,7 +6607,7 @@
         <v>147</v>
       </c>
       <c r="AD33" s="1">
-        <v>1197.198</v>
+        <v>983.5170000000001</v>
       </c>
       <c r="AE33" s="1" t="s">
         <v>177</v>
@@ -6637,15 +6637,15 @@
       </c>
       <c r="J34" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1022.0</v>
+        <v>1026.0</v>
       </c>
       <c r="K34" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000178312428</v>
+        <v>0.000179010324</v>
       </c>
       <c r="L34" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002044</v>
+        <v>0.0002052</v>
       </c>
       <c r="M34" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6670,46 +6670,46 @@
       </c>
       <c r="S34" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>42.0</v>
+        <v>45.0</v>
       </c>
       <c r="T34" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.3967448e-05</v>
+        <v>4.710798e-05</v>
       </c>
       <c r="U34" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.04e-05</v>
+        <v>5.4e-05</v>
       </c>
       <c r="V34" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="W34" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="X34" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="Y34" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.000232748316</v>
+        <v>0.00024077412</v>
       </c>
       <c r="Z34" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.0002668</v>
+        <v>0.000276</v>
       </c>
       <c r="AA34" s="5">
         <f>IF(ISNUMBER(Y34),ROUND(Y34*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="AB34" s="5">
         <f>IF(ISNUMBER(Z34),ROUND(Z34*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
       <c r="AD34" s="1">
-        <v>2213.523</v>
+        <v>2761.857</v>
       </c>
       <c r="AE34" s="1" t="s">
         <v>164</v>
@@ -6742,15 +6742,15 @@
       </c>
       <c r="J35" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1022.0</v>
+        <v>1026.0</v>
       </c>
       <c r="K35" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000178312428</v>
+        <v>0.000179010324</v>
       </c>
       <c r="L35" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002044</v>
+        <v>0.0002052</v>
       </c>
       <c r="M35" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6775,46 +6775,46 @@
       </c>
       <c r="S35" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>42.0</v>
+        <v>45.0</v>
       </c>
       <c r="T35" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.3967448e-05</v>
+        <v>4.710798e-05</v>
       </c>
       <c r="U35" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.04e-05</v>
+        <v>5.4e-05</v>
       </c>
       <c r="V35" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="W35" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="X35" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="Y35" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.000232748316</v>
+        <v>0.00024077412</v>
       </c>
       <c r="Z35" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.0002668</v>
+        <v>0.000276</v>
       </c>
       <c r="AA35" s="5">
         <f>IF(ISNUMBER(Y35),ROUND(Y35*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="AB35" s="5">
         <f>IF(ISNUMBER(Z35),ROUND(Z35*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
       <c r="AD35" s="1">
-        <v>2210.998</v>
+        <v>2758.871</v>
       </c>
       <c r="AE35" s="1" t="s">
         <v>164</v>
@@ -6847,15 +6847,15 @@
       </c>
       <c r="J36" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1022.0</v>
+        <v>1026.0</v>
       </c>
       <c r="K36" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000178312428</v>
+        <v>0.000179010324</v>
       </c>
       <c r="L36" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002044</v>
+        <v>0.0002052</v>
       </c>
       <c r="M36" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6880,46 +6880,46 @@
       </c>
       <c r="S36" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>42.0</v>
+        <v>45.0</v>
       </c>
       <c r="T36" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.3967448e-05</v>
+        <v>4.710798e-05</v>
       </c>
       <c r="U36" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.04e-05</v>
+        <v>5.4e-05</v>
       </c>
       <c r="V36" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="W36" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="X36" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="Y36" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.000232748316</v>
+        <v>0.00024077412</v>
       </c>
       <c r="Z36" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.0002668</v>
+        <v>0.000276</v>
       </c>
       <c r="AA36" s="5">
         <f>IF(ISNUMBER(Y36),ROUND(Y36*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>23.0</v>
+        <v>24.0</v>
       </c>
       <c r="AB36" s="5">
         <f>IF(ISNUMBER(Z36),ROUND(Z36*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>27.0</v>
+        <v>28.0</v>
       </c>
       <c r="AD36" s="1">
-        <v>2209.448</v>
+        <v>2757.654</v>
       </c>
       <c r="AE36" s="1" t="s">
         <v>164</v>
@@ -6997,23 +6997,23 @@
       </c>
       <c r="V37" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="W37" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="X37" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="Y37" s="2">
         <f>IF(COUNT('Turns'!E118)=1,SUM('Turns'!E118),"Unknown")</f>
-        <v>0.000109744146</v>
+        <v>0.000113931522</v>
       </c>
       <c r="Z37" s="2">
         <f>IF(COUNT('Turns'!F118)=1,SUM('Turns'!F118),"Unknown")</f>
-        <v>0.0001258</v>
+        <v>0.0001306</v>
       </c>
       <c r="AA37" s="5">
         <f>IF(ISNUMBER(Y37),ROUND(Y37*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7024,7 +7024,7 @@
         <v>13.0</v>
       </c>
       <c r="AD37" s="1">
-        <v>1152.349</v>
+        <v>1506.315</v>
       </c>
       <c r="AE37" s="1" t="s">
         <v>164</v>
@@ -7105,23 +7105,23 @@
       </c>
       <c r="V38" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>10.0</v>
+        <v>14.0</v>
       </c>
       <c r="W38" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.046844e-05</v>
+        <v>1.4655816e-05</v>
       </c>
       <c r="X38" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.2e-05</v>
+        <v>1.68e-05</v>
       </c>
       <c r="Y38" s="2">
         <f>IF(COUNT('Turns'!E118)=1,SUM('Turns'!E118),"Unknown")</f>
-        <v>0.000109744146</v>
+        <v>0.000113931522</v>
       </c>
       <c r="Z38" s="2">
         <f>IF(COUNT('Turns'!F118)=1,SUM('Turns'!F118),"Unknown")</f>
-        <v>0.0001258</v>
+        <v>0.0001306</v>
       </c>
       <c r="AA38" s="5">
         <f>IF(ISNUMBER(Y38),ROUND(Y38*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7135,7 +7135,7 @@
         <v>152</v>
       </c>
       <c r="AD38" s="1">
-        <v>1150.31</v>
+        <v>1504.393</v>
       </c>
       <c r="AE38" s="1" t="s">
         <v>177</v>
@@ -7167,7 +7167,7 @@
         <v>208</v>
       </c>
       <c r="AD39" s="1">
-        <v>2.011</v>
+        <v>2.889</v>
       </c>
       <c r="AE39" s="1" t="s">
         <v>181</v>
@@ -7199,7 +7199,7 @@
         <v>210</v>
       </c>
       <c r="AD40" s="1">
-        <v>0.48</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="AE40" s="1" t="s">
         <v>181</v>
@@ -7232,15 +7232,15 @@
       </c>
       <c r="J41" s="2">
         <f>IF(COUNT('Turns'!D124)=1,SUM('Turns'!D124),"Unknown")</f>
-        <v>549.0</v>
+        <v>553.0</v>
       </c>
       <c r="K41" s="2">
         <f>IF(COUNT('Turns'!E124)=1,SUM('Turns'!E124),"Unknown")</f>
-        <v>9.5786226e-05</v>
+        <v>9.6484122e-05</v>
       </c>
       <c r="L41" s="2">
         <f>IF(COUNT('Turns'!F124)=1,SUM('Turns'!F124),"Unknown")</f>
-        <v>0.0001098</v>
+        <v>0.0001106</v>
       </c>
       <c r="M41" s="2">
         <f>IF(COUNT('Turns'!D123)=1,SUM('Turns'!D123),"Unknown")</f>
@@ -7265,15 +7265,15 @@
       </c>
       <c r="S41" s="2">
         <f>IF(COUNT('Turns'!D129)=1,SUM('Turns'!D129),"Unknown")</f>
-        <v>26.0</v>
+        <v>29.0</v>
       </c>
       <c r="T41" s="2">
         <f>IF(COUNT('Turns'!E129)=1,SUM('Turns'!E129),"Unknown")</f>
-        <v>2.7217944e-05</v>
+        <v>3.0358476e-05</v>
       </c>
       <c r="U41" s="2">
         <f>IF(COUNT('Turns'!F129)=1,SUM('Turns'!F129),"Unknown")</f>
-        <v>3.12e-05</v>
+        <v>3.48e-05</v>
       </c>
       <c r="V41" s="2">
         <v>0</v>
@@ -7286,22 +7286,22 @@
       </c>
       <c r="Y41" s="2">
         <f>IF(COUNT('Turns'!E133)=1,SUM('Turns'!E133),"Unknown")</f>
-        <v>0.00012300417</v>
+        <v>0.000126842598</v>
       </c>
       <c r="Z41" s="2">
         <f>IF(COUNT('Turns'!F133)=1,SUM('Turns'!F133),"Unknown")</f>
-        <v>0.000141</v>
+        <v>0.0001454</v>
       </c>
       <c r="AA41" s="5">
         <f>IF(ISNUMBER(Y41),ROUND(Y41*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="AB41" s="5">
         <f>IF(ISNUMBER(Z41),ROUND(Z41*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="AD41" s="1">
-        <v>1050.807</v>
+        <v>1244.071</v>
       </c>
       <c r="AE41" s="1" t="s">
         <v>164</v>
@@ -7324,7 +7324,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="1">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>176</v>
@@ -7337,15 +7337,15 @@
       </c>
       <c r="J42" s="2">
         <f>IF(COUNT('Turns'!D124)=1,SUM('Turns'!D124),"Unknown")</f>
-        <v>549.0</v>
+        <v>553.0</v>
       </c>
       <c r="K42" s="2">
         <f>IF(COUNT('Turns'!E124)=1,SUM('Turns'!E124),"Unknown")</f>
-        <v>9.5786226e-05</v>
+        <v>9.6484122e-05</v>
       </c>
       <c r="L42" s="2">
         <f>IF(COUNT('Turns'!F124)=1,SUM('Turns'!F124),"Unknown")</f>
-        <v>0.0001098</v>
+        <v>0.0001106</v>
       </c>
       <c r="M42" s="2">
         <f>IF(COUNT('Turns'!D123)=1,SUM('Turns'!D123),"Unknown")</f>
@@ -7370,15 +7370,15 @@
       </c>
       <c r="S42" s="2">
         <f>IF(COUNT('Turns'!D129)=1,SUM('Turns'!D129),"Unknown")</f>
-        <v>26.0</v>
+        <v>29.0</v>
       </c>
       <c r="T42" s="2">
         <f>IF(COUNT('Turns'!E129)=1,SUM('Turns'!E129),"Unknown")</f>
-        <v>2.7217944e-05</v>
+        <v>3.0358476e-05</v>
       </c>
       <c r="U42" s="2">
         <f>IF(COUNT('Turns'!F129)=1,SUM('Turns'!F129),"Unknown")</f>
-        <v>3.12e-05</v>
+        <v>3.48e-05</v>
       </c>
       <c r="V42" s="2">
         <v>0</v>
@@ -7391,25 +7391,25 @@
       </c>
       <c r="Y42" s="2">
         <f>IF(COUNT('Turns'!E133)=1,SUM('Turns'!E133),"Unknown")</f>
-        <v>0.00012300417</v>
+        <v>0.000126842598</v>
       </c>
       <c r="Z42" s="2">
         <f>IF(COUNT('Turns'!F133)=1,SUM('Turns'!F133),"Unknown")</f>
-        <v>0.000141</v>
+        <v>0.0001454</v>
       </c>
       <c r="AA42" s="5">
         <f>IF(ISNUMBER(Y42),ROUND(Y42*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>12.0</v>
+        <v>13.0</v>
       </c>
       <c r="AB42" s="5">
         <f>IF(ISNUMBER(Z42),ROUND(Z42*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>14.0</v>
+        <v>15.0</v>
       </c>
       <c r="AC42" s="1" t="s">
         <v>158</v>
       </c>
       <c r="AD42" s="1">
-        <v>1048.948</v>
+        <v>1242.056</v>
       </c>
       <c r="AE42" s="1" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
Publish workflow samples, refreshed reports, and rebuilt distributions
</commit_message>
<xml_diff>
--- a/reports/claims_context_managed/report.xlsx
+++ b/reports/claims_context_managed/report.xlsx
@@ -75,13 +75,13 @@
     <t>Parent ID</t>
   </si>
   <si>
-    <t>Fresh input tokens</t>
-  </si>
-  <si>
-    <t>Fresh input EUR</t>
-  </si>
-  <si>
-    <t>Fresh input USD</t>
+    <t>Input at standard rate tokens</t>
+  </si>
+  <si>
+    <t>Input at standard rate EUR</t>
+  </si>
+  <si>
+    <t>Input at standard rate USD</t>
   </si>
   <si>
     <t>Cache read tokens</t>
@@ -165,7 +165,7 @@
     <t>Run ID</t>
   </si>
   <si>
-    <t>01a0ccdf-b7b4-7282-a01f-e7dd9f070b7d</t>
+    <t>01a0d12d-5d05-7c53-873c-3dc935c4adaa</t>
   </si>
   <si>
     <t>Recording</t>
@@ -177,13 +177,13 @@
     <t>FX reference date</t>
   </si>
   <si>
-    <t>2026-09-22</t>
+    <t>2026-09-23</t>
   </si>
   <si>
     <t>FX fetched at</t>
   </si>
   <si>
-    <t>2026-09-23T06:06:28.037095Z</t>
+    <t>2026-09-24T02:09:35.117183Z</t>
   </si>
   <si>
     <t>UTC</t>
@@ -306,10 +306,10 @@
     <t>gpt-5.6-luna</t>
   </si>
   <si>
-    <t>01a0ccdf-b7bb-7643-9f73-5583342bd8b2</t>
-  </si>
-  <si>
-    <t>Fresh input</t>
+    <t>01a0d12d-5d0b-7902-932d-67b7882261bb</t>
+  </si>
+  <si>
+    <t>Input at standard rate</t>
   </si>
   <si>
     <t xml:space="preserve">    Tool definitions</t>
@@ -357,8 +357,8 @@
     <t xml:space="preserve">    Output content</t>
   </si>
   <si>
-    <t>[{"id": "rs_08acf24a3e239f6a006ab36c795cb087d28ebbb1d47994f32f", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x5_Wgphp9Sf8NFOLXYsJNwFrOGSvHpwsXSNNJrZbRlaAdLrEIv2LZc7i3SZshIgBijJJPSCWpWKgvmqyjAB3-y4Bg0ZPyuHNtAcM_8iEjFKxvq0ZoUyq0fyPRacA8au8U4Na_TujB9F93P5gz0vbBPiRTtbsKx8OToiBd2id6X5vKBSOYYj4HAQqdy_GieOrYoFZcUAOghheMqZCQv8LYiGxh1KHnZKAFfg0oyopHuWw7W79VDqhoIcXF3JdEU1l3Bh3vLFVTAFAvNeeGXsA_nTWbeYOJ-opbm6Pl2BrNjBQRorbv8MJv-3pzGu0IG8CnCVEM-ja7BCwm-0lh5n5xpYLSHb-Zb11OccCrrts9I3aFpTVcbS8P8GKKjpVr5ySUKijGaY_VZIb7_dDtAiBbiuY4PI3SFl4KsaFtwKfeLj5do8Wx49KM7OlFHQrWMpbWcYsq5smhis-Loc3u05QeLqAJbxv-K37r3O_rrNHA_Xh77QSq75XdwpGsBWObENsaC4w7M4SCZVnZAiPhS4eixcQiRmcC1aqEpSjADyUZPVXnV8HYBQnKPpr_A71TXqfbOxjvNsrHHx3xYfy_ihIXIKGhRqHTFKd9EqZjA4GTS7CtFbJelrlur9jMOyb30CV2VAsZQL9gMA1d3lEhnTl_QsvH8b_l8OCaZOLGBY7wYVQlOEMG465esivFJndemdcVqe0LzW2_NKmS7lOHzqmiORe0rMZmlr1ZOQBTpAQClpghkdO6XpL4tOlSlB157f6G_eUyQy1MB8GACtlNYKfvCCNjzPQZHgRbd3iGHf6GABuMDnmPOx-S3Y1595G5mq4nrMXq2HQJGShD7hn1JfERyQDLK6F-g3FR8muhl57akKzZcqW0I4_lhw3swc6-p0A4oU9TAlTTOriJFXRmk2V2gNvNwXtCW2WtjmqhnPpdTgQZYN3lMqQZKKAMezRuuOJ-af_uAn1a4o4JTumnZSqj_HJvXjX2ln9fIrG8Uz1LVREi8qaaJKG6srgCda-WQnUcn_aWgU5zcPYwDQIA_dJobLTEp_u8TWcMeZrd8PTm77BJJHMW4i2WnAF_xFWb3xwBA5KpoylSeq7IT-b63ZKpFV-gtbSwxR_us3NS26IgnzJDy9TtfLfYK1h9Acpb1b8-3lD24Mb9-Xf2FUR2IIMrscjyVSUSCBhOR9xZxQVyCCDdprRg7x5E_PAkJB0vdmRET"}, {"type": "function_call", "name": "read_policy", "arguments": "{}", "call_id": "call_KpG3hBdlMxiECjhYb4CXiCnZ", "id": "fc_08acf24a3e239f6a006ab36c79963087d28b6769ea89a88da9", "index": 1}]
-{"name": "read_policy", "args": {}, "id": "call_KpG3hBdlMxiECjhYb4CXiCnZ", "type": "tool_call"}</t>
+    <t>[{"id": "rs_0872d4ff337ce520006ab4867f168887d28ff77936cf2ef367", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqtIZ_yo0G6yBGuzkFqSjEu6yyUpW4f7pzqEeQilqfCRPD2ZHmFzANXtZTBRmAC8B8ZbGBzBLrI84K_vyjBTVlsxnCDnU78iadJMG3wsBNOxpAuCjncan58UPvZK9YuAbOc_qQ2DzSOk2Fs-Fn9zb4pRVqJu6-49H2j6fkhP5LPIBeNA4aTMkVD1SyZh-juu51u52r6dLTgwlQLnnOufJRlZOR8F9OrLsi-uWT8JKuD_EnEPsmvyFmXQ4soV7NvK5ckJzpFeXl3VaQmdqmA8lEZfA_wzf0OVsV22DcTv1wLB4gSVEcGU1y-jhhBCKAzUxsms_sxOcZPaE1EuOcE28FuIhcQsBkMsLl4yk4l377DV5dq_if0POZCM0_DeTtL5TbxGgEXyI_FaiPGo4hpJ0_IUgKimiXoveD4xMIc47e0Bn0KZRkJedjvyi8Pl2kLKL7hEe1TDqJWIE677fYhPLRyyUFLvG6FiG55dnVA9jVLaGH97jh8gSiZWqXJ2rg7nbi_ek7lGyS9bcQyqYPdKjsAVjsd0x82heiiKm9v1A3vcNhtjNnoWn3fWwKq_ZvCP9OiFdp7pspNnGAXbVvcuLEqFhGIUCglcwMrUO8O1RLJr9em4SgMIY-TGyccpbS45FroAPW6unmxZZbWrkHGkGa_znD9FBmqIvrHeYTuwHw_eL29Y8BEvi8Az9WtvFQFz-NGdjYzG7xkmRgKW9ci9QksSqJGC0z_BADp8eBD6jlEaUPqBpILL_TirnXNWJTAhJjD7EFmlv675FJQUQl9V3OasaDoANNkx2JZqgGyGAUUPsc_Nfmw2Gfa-ZPk255sTv4M26m1sR6wUjBbrNysxo9dIkOQZBiiJSG--BlkHiLHzO6hOJLIhz-LQjf2QwKnLbIgP71LhmO91j8xCZ-z2AsbgTkVi4mysI21LosqBVrTJyhkMcdJQwzAbmqzrnE39CJ7XBXLgf7l-1k5yGkLZ0kWDAJo4Qr5x8g0bVV5L-PrrnPTt_H86fv7jsOZ45mwfQWaAIRV49hlWfCxmzpC5dOoCeUbKj-FIY7Gf4iiG4e-C-yv4-hHh7e8JaCXk9xCVn-eZk9nwPiD0oxKtAvUVMaoMglrymXArw-Nh3KGZJCSI9GAFUut8sEmoZws2OHns_p_YQwHexgL75DYFM9phTFGWo9r5sYdSEir8L51BVI-BPuxQmvTXd2WXvyxsRVuX52tHan"}, {"type": "function_call", "name": "read_policy", "arguments": "{}", "call_id": "call_ghLY0nrmhuwMrIp5bp3MzZhe", "id": "fc_0872d4ff337ce520006ab4867f3f6c87d28b0668249fde2426", "index": 1}]
+{"name": "read_policy", "args": {}, "id": "call_ghLY0nrmhuwMrIp5bp3MzZhe", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Call total</t>
@@ -370,7 +370,7 @@
     <t>Tool · read_policy</t>
   </si>
   <si>
-    <t>01a0ccdf-bc28-74a1-9d0f-67b8c1faddaa</t>
+    <t>01a0d12d-61d8-7ef0-80c1-f5c6deb83ff6</t>
   </si>
   <si>
     <t xml:space="preserve">    Arguments</t>
@@ -388,7 +388,7 @@
     <t>R2</t>
   </si>
   <si>
-    <t>01a0ccdf-bc2b-72c0-88f0-5490bade1f97</t>
+    <t>01a0d12d-61db-7cc2-b075-b20f700aafe7</t>
   </si>
   <si>
     <t>Conversation history · cache read</t>
@@ -397,7 +397,7 @@
     <t xml:space="preserve">    Tool result</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "Policy POL-001 applies a **CAD 150 deductible** to accidental laptop damage.", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c7a8ae487d2a2bed20de84b96d9"}]</t>
+    <t>[{"type": "text", "text": "Policy POL-001 applies a **CAD 150 deductible** to accidental laptop damage.", "phase": "final_answer", "index": 0, "id": "msg_0872d4ff337ce520006ab4868052f887d2b48768f1d412be0a"}]</t>
   </si>
   <si>
     <t>Turn 2</t>
@@ -406,20 +406,20 @@
     <t>R3</t>
   </si>
   <si>
-    <t>01a0ccdf-bfdf-7370-a947-75db376a8377</t>
+    <t>01a0d12d-6664-78b0-b59f-969bd2228f7a</t>
   </si>
   <si>
     <t>What happened in claim CLM-001, and what is its status?</t>
   </si>
   <si>
-    <t>[{"id": "rs_08acf24a3e239f6a006ab36c7b6b1c87d298298a6c599f981d", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x7y1_D29XwcxpNBCWtwTjbHl126ixQ1Vy0A_gmMEggm99GUqg7KwDS7Xpkev-Uup9_LRQ_-WQP9avAuzN89L2vMWtLdvDrZvZiowgpwN5eAfizhKpLgjc3vVU1ThawGCO0eX6DIKDM9nOh4is8Dyt2AkM7Ux1UcTLvm1UgW2iJdXG1PyurLpied_NYuaSEzh3gtlhx5w1YBzdwMGBRVgyA0aS8T8IYIQsOo-oP1dODeGCyMoH88acRxYkUCIqgfyqTpczzaPmqdvOKsyiMjo3uTq_vdCaDJgrpxFijwxXixXO5tGzP5BPCr92Pg0Ap2VUJ7dKNWVwli-0VSkQbZyFXC0XCuG-sydsYvcTo_dJcB3z7HzRE9P1Ade4GPfMtBoq3earqeK1aafwu2798jo1ILDwx-uDh0ADwqSQzcwb5fdcrkRaEqoEI2ElxW2n4nfKoskbkFTejjCW46yIsNdC3YC3cqgaqmoAq7kOoTMYt1XuOtVMz8rXzKG0JVNGoW9HDe_cmBFg5dX7o-XVdvvS0FmkE56YQQJNRwcWiObNegnoH_uuSopRG9Wl3q4rnZOrZDFGTyFOKTs0MwBFpLAsu3Dfrak3BUfCL12aG0Uou2RXajjQT3O4UmIorpS6tBYq94m7NpAlK_t4hYEmvvpZaotxBV1AMT00RlS4pOf4D1ioFbnW8PF1XNEL5EG1Z3AkoFBzeBjkuJHZgynw2cLtlZyCMh74-ZlYE4LI7bdwLLfiuhrfwhPUIWwe3xtd0QV9_zpxBDCCfulN4GPz7oE6CdTNbfk88UOBo1_hI46zZM-MGTuDckg0GjKO4y8zJ4lIgsUAfN8ishSxhie4zc0mlnAiy2WzA2ktluANdt4uNk84hXyGghThjuOS8HentlSMnCBnUxakBXYKZ0exgIDUZewT0_1DDGIxUcOijy3XyqtcFC9yBuq2nypj2qT9zFld8J7vHnjTDiNs7Y_tGVGZhGiqxw16Pw4Rv_pjT5NIOSQBQx4HDJLMcwjaxlumHHPyZNu6rDsFIPs8LFioOulPF6_kVcNf46GVHL68ZGj8lrbktNs0-_0jjTvfQ8RSmJlVrx90vvKSYKb3UkqBNj1h_d0_2VAzH7_qEDGGBoqfhTbg1QL-NuNe3a45gOs1HYuv_WFgbsJwlhax7oQl91IWudRhdGwsIp7pPZKNCgY39IuD4jI-IR3Ju9Mu372ceADvM"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_78AYLUwYWh6NWaqvO8hpsVMS", "id": "fc_08acf24a3e239f6a006ab36c7bced487d2b2a1a89aa0a6b9ac", "index": 1}]
-{"name": "read_claim", "args": {}, "id": "call_78AYLUwYWh6NWaqvO8hpsVMS", "type": "tool_call"}</t>
+    <t>[{"id": "rs_0872d4ff337ce520006ab486815bc087d2b02a6414ea2148cf", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqtIaBmBKfkQE1Qeg5yLqLuzTVmLzCzv8Ox2_D1i0iKyGiqhseMGAhMIhivGMMMrCcTdr61manV47dSALn0SFvCKEqaqqr_nqNYJ-XAQkjSBL5Dd1Zg0wP-0EBrR5owMYWCFvuE7Xvv6iU5n1Z6FwNyCheXyleWVyp6l-FAG7qY4694nh0oEUjcBsB4hSFQIIrawFsoKZq19-Q15wmdkouyEVv9lCjQ4EalGXln1PIwu6o4QstSagobPFvFVcS_Y1RV6qLutdHph6iBTrjbJi7JYbV5zI-NSXhUv1oprk62wT6jChtuPhHyRFBzd1TzibB4yfm8TngBPj_ooOmZHkeXpIX0eLsxhmDHLuMeHVaEicWSAmR28ZMlT28402FnCpEBY6mgJNXe30ZhHPYlYBWspU8j3aunE02HzIQZWc4hA8OjKNGp0gzy_I_LhEx3Qmx_0Cn4h30C1iKGl78ilwGFrcwBoTvgQJvjVdS2ow9ODOdyr7npcrBW-qvrnBt7y6ZXvjft9UV5aIplMXc5ZqisWfjVcjWpp15_e8EJWrYttcn0QCTa2Qcq8DyezJ631qJr2esMsFqgOin8hMZuxjIPOXIGTnoVFbZqiytlvJiFmllA0KnHKQT-CdM64bo3zCp8bn3AcgToEGjQ7MUOtx9vrLI-2K5o6FdFg9qaeeH4NoIfTQrofARG0sKpW6US1rRTvCllyUg1q9424b4hGdk_2AEDF8J7zG56aFKNRo7HvZHT4gORzlzAj-ynkLGPBPfXRaVyP2inHuUu0cblVtR3v4zyB7R2QBixSrM-xwL15WzmANsMjc3AXdM_UxRgfdgeGszWPvF40i6ycm3fKaxwE2QGA-xATHgMVO6vNGgOiqaE780Tay-hrC3MAHK9HsOMhnovKk3VE_wqgE_RAa5aYxsFh8Q9l5DhGXebmiJdGD6r1wi3BrO_UuL76NeWowmZAQVp3v6Bi8hvSej9WmlG4nlNN9Ct-LkelGZ0q7vK5T7V1zlWMtc8f6a1AxVRsHVgxybMJv2HwdaU-NywFgBqL2w0zk0SRALvf-W4s8BVCGKin73sO7yOFXbeWA4qKuzUoQ_EPEcOajoUgDtH2V6B_a7lHTYgc69mfWmYMzwB5J3el4MIVw7tBfsF-TEkRLs5W3dtiEGUPc6qyF5eBJ5bCfn3lrpvnNKzGyWZ38AwV3rL-Gd6v92MJ4XQm1aQdcn-CFE"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_b3KToV0FVuAnZl86LmL1Kdgg", "id": "fc_0872d4ff337ce520006ab486817cc087d2971a3acf1f70fc28", "index": 1}]
+{"name": "read_claim", "args": {}, "id": "call_b3KToV0FVuAnZl86LmL1Kdgg", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Tool · read_claim</t>
   </si>
   <si>
-    <t>01a0ccdf-c7a7-7571-982f-202ee708c675</t>
+    <t>01a0d12d-6ac1-7993-9dd9-5da7c71357d1</t>
   </si>
   <si>
     <t>{"claim_id": "CLM-001", "revision": 1, "description": "A laptop was stolen from a parked car.", "status": "pending"}</t>
@@ -428,10 +428,10 @@
     <t>R4</t>
   </si>
   <si>
-    <t>01a0ccdf-c7aa-7073-9062-c33e52e5abcc</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "Claim CLM-001 concerns **a laptop stolen from a parked car**. Its status is **pending**.", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c7d6c7c87d2a3a592be1fba4fe9"}]</t>
+    <t>01a0d12d-6ac4-75b3-97d5-b28c317fd852</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "Claim CLM-001 concerns **a laptop stolen from a parked car**. Its status is **pending**.", "phase": "final_answer", "index": 0, "id": "msg_0872d4ff337ce520006ab48682a41c87d29c91f7e237958e4f"}]</t>
   </si>
   <si>
     <t>Turn 3</t>
@@ -440,20 +440,20 @@
     <t>R5</t>
   </si>
   <si>
-    <t>01a0ccdf-cbc9-71c2-bf15-0ce6b5568029</t>
+    <t>01a0d12d-6f86-7f40-8b7e-fdb723a119b2</t>
   </si>
   <si>
     <t>Correct the claim: the laptop was not stolen. Its screen cracked when it fell from a desk at home. Replace the description with 'The laptop screen cracked when it fell from a desk at home.' and change the status to approved.</t>
   </si>
   <si>
-    <t>[{"id": "rs_08acf24a3e239f6a006ab36c7eca4887d2b43c97c61c8f7a94", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2x_jYNbPJ18Vz45kZQLd0QPFXPKxTnH0RqCGG4eb9Ir4lwm3Z1gwvhHt-L_bONsAHnc0-nwLsaD8MGIONU8kuaVa9_cVHlG77yoo0XjeU8xwhJz6-019Y4TUMBheHwGT4PL-JeHvVDeMrKxmAC4PxYSqjvCnjdSGcDfEsrx7_bZxG6j8L4tjvIUEg5alFHbg5i5Cwssirjt_Kx-Zs59D6Sv09C7WEjEYoEt7pwQZtRQUWzjMYo6Ha-PShe3Bm18-2sUnHKC4_ilSKhF1euFW4ngCEAdK7e-NzgK5z1Cc6ZsgR08VZdDpsg2x8lpX0_sgxs-4lx7jcq_q_bmSpdNzMf4hykh0UUVo0rneMqNNkk8cRLFGauha69TC333MA7YcGOcvHHqvSWwDw5jTPNBQs38Ce-GDSbZePt4le9qwU60_L53xH6baWrc6c4o2ACOIWZl6U7hB7nYOti3pwWCQEXvJJ26s-QrqYApgaKPqIoKDe48GcHwyYxh364To-3yM7Omp-LFbxVy0pFvkGxbOsbqdFWkQpDe9_XCDUizpT4MT_wH9hd_CwV972cSB5Z2rXrpxlyiO_d3Um0iAcjOw4t0Q_AxN-Yfg9hY9BiDl-RVkZFSMDCdtczcf61ozbC-hUz78P4hFxts9ShXrg0Cii2MVaigtI9NJaHyG9HKNO0oJfx47KvgNIgNRwntMoWF4gvdyKbekpXY-bx_kN6vq0fDayWJtEmeaGO1YeyYl_bGFWlzMKdBX4rLstK0UlUX8N-40lGkxAB7Ql2ITfrHmQJHwj6v5G1skKuIgLvpkmlDX-n26trlATBqr1py6OcoHxx9fhMFjFOA4bOKNCAjFEzhn5GDyGOnyH3VShOgubn3BBAGnGgz7Z_bvrJmRRaer1s9vyy9RLgHpG6RblCZYDk-GpHeq2JTJF1vUAaYPYXkLioIxwMocNbcNZ8nTC2KHbHwhQq4A_AWwaZAl5inh9SwaT5xB1EMuNCdRdhge2h6PhvN7MzUbt1K_2UkyScN2PvsDe5Ak84rCxsPEKzV9f83m768HugqTwSkygp6X7xUAv51f7JVAFUmVXpWlm4pc4eHqA5dhMmKjvVtE0KlLd2cIPsfFxCrnby4ysuN6fSxroK9jYqQt608-N7dw9GmQLpxb6dGaO4avTqCxzGZC3jsL9XM0mIC3FFFWhrB8k4T1DSe94FGHxXK0pPd97E9_Ce3fFVjoFl43XOqQmvvnSzK8zEV5jyFTit3JCB_g_Sl02TqBbfbY9u8FYyD9zMmb3tR"}, {"type": "function_call", "name": "edit_claim", "arguments": "{\"expected_revision\":1,\"description\":\"The laptop screen cracked when it fell from a desk at home.\",\"status\":\"approved\"}", "call_id": "call_dYUixnYLB2nLVku0kx5CQMiT", "id": "fc_08acf24a3e239f6a006ab36c7f120087d2b40371b1dfbf91da", "index": 1}]
-{"name": "edit_claim", "args": {"expected_revision": 1, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}, "id": "call_dYUixnYLB2nLVku0kx5CQMiT", "type": "tool_call"}</t>
+    <t>[{"id": "rs_0872d4ff337ce520006ab48683e04487d28651c044068e19bf", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqtIaEpvOXl1RTXbTqhKnzLQ8Xy7oOkSIyIVwxUag4mnP05hnJfm22sjVmDGPJQQn2ywdFCJ-BcZnlQHG6J3FH1vfi0mZmgwm8b_8Wjj_M5xrXck-2yEt4bjhDuhatPpWLdOdM_rF2yDnKlszeSSLxyO9DUT5TuEN3nBP6sbffeciN2WgI7ZLrKiZuletyLk6infMfCZfcLwD6QeRDnzGy9kSZNRzJ7QjUkDJKPP3aAKw0bJtRk_tE2vWp5wGcl6GnPDOpvCPuEVxnKNZuWot8OwAkOdroFkjn3E62b4CmPAqPao31mBr1B4j1qNAY4yWXBtEts3SO80rM2in7KcS9XsbhrzDba6tr4Yc6XpE7ALlj0ZQPr-H98FKJiLPCqWrhUyWiCbzsmq6k_-nObY7gT0dCzw43yCy8IEY9Dygb8DIe_f3_DwgHVxRynb95vMu_UuIWVRcy9UoQhVp7PPM598YB46RN1dnDIIJY9Pz_muXZB8q6imWOOKNfGsXEpK7obiDEeB89JaymhRxEaVo1VdvW3vqRy877pIPU7Z5zO00OLyzCaD_ulhEPQNkwYvVXkjpDEuGFs85suxeVxOBsdDaAYNJbbEA7SfJ-THsIuZX0_PjIUSUxpukwmyWdlR9DtXzVEKVAX7OzWYVq3DfaK8f0rkoEGivveSPpIM_-cnn-TvIGnSv6T990hA9PA15lBTYXJWOb5vnlyb5izuMon56XTUm80RJjgj3UbN_JRA7KsDGhjEtM3nqqLoZxTSzfXW1AeCrfmSETxxi4bJIcziKOwVD3VO-Icv21ygGQTdK_2XR5cWd-UhIWDdiiQ4U_mL35VHvYxsfQeYRkREO-kzZJJ2F-5IdghN8NhrBs7vLyj8OTgXzb3TEqDXgKHw8AyylH1vavW23N9FKWlvoKm4-rcRpkSIi23AmRC7JHlTjhbYUsZzbIbGZX_taQ6mqjKGriQ_V0PiJXv2eEmAXkQgIU0sq6kM4S_Gxvp_lp428Zvl4s3rQDM_ig8qDO9JUOhxuAv5sFogdX2iWFhrj5bfArtrAL6p-crr8hwQ7KY1sUlz5cj6QGhuWk0fJCLQBbyl7v5WcTVoCKMU6CvFsp6V9_pRaOeXDqS5zRvB26GcOAWgMQwY4iTw_ps2IlI7M62NZbGOeALfobm5CL0YJrBihgDONNjSaGQYrhMD7lnTcM2UtF8YubTOvoGb-0n1H6IbGgRVO8tikS4FZa5wU5U7eBeBIHkwXw0fV4GtyZqz_fIlpdolT7Z3aF3PD0tgSmdxoZJBD5MFVscPPfZcl4_k_U3Q=="}, {"type": "function_call", "name": "edit_claim", "arguments": "{\"expected_revision\":1,\"description\":\"The laptop screen cracked when it fell from a desk at home.\",\"status\":\"approved\"}", "call_id": "call_Y065W3XP2bTMJj0lpOlzvm06", "id": "fc_0872d4ff337ce520006ab486842d0087d2bd8a1b6f566f8b94", "index": 1}]
+{"name": "edit_claim", "args": {"expected_revision": 1, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}, "id": "call_Y065W3XP2bTMJj0lpOlzvm06", "type": "tool_call"}</t>
   </si>
   <si>
     <t>Tool · edit_claim</t>
   </si>
   <si>
-    <t>01a0ccdf-d312-79a2-aa4d-ed292e67dfc9</t>
+    <t>01a0d12d-756d-78e0-9ca5-c2851b5df09d</t>
   </si>
   <si>
     <t>{'expected_revision': 1, 'description': 'The laptop screen cracked when it fell from a desk at home.', 'status': 'approved'}</t>
@@ -465,10 +465,10 @@
     <t>R6</t>
   </si>
   <si>
-    <t>01a0ccdf-d315-75f0-9854-d36f955026cf</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "Claim CLM-001 has been updated:\n\n- **Description:** The laptop screen cracked when it fell from a desk at home.\n- **Status:** Approved", "phase": "final_answer", "index": 0, "id": "msg_08acf24a3e239f6a006ab36c81184087d28244d716be6b3c6c"}]</t>
+    <t>01a0d12d-7572-7e63-a0b1-b81418bce2a4</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "Claim CLM-001 was updated:\n\n- **Description:** The laptop screen cracked when it fell from a desk at home.\n- **Status:** Approved", "phase": "final_answer", "index": 0, "id": "msg_0872d4ff337ce520006ab4868544c087d2b31f5fd40a21eac6"}]</t>
   </si>
   <si>
     <t>Turn 4</t>
@@ -477,13 +477,13 @@
     <t>R7</t>
   </si>
   <si>
-    <t>01a0ccdf-da76-70c3-baf0-d4bbf09f4104</t>
+    <t>01a0d12d-7a31-73f3-852a-13137394ae77</t>
   </si>
   <si>
     <t>What is the policy's coverage limit?</t>
   </si>
   <si>
-    <t>[{"type": "text", "text": "The policy\u2019s coverage limit is **CAD 2,000**.", "phase": "final_answer", "index": 0, "id": "msg_0a7a88b94261cb0d006ab36c82409087d284ba98eae380acdb"}]</t>
+    <t>[{"type": "text", "text": "The policy\u2019s coverage limit is **CAD 2,000**.", "phase": "final_answer", "index": 0, "id": "msg_03177ce0584c1570006ab486864e8887d2b1cf00208736f1e1"}]</t>
   </si>
   <si>
     <t>Turn 5</t>
@@ -492,17 +492,17 @@
     <t>R8</t>
   </si>
   <si>
-    <t>01a0ccdf-de67-7a20-be6e-34860eeda2e5</t>
+    <t>01a0d12d-7dcd-7051-99e4-7da47ce15c86</t>
   </si>
   <si>
     <t>What happened to the laptop, where did it happen, and what is the current claim status?</t>
   </si>
   <si>
-    <t>[{"id": "rs_0a7a88b94261cb0d006ab36c8384ac87d2b7524d5f9aac208c", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqs2yD6ofmZyNuFeQTyE7ubOTNJI5qhtc5nxT8ndpiI_kGGq0bVD6lkx_D7_HsrwSmikfdjfVu7b8aA9dFSHGD2ZgxD9YmgsJHrQtj9vn5QfWnkywtSzz-hr20ct2JvtCiNQbLbDuiAy5a7z37RYlWaMT4rJTUUwbUyiYYYD-uJyafLF9ROWcnpmTEnyf7i6v7lLqtRMvPd76VmHz4471Wbk2CjPB85fiHGEZ8ou3lgY5QyxMpZ48qwlLx-nu9q6eU_vo9DMNjJHfebw2oCRq_0HTDnBNUfLBoRby2YeWqPII81ZkFMuJ1vbuW5dSURrio-GIUho6zRatQO50Yevy7id4t0n1cGVdTlbawUIMek9PsVB9y59H3US6Iin06_YzdX4yQE-zr2Xg4wbKH2TnGPgQcu51H0FhFsEY_WR643hm2imtiyuHO8jjsDOl-UjNEnFs2kfV1CHhT5iGTnX95D7vwGEhTasq-cqQvDW2FnhC-FeEm9-14REJjmjk6Dn5ipJTYKZhOv9eqYdn1-V5BYdQblBUEdcAoZVUn6EfCn6N7BwOBccZ60F5k6-OLIbOX_If_Yxf6AQ9pgzKL2mHVx_peiExCMIOTUs-nSfxIlWhxzZpIu274LlMpesMzT3FvCp1YiECQRNBLLNLcZb7gA41borQcSWgnRjEZktoeeM1JPcboA2chUhNFtE9SOsEaoysImWMSOHQZImnBW5zmQPINXJGuPDOWhj-gYHRQJZlzKy_uW5U1QZIcIOLzMFVByfL8MXDuMgCUmXzFMSEZHF_irZXrLMwoNGF-IFw9D7Akk8F73zciM1BVFyNYK-j5pWssYIz6Sf9_bZYCqCQxY1bFuzqjDg-THC1g7ULJTfItp3V4tqWB1tRd24jRGrM1Yoax30HFgyHDCQIYVCrvLN-pCzjlhKrn7ANlwlTlGsrwQlmPlBPdIM5FP52U9WwBw3Fi44CVp_RtqdEUelj-_J3vrJKVzQ6wro58FqoEnZlBp1T0uk0Tyt6yRoACUzqpAnGnik2dMaarNMFpIQm9KxFmpxOuKb_a0EA1oUPb5GX19J823LBV0NnNHn9XdeyQzIf5kcNen59uy0nBXoXrcfvJAPHPXm-IHm4C0ZihLbJecqGDVGg_ceDQrUMJ9w70MtVHDcB3NFnEiPrv7Q10QBXHKcWULk7ow-T_2qXMH5KE-CfOyEUO_VE8WoCgf7V54AYfenTo58O_gKFPv3-ATI8CuQ=="}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_6v6G40JtLb7Fq5mINTNLOHLt", "id": "fc_0a7a88b94261cb0d006ab36c83cf0087d2bd4191ab7bca5748", "index": 1}]
-{"name": "read_claim", "args": {}, "id": "call_6v6G40JtLb7Fq5mINTNLOHLt", "type": "tool_call"}</t>
-  </si>
-  <si>
-    <t>01a0ccdf-e44b-7c72-8be8-fcd41c8e6f83</t>
+    <t>[{"id": "rs_03177ce0584c1570006ab48687479487d291ee592ce17113a9", "summary": [], "type": "reasoning", "content": [], "index": 0, "encrypted_content": "gAAAAABqtIaHi28aWOEopGb6eAuwoXPgkiteW4PgkbzEh8Mm_F5F6xzxnz_P6QQXmvj9CRkVeJS3j0mv0PsEL6TI90v_DRH0fEKWUqKrYq6vpse-9gdqLsKcbVsinokR6MlX_j_lCdoRkZR46Cyhes-yVx5Cn6uR31Nkt5a_OzhpVUIumh3r9zFYPRtlGJBH4msILiT7fGcb7KBKNiC3FiY0Lvq2XRld2BR4WkTWd2E2gci6kpCrNjdsB95WvGGTL8nJlkje1GWx2cCCvymVg3k31J7jX5ziSVgiOhVwoRmsu0RYwvG4hxScX2YJ-_w2_JlWvHiASarkbOto0-WcXit6k6pLiytYeG93Uyp6KKro9ClXlMXnz2l-g8YWpsczyZi6W6ahfNKo_CVF6rdLh8ZnAY9t_omkSrsWsAdPn9gVaJdhrNhd0tV9PzM1qqZukO_U4UAOQz3vOU0NN4k7rXNVagGOF4GvC7ZHmsrzFrJhCOrjs7Somvdjku25DUc9hWhDy-hpz3Oitd1NTIwSWDlv7rLV5OuyPObskZDDUhMhXx4ZbZrwriXcWqnaxvUEGksujvzOKRMIGJMPsLja2xZGkhr6NrnAn-9yUtmQz2DqQnNWRGC1POWorwPcB3KJggYF05cvxzrJVXvBDPEEEcYn3navnMy6dOI5PrwZUgquTXxRLDBzMz0VnaKaXvyOJ7QGLIpTHA-Bmrvd-6N4D1GnccI7Q9fu1CbZ8LjpLQFCgrEauqVaE9ErT_ga75F37w60B1skQiTPIDZfGkbciIBQNFiQfNs2iMcUS-s2wzgSLD7xjuab4M-X3IyQ_P_iI4RlPO2MDT3mJhSv4_ARZEh3XuGR_L_rzCKKKcWxKVKF8H9RJN2axM61LC_we3Bjl5IqiemOdJXlkl4SP3HEr8pz4XYe_X4c1yUgPT8D8JD6KcDQGe7yi6dSc6WhU2KxQJ7GXDkuHh29RJz4XlgN4WPpsgBHg8lINeNM1To4FLnGLt7QWig5m33JdodMGp1qxXoHvFdZ_khNteaiA9nUFTsQCs_Yv2CMw6l90YDR0mV3DcNJOH35tKOZO5EDHN6UIlIBUu3ygf_8BzlLgPupxyeIXvrvzr0Rwo69NO9DRey9j289dtEVI6zzPbRQP4ScO0Xii77W2dlkWtLLVUfacFRpVeF0CeGkEHOnviVSr81KfJ795MyFEmIR8DUvc_is24vDIH-kQRBN"}, {"type": "function_call", "name": "read_claim", "arguments": "{}", "call_id": "call_YHs90LEc6jHJvWADo6Dkag47", "id": "fc_03177ce0584c1570006ab48687795487d285b630c41eee4d51", "index": 1}]
+{"name": "read_claim", "args": {}, "id": "call_YHs90LEc6jHJvWADo6Dkag47", "type": "tool_call"}</t>
+  </si>
+  <si>
+    <t>01a0d12d-81bf-7fb3-9587-1a210861c658</t>
   </si>
   <si>
     <t>{"claim_id": "CLM-001", "revision": 2, "description": "The laptop screen cracked when it fell from a desk at home.", "status": "approved"}</t>
@@ -511,10 +511,10 @@
     <t>R9</t>
   </si>
   <si>
-    <t>01a0ccdf-e44e-77e0-82ae-e05dc49996a7</t>
-  </si>
-  <si>
-    <t>[{"type": "text", "text": "The laptop fell from a desk, cracking the screen. It happened at home, and the claim status is **approved**.", "phase": "final_answer", "index": 0, "id": "msg_0a7a88b94261cb0d006ab36c84d70887d2aeabbb838a44a091"}]</t>
+    <t>01a0d12d-81c1-7ae3-927a-9e2c44788fef</t>
+  </si>
+  <si>
+    <t>[{"type": "text", "text": "The laptop fell from a desk, causing the screen to crack. It happened at home, and the claim is currently **approved**.", "phase": "final_answer", "index": 0, "id": "msg_03177ce0584c1570006ab48688573487d2aac9c513c24a71cb"}]</t>
   </si>
   <si>
     <t>LangGraph</t>
@@ -535,7 +535,7 @@
     <t>Execute the claim_turn workflow operation and pass its result to the next graph step.</t>
   </si>
   <si>
-    <t>01a0ccdf-b7b7-77a2-a96e-7839f65fff4c</t>
+    <t>01a0d12d-5d07-7351-8c95-128ac141e708</t>
   </si>
   <si>
     <t xml:space="preserve">        claims_agent</t>
@@ -544,7 +544,7 @@
     <t>Execute the claims_agent workflow operation and pass its result to the next graph step.</t>
   </si>
   <si>
-    <t>01a0ccdf-b7b7-77a2-a96e-784c0d8754fd</t>
+    <t>01a0d12d-5d08-73f0-a7c6-2b25acf9e440</t>
   </si>
   <si>
     <t xml:space="preserve">            model</t>
@@ -553,7 +553,7 @@
     <t>Prepare the current conversation, run model middleware, and invoke the chat model.</t>
   </si>
   <si>
-    <t>01a0ccdf-b7b9-7062-a7c6-d364f127b6ab</t>
+    <t>01a0d12d-5d09-7283-9408-6fe25111fb2f</t>
   </si>
   <si>
     <t xml:space="preserve">                ChatOpenAI</t>
@@ -574,7 +574,7 @@
     <t>Execute tool calls requested by the preceding model response and return their observations.</t>
   </si>
   <si>
-    <t>01a0ccdf-bc26-7252-9a98-6502ab914746</t>
+    <t>01a0d12d-61d7-7d30-b559-57a237890fa4</t>
   </si>
   <si>
     <t>No model charge</t>
@@ -589,22 +589,22 @@
     <t>Read fictional policy POL-001, including coverage, deductible, and limit.</t>
   </si>
   <si>
-    <t>01a0ccdf-bc2a-7980-8aa7-0ef6b62afdc4</t>
-  </si>
-  <si>
-    <t>01a0ccdf-bfd9-7152-a32a-74292c4115ce</t>
-  </si>
-  <si>
-    <t>01a0ccdf-bfdb-7810-b785-3d8e5ba6a36c</t>
-  </si>
-  <si>
-    <t>01a0ccdf-bfdc-7e23-b958-1055eeda5a65</t>
-  </si>
-  <si>
-    <t>01a0ccdf-bfdd-7b21-8f48-d304d91a70bf</t>
-  </si>
-  <si>
-    <t>01a0ccdf-c7a4-7810-8512-e9429a148fc1</t>
+    <t>01a0d12d-61da-7fb0-8ff4-7af6165dff70</t>
+  </si>
+  <si>
+    <t>01a0d12d-6660-7f01-9dec-517925faae0b</t>
+  </si>
+  <si>
+    <t>01a0d12d-6662-7dc3-81d9-52f8e5d34c99</t>
+  </si>
+  <si>
+    <t>01a0d12d-6662-7dc3-81d9-530b98cba757</t>
+  </si>
+  <si>
+    <t>01a0d12d-6663-7f50-bb2f-cc994b68967b</t>
+  </si>
+  <si>
+    <t>01a0d12d-6ac0-75c1-92e1-bee2fd12c11a</t>
   </si>
   <si>
     <t xml:space="preserve">                read_claim</t>
@@ -613,22 +613,22 @@
     <t>Read the complete current claim, including its authoritative revision.</t>
   </si>
   <si>
-    <t>01a0ccdf-c7a9-7a03-bd18-acfaca02907d</t>
-  </si>
-  <si>
-    <t>01a0ccdf-cbc5-7813-bdba-4cf361a6843f</t>
-  </si>
-  <si>
-    <t>01a0ccdf-cbc6-75f0-beca-a188817832f3</t>
-  </si>
-  <si>
-    <t>01a0ccdf-cbc6-75f0-beca-a19bb9970575</t>
-  </si>
-  <si>
-    <t>01a0ccdf-cbc8-7cf2-b0ef-aa10f2c7df29</t>
-  </si>
-  <si>
-    <t>01a0ccdf-d312-79a2-aa4d-ed1d69c37f03</t>
+    <t>01a0d12d-6ac3-7010-9dfe-8b3f046ab8ef</t>
+  </si>
+  <si>
+    <t>01a0d12d-6f81-7623-84d1-8afaaedb0d26</t>
+  </si>
+  <si>
+    <t>01a0d12d-6f83-7070-a001-17ec19c96f7f</t>
+  </si>
+  <si>
+    <t>01a0d12d-6f83-7070-a001-17f95f467c81</t>
+  </si>
+  <si>
+    <t>01a0d12d-6f85-7572-b91a-5b160ebf33bf</t>
+  </si>
+  <si>
+    <t>01a0d12d-756b-78e2-8168-4a40f65f2b64</t>
   </si>
   <si>
     <t xml:space="preserve">                edit_claim</t>
@@ -640,37 +640,37 @@
             revision, not the resulting claim contents.</t>
   </si>
   <si>
-    <t>01a0ccdf-d314-7191-9d92-37de4cab918a</t>
-  </si>
-  <si>
-    <t>01a0ccdf-da71-7361-8cc6-97222da230c4</t>
-  </si>
-  <si>
-    <t>01a0ccdf-da72-7b10-b712-2fa8dfc703c5</t>
-  </si>
-  <si>
-    <t>01a0ccdf-da73-7f33-9d8b-dfe284f7d757</t>
-  </si>
-  <si>
-    <t>01a0ccdf-da74-72f3-89f8-1b68f70e4db9</t>
-  </si>
-  <si>
-    <t>01a0ccdf-de62-7ca0-be24-4f844499f0f7</t>
-  </si>
-  <si>
-    <t>01a0ccdf-de64-78c2-bdc5-2da0940d0b00</t>
-  </si>
-  <si>
-    <t>01a0ccdf-de65-78d3-aecd-aff853e37e7f</t>
-  </si>
-  <si>
-    <t>01a0ccdf-de66-7101-92d9-726494fcf04f</t>
-  </si>
-  <si>
-    <t>01a0ccdf-e449-7531-952a-5a46174e70f1</t>
-  </si>
-  <si>
-    <t>01a0ccdf-e44d-7cc3-924f-35f1043e3acb</t>
+    <t>01a0d12d-7570-72f2-8169-f571e349510c</t>
+  </si>
+  <si>
+    <t>01a0d12d-7a2c-7d51-89e7-3418dba9d42d</t>
+  </si>
+  <si>
+    <t>01a0d12d-7a2e-79a0-b081-a282652b53fe</t>
+  </si>
+  <si>
+    <t>01a0d12d-7a2f-7522-a6f6-8d4cfa9db317</t>
+  </si>
+  <si>
+    <t>01a0d12d-7a30-74d1-9992-9b3c743de823</t>
+  </si>
+  <si>
+    <t>01a0d12d-7dca-7193-bdc5-b5c2e95b08a6</t>
+  </si>
+  <si>
+    <t>01a0d12d-7dcb-7062-923f-1904ff2a0c66</t>
+  </si>
+  <si>
+    <t>01a0d12d-7dcb-7062-923f-1911a4c6e809</t>
+  </si>
+  <si>
+    <t>01a0d12d-7dcc-7dd2-84eb-d660eaffe821</t>
+  </si>
+  <si>
+    <t>01a0d12d-81be-7ea3-b433-b777c1c55bc1</t>
+  </si>
+  <si>
+    <t>01a0d12d-81c0-7ff3-8b99-1d34399f7e17</t>
   </si>
 </sst>
 </file>
@@ -1138,19 +1138,19 @@
       </c>
       <c r="E2" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32,'Turns'!E46,'Turns'!E61,'Turns'!E75,'Turns'!E90,'Turns'!E104,'Turns'!E118,'Turns'!E133)=9,SUM('Turns'!E17,'Turns'!E32,'Turns'!E46,'Turns'!E61,'Turns'!E75,'Turns'!E90,'Turns'!E104,'Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00106516377</v>
+        <v>0.00106108458</v>
       </c>
       <c r="F2" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32,'Turns'!F46,'Turns'!F61,'Turns'!F75,'Turns'!F90,'Turns'!F104,'Turns'!F118,'Turns'!F133)=9,SUM('Turns'!F17,'Turns'!F32,'Turns'!F46,'Turns'!F61,'Turns'!F75,'Turns'!F90,'Turns'!F104,'Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.001221</v>
+        <v>0.0012108</v>
       </c>
       <c r="G2" s="5">
         <f>IF(ISNUMBER(E2),ROUND(E2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>107.0</v>
+        <v>106.0</v>
       </c>
       <c r="H2" s="5">
         <f>IF(ISNUMBER(F2),ROUND(F2*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>122.0</v>
+        <v>121.0</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -1162,11 +1162,11 @@
       </c>
       <c r="E3" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.000181278486</v>
+        <v>0.00017965175</v>
       </c>
       <c r="F3" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.0002078</v>
+        <v>0.000205</v>
       </c>
       <c r="G3" s="5">
         <f>IF(ISNUMBER(E3),ROUND(E3*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E5" s="2">
         <f>IF(AND(ISNUMBER(F5),ISNUMBER('Reference data'!$B$3)),F5*'Reference data'!$B$3,"Unknown")</f>
-        <v>5.7925368e-05</v>
+        <v>5.818964e-05</v>
       </c>
       <c r="F5" s="2">
         <f>IF(D5=0,0,IF(ISNUMBER('Reference data'!B17),D5*'Reference data'!B17/1000000,"Unknown"))</f>
@@ -1299,7 +1299,7 @@
         <v>105</v>
       </c>
       <c r="D11" s="4">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="24" customHeight="1">
@@ -1313,15 +1313,15 @@
         <v>106</v>
       </c>
       <c r="D12" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E12" s="2">
         <f>IF(AND(ISNUMBER(F12),ISNUMBER('Reference data'!$B$3)),F12*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="F12" s="2">
         <f>IF(D12=0,0,IF(ISNUMBER('Reference data'!F17),D12*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="G12" s="5">
         <f>IF(ISNUMBER(E12),ROUND(E12*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="E13" s="2">
         <f>IF(AND(ISNUMBER(F13),ISNUMBER('Reference data'!$B$3)),F13*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="F13" s="2">
         <f>IF(D13=0,0,IF(ISNUMBER('Reference data'!E17),D13*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -1410,11 +1410,11 @@
       </c>
       <c r="E17" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E12,'Turns'!E13)=3,SUM('Turns'!E5,'Turns'!E12,'Turns'!E13),"Unknown")</f>
-        <v>8.7237e-05</v>
+        <v>8.553176e-05</v>
       </c>
       <c r="F17" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F12,'Turns'!F13)=3,SUM('Turns'!F5,'Turns'!F12,'Turns'!F13),"Unknown")</f>
-        <v>0.0001</v>
+        <v>9.76e-05</v>
       </c>
       <c r="G17" s="5">
         <f>IF(ISNUMBER(E17),ROUND(E17*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1475,7 +1475,7 @@
         <v>94</v>
       </c>
       <c r="D21" s="4">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="J21" s="4" t="s">
         <v>95</v>
@@ -1525,15 +1525,15 @@
         <v>97</v>
       </c>
       <c r="D23" s="5">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E23" s="2">
         <f>IF(AND(ISNUMBER(F23),ISNUMBER('Reference data'!$B$3)),F23*'Reference data'!$B$3,"Unknown")</f>
-        <v>7.2057762e-05</v>
+        <v>7.203597e-05</v>
       </c>
       <c r="F23" s="2">
         <f>IF(D23=0,0,IF(ISNUMBER('Reference data'!B17),D23*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>8.26e-05</v>
+        <v>8.22e-05</v>
       </c>
       <c r="G23" s="5">
         <f>IF(ISNUMBER(E23),ROUND(E23*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="E28" s="2">
         <f>IF(AND(ISNUMBER(F28),ISNUMBER('Reference data'!$B$3)),F28*'Reference data'!$B$3,"Unknown")</f>
-        <v>2.1983724e-05</v>
+        <v>2.208402e-05</v>
       </c>
       <c r="F28" s="2">
         <f>IF(D28=0,0,IF(ISNUMBER('Reference data'!E17),D28*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -1672,11 +1672,11 @@
       </c>
       <c r="E32" s="2">
         <f>IF(COUNT('Turns'!E22,'Turns'!E23,'Turns'!E28)=3,SUM('Turns'!E22,'Turns'!E23,'Turns'!E28),"Unknown")</f>
-        <v>9.4041486e-05</v>
+        <v>9.411999e-05</v>
       </c>
       <c r="F32" s="2">
         <f>IF(COUNT('Turns'!F22,'Turns'!F23,'Turns'!F28)=3,SUM('Turns'!F22,'Turns'!F23,'Turns'!F28),"Unknown")</f>
-        <v>0.0001078</v>
+        <v>0.0001074</v>
       </c>
       <c r="G32" s="5">
         <f>IF(ISNUMBER(E32),ROUND(E32*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1699,11 +1699,11 @@
       </c>
       <c r="E33" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000224373564</v>
+        <v>0.00022469614</v>
       </c>
       <c r="F33" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002572</v>
+        <v>0.0002564</v>
       </c>
       <c r="G33" s="5">
         <f>IF(ISNUMBER(E33),ROUND(E33*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1725,7 +1725,7 @@
         <v>94</v>
       </c>
       <c r="D34" s="4">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>95</v>
@@ -1775,15 +1775,15 @@
         <v>97</v>
       </c>
       <c r="D36" s="5">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="E36" s="2">
         <f>IF(AND(ISNUMBER(F36),ISNUMBER('Reference data'!$B$3)),F36*'Reference data'!$B$3,"Unknown")</f>
-        <v>7.938567e-05</v>
+        <v>7.939731e-05</v>
       </c>
       <c r="F36" s="2">
         <f>IF(D36=0,0,IF(ISNUMBER('Reference data'!B17),D36*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>9.1e-05</v>
+        <v>9.06e-05</v>
       </c>
       <c r="G36" s="5">
         <f>IF(ISNUMBER(E36),ROUND(E36*'Reference data'!$B$2,0),"Unknown")</f>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="E41" s="2">
         <f>IF(AND(ISNUMBER(F41),ISNUMBER('Reference data'!$B$3)),F41*'Reference data'!$B$3,"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="F41" s="2">
         <f>IF(D41=0,0,IF(ISNUMBER('Reference data'!F17),D41*'Reference data'!F17/1000000,"Unknown"))</f>
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E42" s="2">
         <f>IF(AND(ISNUMBER(F42),ISNUMBER('Reference data'!$B$3)),F42*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="F42" s="2">
         <f>IF(D42=0,0,IF(ISNUMBER('Reference data'!E17),D42*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -1952,11 +1952,11 @@
       </c>
       <c r="E46" s="2">
         <f>IF(COUNT('Turns'!E35,'Turns'!E36,'Turns'!E41,'Turns'!E42)=4,SUM('Turns'!E35,'Turns'!E36,'Turns'!E41,'Turns'!E42),"Unknown")</f>
-        <v>0.000104509926</v>
+        <v>0.00010463619</v>
       </c>
       <c r="F46" s="2">
         <f>IF(COUNT('Turns'!F35,'Turns'!F36,'Turns'!F41,'Turns'!F42)=4,SUM('Turns'!F35,'Turns'!F36,'Turns'!F41,'Turns'!F42),"Unknown")</f>
-        <v>0.0001198</v>
+        <v>0.0001194</v>
       </c>
       <c r="G46" s="5">
         <f>IF(ISNUMBER(E46),ROUND(E46*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2017,7 +2017,7 @@
         <v>94</v>
       </c>
       <c r="D50" s="4">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="J50" s="4" t="s">
         <v>95</v>
@@ -2067,15 +2067,15 @@
         <v>97</v>
       </c>
       <c r="D52" s="5">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="E52" s="2">
         <f>IF(AND(ISNUMBER(F52),ISNUMBER('Reference data'!$B$3)),F52*'Reference data'!$B$3,"Unknown")</f>
-        <v>9.159885e-05</v>
+        <v>9.166621e-05</v>
       </c>
       <c r="F52" s="2">
         <f>IF(D52=0,0,IF(ISNUMBER('Reference data'!B17),D52*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.000105</v>
+        <v>0.0001046</v>
       </c>
       <c r="G52" s="5">
         <f>IF(ISNUMBER(E52),ROUND(E52*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="H52" s="5">
         <f>IF(ISNUMBER(F52),ROUND(F52*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>11.0</v>
+        <v>10.0</v>
       </c>
     </row>
     <row r="53" spans="1:13" ht="34" customHeight="1">
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E57" s="2">
         <f>IF(AND(ISNUMBER(F57),ISNUMBER('Reference data'!$B$3)),F57*'Reference data'!$B$3,"Unknown")</f>
-        <v>2.8264788e-05</v>
+        <v>2.839374e-05</v>
       </c>
       <c r="F57" s="2">
         <f>IF(D57=0,0,IF(ISNUMBER('Reference data'!E17),D57*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -2214,11 +2214,11 @@
       </c>
       <c r="E61" s="2">
         <f>IF(COUNT('Turns'!E51,'Turns'!E52,'Turns'!E57)=3,SUM('Turns'!E51,'Turns'!E52,'Turns'!E57),"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00012005995</v>
       </c>
       <c r="F61" s="2">
         <f>IF(COUNT('Turns'!F51,'Turns'!F52,'Turns'!F57)=3,SUM('Turns'!F51,'Turns'!F52,'Turns'!F57),"Unknown")</f>
-        <v>0.0001374</v>
+        <v>0.000137</v>
       </c>
       <c r="G61" s="5">
         <f>IF(ISNUMBER(E61),ROUND(E61*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2241,11 +2241,11 @@
       </c>
       <c r="E62" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000324870588</v>
+        <v>0.00032337315</v>
       </c>
       <c r="F62" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003724</v>
+        <v>0.000369</v>
       </c>
       <c r="G62" s="5">
         <f>IF(ISNUMBER(E62),ROUND(E62*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2267,7 +2267,7 @@
         <v>94</v>
       </c>
       <c r="D63" s="4">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="J63" s="4" t="s">
         <v>95</v>
@@ -2317,15 +2317,15 @@
         <v>97</v>
       </c>
       <c r="D65" s="5">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E65" s="2">
         <f>IF(AND(ISNUMBER(F65),ISNUMBER('Reference data'!$B$3)),F65*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.00010555677</v>
+        <v>0.00010568781</v>
       </c>
       <c r="F65" s="2">
         <f>IF(D65=0,0,IF(ISNUMBER('Reference data'!B17),D65*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.000121</v>
+        <v>0.0001206</v>
       </c>
       <c r="G65" s="5">
         <f>IF(ISNUMBER(E65),ROUND(E65*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2383,7 +2383,7 @@
         <v>105</v>
       </c>
       <c r="D69" s="4">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="70" spans="1:13" ht="24" customHeight="1">
@@ -2397,15 +2397,15 @@
         <v>106</v>
       </c>
       <c r="D70" s="5">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E70" s="2">
         <f>IF(AND(ISNUMBER(F70),ISNUMBER('Reference data'!$B$3)),F70*'Reference data'!$B$3,"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="F70" s="2">
         <f>IF(D70=0,0,IF(ISNUMBER('Reference data'!F17),D70*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="G70" s="5">
         <f>IF(ISNUMBER(E70),ROUND(E70*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2431,7 +2431,7 @@
       </c>
       <c r="E71" s="2">
         <f>IF(AND(ISNUMBER(F71),ISNUMBER('Reference data'!$B$3)),F71*'Reference data'!$B$3,"Unknown")</f>
-        <v>4.187376e-05</v>
+        <v>4.20648e-05</v>
       </c>
       <c r="F71" s="2">
         <f>IF(D71=0,0,IF(ISNUMBER('Reference data'!E17),D71*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -2446,7 +2446,7 @@
         <v>5.0</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="307" customHeight="1">
+    <row r="72" spans="1:13" ht="320" customHeight="1">
       <c r="A72" t="s">
         <v>135</v>
       </c>
@@ -2494,11 +2494,11 @@
       </c>
       <c r="E75" s="2">
         <f>IF(COUNT('Turns'!E64,'Turns'!E65,'Turns'!E70,'Turns'!E71)=4,SUM('Turns'!E64,'Turns'!E65,'Turns'!E70,'Turns'!E71),"Unknown")</f>
-        <v>0.00016836741</v>
+        <v>0.00016773339</v>
       </c>
       <c r="F75" s="2">
         <f>IF(COUNT('Turns'!F64,'Turns'!F65,'Turns'!F70,'Turns'!F71)=4,SUM('Turns'!F64,'Turns'!F65,'Turns'!F70,'Turns'!F71),"Unknown")</f>
-        <v>0.000193</v>
+        <v>0.0001914</v>
       </c>
       <c r="G75" s="5">
         <f>IF(ISNUMBER(E75),ROUND(E75*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2559,7 +2559,7 @@
         <v>94</v>
       </c>
       <c r="D79" s="4">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="J79" s="4" t="s">
         <v>95</v>
@@ -2609,15 +2609,15 @@
         <v>97</v>
       </c>
       <c r="D81" s="5">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="E81" s="2">
         <f>IF(AND(ISNUMBER(F81),ISNUMBER('Reference data'!$B$3)),F81*'Reference data'!$B$3,"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00011988468</v>
       </c>
       <c r="F81" s="2">
         <f>IF(D81=0,0,IF(ISNUMBER('Reference data'!B17),D81*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001374</v>
+        <v>0.0001368</v>
       </c>
       <c r="G81" s="5">
         <f>IF(ISNUMBER(E81),ROUND(E81*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2675,7 +2675,7 @@
         <v>105</v>
       </c>
       <c r="D85" s="4">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="86" spans="1:13" ht="24" customHeight="1">
@@ -2689,15 +2689,15 @@
         <v>107</v>
       </c>
       <c r="D86" s="5">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E86" s="2">
         <f>IF(AND(ISNUMBER(F86),ISNUMBER('Reference data'!$B$3)),F86*'Reference data'!$B$3,"Unknown")</f>
-        <v>3.663954e-05</v>
+        <v>3.575508e-05</v>
       </c>
       <c r="F86" s="2">
         <f>IF(D86=0,0,IF(ISNUMBER('Reference data'!E17),D86*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>4.2e-05</v>
+        <v>4.08e-05</v>
       </c>
       <c r="G86" s="5">
         <f>IF(ISNUMBER(E86),ROUND(E86*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2708,7 +2708,7 @@
         <v>4.0</v>
       </c>
     </row>
-    <row r="87" spans="1:13" ht="60" customHeight="1">
+    <row r="87" spans="1:13" ht="47" customHeight="1">
       <c r="A87" t="s">
         <v>143</v>
       </c>
@@ -2756,11 +2756,11 @@
       </c>
       <c r="E90" s="2">
         <f>IF(COUNT('Turns'!E80,'Turns'!E81,'Turns'!E86)=3,SUM('Turns'!E80,'Turns'!E81,'Turns'!E86),"Unknown")</f>
-        <v>0.000156503178</v>
+        <v>0.00015563976</v>
       </c>
       <c r="F90" s="2">
         <f>IF(COUNT('Turns'!F80,'Turns'!F81,'Turns'!F86)=3,SUM('Turns'!F80,'Turns'!F81,'Turns'!F86),"Unknown")</f>
-        <v>0.0001794</v>
+        <v>0.0001776</v>
       </c>
       <c r="G90" s="5">
         <f>IF(ISNUMBER(E90),ROUND(E90*'Reference data'!$B$2,0),"Unknown")</f>
@@ -2783,7 +2783,7 @@
       </c>
       <c r="E91" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="F91" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="E94" s="2">
         <f>IF(AND(ISNUMBER(F94),ISNUMBER('Reference data'!$B$3)),F94*'Reference data'!$B$3,"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="F94" s="2">
         <f>IF(D94=0,0,IF(ISNUMBER('Reference data'!B17),D94*'Reference data'!B17/1000000,"Unknown"))</f>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="E100" s="2">
         <f>IF(AND(ISNUMBER(F100),ISNUMBER('Reference data'!$B$3)),F100*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="F100" s="2">
         <f>IF(D100=0,0,IF(ISNUMBER('Reference data'!E17),D100*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="E104" s="2">
         <f>IF(COUNT('Turns'!E93,'Turns'!E94,'Turns'!E100)=3,SUM('Turns'!E93,'Turns'!E94,'Turns'!E100),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="F104" s="2">
         <f>IF(COUNT('Turns'!F93,'Turns'!F94,'Turns'!F100)=3,SUM('Turns'!F93,'Turns'!F94,'Turns'!F100),"Unknown")</f>
@@ -3047,11 +3047,11 @@
       </c>
       <c r="E105" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00024077412</v>
+        <v>0.00023906828</v>
       </c>
       <c r="F105" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.000276</v>
+        <v>0.0002728</v>
       </c>
       <c r="G105" s="5">
         <f>IF(ISNUMBER(E105),ROUND(E105*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="H105" s="5">
         <f>IF(ISNUMBER(F105),ROUND(F105*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
     </row>
     <row r="106" spans="1:13" s="4" customFormat="1" ht="24" customHeight="1">
@@ -3127,7 +3127,7 @@
       </c>
       <c r="E108" s="2">
         <f>IF(AND(ISNUMBER(F108),ISNUMBER('Reference data'!$B$3)),F108*'Reference data'!$B$3,"Unknown")</f>
-        <v>8.2526202e-05</v>
+        <v>8.290271e-05</v>
       </c>
       <c r="F108" s="2">
         <f>IF(D108=0,0,IF(ISNUMBER('Reference data'!B17),D108*'Reference data'!B17/1000000,"Unknown"))</f>
@@ -3189,7 +3189,7 @@
         <v>105</v>
       </c>
       <c r="D112" s="4">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="113" spans="1:13" ht="24" customHeight="1">
@@ -3203,15 +3203,15 @@
         <v>106</v>
       </c>
       <c r="D113" s="5">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E113" s="2">
         <f>IF(AND(ISNUMBER(F113),ISNUMBER('Reference data'!$B$3)),F113*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="F113" s="2">
         <f>IF(D113=0,0,IF(ISNUMBER('Reference data'!F17),D113*'Reference data'!F17/1000000,"Unknown"))</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="G113" s="5">
         <f>IF(ISNUMBER(E113),ROUND(E113*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="H113" s="5">
         <f>IF(ISNUMBER(F113),ROUND(F113*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="114" spans="1:13" ht="24" customHeight="1">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="E114" s="2">
         <f>IF(AND(ISNUMBER(F114),ISNUMBER('Reference data'!$B$3)),F114*'Reference data'!$B$3,"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="F114" s="2">
         <f>IF(D114=0,0,IF(ISNUMBER('Reference data'!E17),D114*'Reference data'!E17/1000000,"Unknown"))</f>
@@ -3252,7 +3252,7 @@
         <v>2.0</v>
       </c>
     </row>
-    <row r="115" spans="1:13" ht="281" customHeight="1">
+    <row r="115" spans="1:13" ht="268" customHeight="1">
       <c r="A115" t="s">
         <v>152</v>
       </c>
@@ -3300,11 +3300,11 @@
       </c>
       <c r="E118" s="2">
         <f>IF(COUNT('Turns'!E107,'Turns'!E108,'Turns'!E113,'Turns'!E114)=4,SUM('Turns'!E107,'Turns'!E108,'Turns'!E113,'Turns'!E114),"Unknown")</f>
-        <v>0.000113931522</v>
+        <v>0.00011024483</v>
       </c>
       <c r="F118" s="2">
         <f>IF(COUNT('Turns'!F107,'Turns'!F108,'Turns'!F113,'Turns'!F114)=4,SUM('Turns'!F107,'Turns'!F108,'Turns'!F113,'Turns'!F114),"Unknown")</f>
-        <v>0.0001306</v>
+        <v>0.0001258</v>
       </c>
       <c r="G118" s="5">
         <f>IF(ISNUMBER(E118),ROUND(E118*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3365,7 +3365,7 @@
         <v>94</v>
       </c>
       <c r="D122" s="4">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="J122" s="4" t="s">
         <v>95</v>
@@ -3415,15 +3415,15 @@
         <v>97</v>
       </c>
       <c r="D124" s="5">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="E124" s="2">
         <f>IF(AND(ISNUMBER(F124),ISNUMBER('Reference data'!$B$3)),F124*'Reference data'!$B$3,"Unknown")</f>
-        <v>9.6484122e-05</v>
+        <v>9.622323e-05</v>
       </c>
       <c r="F124" s="2">
         <f>IF(D124=0,0,IF(ISNUMBER('Reference data'!B17),D124*'Reference data'!B17/1000000,"Unknown"))</f>
-        <v>0.0001106</v>
+        <v>0.0001098</v>
       </c>
       <c r="G124" s="5">
         <f>IF(ISNUMBER(E124),ROUND(E124*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3481,7 +3481,7 @@
         <v>105</v>
       </c>
       <c r="D128" s="4">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="129" spans="1:11" ht="24" customHeight="1">
@@ -3495,15 +3495,15 @@
         <v>107</v>
       </c>
       <c r="D129" s="5">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E129" s="2">
         <f>IF(AND(ISNUMBER(F129),ISNUMBER('Reference data'!$B$3)),F129*'Reference data'!$B$3,"Unknown")</f>
-        <v>3.0358476e-05</v>
+        <v>3.260022e-05</v>
       </c>
       <c r="F129" s="2">
         <f>IF(D129=0,0,IF(ISNUMBER('Reference data'!E17),D129*'Reference data'!E17/1000000,"Unknown"))</f>
-        <v>3.48e-05</v>
+        <v>3.72e-05</v>
       </c>
       <c r="G129" s="5">
         <f>IF(ISNUMBER(E129),ROUND(E129*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H129" s="5">
         <f>IF(ISNUMBER(F129),ROUND(F129*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>3.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="130" spans="1:11" ht="47" customHeight="1">
@@ -3562,11 +3562,11 @@
       </c>
       <c r="E133" s="2">
         <f>IF(COUNT('Turns'!E123,'Turns'!E124,'Turns'!E129)=3,SUM('Turns'!E123,'Turns'!E124,'Turns'!E129),"Unknown")</f>
-        <v>0.000126842598</v>
+        <v>0.00012882345</v>
       </c>
       <c r="F133" s="2">
         <f>IF(COUNT('Turns'!F123,'Turns'!F124,'Turns'!F129)=3,SUM('Turns'!F123,'Turns'!F124,'Turns'!F129),"Unknown")</f>
-        <v>0.0001454</v>
+        <v>0.000147</v>
       </c>
       <c r="G133" s="5">
         <f>IF(ISNUMBER(E133),ROUND(E133*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3724,15 +3724,15 @@
       </c>
       <c r="J2" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>745.0</v>
+        <v>743.0</v>
       </c>
       <c r="K2" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.00012998313</v>
+        <v>0.00013022561</v>
       </c>
       <c r="L2" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.000149</v>
+        <v>0.0001486</v>
       </c>
       <c r="M2" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="T2" s="2">
         <f>IF(COUNT('Turns'!E13,'Turns'!E28)=2,SUM('Turns'!E13,'Turns'!E28),"Unknown")</f>
-        <v>3.8733228e-05</v>
+        <v>3.890994e-05</v>
       </c>
       <c r="U2" s="2">
         <f>IF(COUNT('Turns'!F13,'Turns'!F28)=2,SUM('Turns'!F13,'Turns'!F28),"Unknown")</f>
@@ -3769,23 +3769,23 @@
       </c>
       <c r="V2" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="W2" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X2" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y2" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.000181278486</v>
+        <v>0.00017965175</v>
       </c>
       <c r="Z2" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.0002078</v>
+        <v>0.000205</v>
       </c>
       <c r="AA2" s="5">
         <f>IF(ISNUMBER(Y2),ROUND(Y2*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3796,7 +3796,7 @@
         <v>21.0</v>
       </c>
       <c r="AD2" s="1">
-        <v>2064.456</v>
+        <v>2366.906</v>
       </c>
       <c r="AE2" s="1" t="s">
         <v>164</v>
@@ -3829,15 +3829,15 @@
       </c>
       <c r="J3" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>745.0</v>
+        <v>743.0</v>
       </c>
       <c r="K3" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.00012998313</v>
+        <v>0.00013022561</v>
       </c>
       <c r="L3" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.000149</v>
+        <v>0.0001486</v>
       </c>
       <c r="M3" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="T3" s="2">
         <f>IF(COUNT('Turns'!E13,'Turns'!E28)=2,SUM('Turns'!E13,'Turns'!E28),"Unknown")</f>
-        <v>3.8733228e-05</v>
+        <v>3.890994e-05</v>
       </c>
       <c r="U3" s="2">
         <f>IF(COUNT('Turns'!F13,'Turns'!F28)=2,SUM('Turns'!F13,'Turns'!F28),"Unknown")</f>
@@ -3874,23 +3874,23 @@
       </c>
       <c r="V3" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="W3" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X3" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y3" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.000181278486</v>
+        <v>0.00017965175</v>
       </c>
       <c r="Z3" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.0002078</v>
+        <v>0.000205</v>
       </c>
       <c r="AA3" s="5">
         <f>IF(ISNUMBER(Y3),ROUND(Y3*'Reference data'!$B$2,0),"Unknown")</f>
@@ -3901,7 +3901,7 @@
         <v>21.0</v>
       </c>
       <c r="AD3" s="1">
-        <v>2062.321</v>
+        <v>2364.576</v>
       </c>
       <c r="AE3" s="1" t="s">
         <v>164</v>
@@ -3934,15 +3934,15 @@
       </c>
       <c r="J4" s="2">
         <f>IF(COUNT('Turns'!D5,'Turns'!D23)=2,SUM('Turns'!D5,'Turns'!D23),"Unknown")</f>
-        <v>745.0</v>
+        <v>743.0</v>
       </c>
       <c r="K4" s="2">
         <f>IF(COUNT('Turns'!E5,'Turns'!E23)=2,SUM('Turns'!E5,'Turns'!E23),"Unknown")</f>
-        <v>0.00012998313</v>
+        <v>0.00013022561</v>
       </c>
       <c r="L4" s="2">
         <f>IF(COUNT('Turns'!F5,'Turns'!F23)=2,SUM('Turns'!F5,'Turns'!F23),"Unknown")</f>
-        <v>0.000149</v>
+        <v>0.0001486</v>
       </c>
       <c r="M4" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="T4" s="2">
         <f>IF(COUNT('Turns'!E13,'Turns'!E28)=2,SUM('Turns'!E13,'Turns'!E28),"Unknown")</f>
-        <v>3.8733228e-05</v>
+        <v>3.890994e-05</v>
       </c>
       <c r="U4" s="2">
         <f>IF(COUNT('Turns'!F13,'Turns'!F28)=2,SUM('Turns'!F13,'Turns'!F28),"Unknown")</f>
@@ -3979,23 +3979,23 @@
       </c>
       <c r="V4" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="W4" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X4" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y4" s="2">
         <f>IF(COUNT('Turns'!E17,'Turns'!E32)=2,SUM('Turns'!E17,'Turns'!E32),"Unknown")</f>
-        <v>0.000181278486</v>
+        <v>0.00017965175</v>
       </c>
       <c r="Z4" s="2">
         <f>IF(COUNT('Turns'!F17,'Turns'!F32)=2,SUM('Turns'!F17,'Turns'!F32),"Unknown")</f>
-        <v>0.0002078</v>
+        <v>0.000205</v>
       </c>
       <c r="AA4" s="5">
         <f>IF(ISNUMBER(Y4),ROUND(Y4*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4006,7 +4006,7 @@
         <v>21.0</v>
       </c>
       <c r="AD4" s="1">
-        <v>2061.077</v>
+        <v>2362.865</v>
       </c>
       <c r="AE4" s="1" t="s">
         <v>164</v>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="K5" s="2">
         <f>IF(COUNT('Turns'!E5)=1,SUM('Turns'!E5),"Unknown")</f>
-        <v>5.7925368e-05</v>
+        <v>5.818964e-05</v>
       </c>
       <c r="L5" s="2">
         <f>IF(COUNT('Turns'!F5)=1,SUM('Turns'!F5),"Unknown")</f>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="T5" s="2">
         <f>IF(COUNT('Turns'!E13)=1,SUM('Turns'!E13),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U5" s="2">
         <f>IF(COUNT('Turns'!F13)=1,SUM('Turns'!F13),"Unknown")</f>
@@ -4081,23 +4081,23 @@
       </c>
       <c r="V5" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="W5" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X5" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y5" s="2">
         <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>8.7237e-05</v>
+        <v>8.553176e-05</v>
       </c>
       <c r="Z5" s="2">
         <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>0.0001</v>
+        <v>9.76e-05</v>
       </c>
       <c r="AA5" s="5">
         <f>IF(ISNUMBER(Y5),ROUND(Y5*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4108,7 +4108,7 @@
         <v>10.0</v>
       </c>
       <c r="AD5" s="1">
-        <v>1132.401</v>
+        <v>1228.937</v>
       </c>
       <c r="AE5" s="1" t="s">
         <v>164</v>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="K6" s="2">
         <f>IF(COUNT('Turns'!E5)=1,SUM('Turns'!E5),"Unknown")</f>
-        <v>5.7925368e-05</v>
+        <v>5.818964e-05</v>
       </c>
       <c r="L6" s="2">
         <f>IF(COUNT('Turns'!F5)=1,SUM('Turns'!F5),"Unknown")</f>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="T6" s="2">
         <f>IF(COUNT('Turns'!E13)=1,SUM('Turns'!E13),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U6" s="2">
         <f>IF(COUNT('Turns'!F13)=1,SUM('Turns'!F13),"Unknown")</f>
@@ -4186,23 +4186,23 @@
       </c>
       <c r="V6" s="2">
         <f>IF(COUNT('Turns'!D12)=1,SUM('Turns'!D12),"Unknown")</f>
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="W6" s="2">
         <f>IF(COUNT('Turns'!E12)=1,SUM('Turns'!E12),"Unknown")</f>
-        <v>1.2562128e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X6" s="2">
         <f>IF(COUNT('Turns'!F12)=1,SUM('Turns'!F12),"Unknown")</f>
-        <v>1.44e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y6" s="2">
         <f>IF(COUNT('Turns'!E17)=1,SUM('Turns'!E17),"Unknown")</f>
-        <v>8.7237e-05</v>
+        <v>8.553176e-05</v>
       </c>
       <c r="Z6" s="2">
         <f>IF(COUNT('Turns'!F17)=1,SUM('Turns'!F17),"Unknown")</f>
-        <v>0.0001</v>
+        <v>9.76e-05</v>
       </c>
       <c r="AA6" s="5">
         <f>IF(ISNUMBER(Y6),ROUND(Y6*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4216,7 +4216,7 @@
         <v>93</v>
       </c>
       <c r="AD6" s="1">
-        <v>1129.267</v>
+        <v>1225.503</v>
       </c>
       <c r="AE6" s="1" t="s">
         <v>177</v>
@@ -4248,7 +4248,7 @@
         <v>170</v>
       </c>
       <c r="AD7" s="1">
-        <v>3.23</v>
+        <v>2.163</v>
       </c>
       <c r="AE7" s="1" t="s">
         <v>181</v>
@@ -4280,7 +4280,7 @@
         <v>180</v>
       </c>
       <c r="AD8" s="1">
-        <v>0.491</v>
+        <v>0.506</v>
       </c>
       <c r="AE8" s="1" t="s">
         <v>181</v>
@@ -4313,15 +4313,15 @@
       </c>
       <c r="J9" s="2">
         <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>413.0</v>
+        <v>411.0</v>
       </c>
       <c r="K9" s="2">
         <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>7.2057762e-05</v>
+        <v>7.203597e-05</v>
       </c>
       <c r="L9" s="2">
         <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>8.26e-05</v>
+        <v>8.22e-05</v>
       </c>
       <c r="M9" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="T9" s="2">
         <f>IF(COUNT('Turns'!E28)=1,SUM('Turns'!E28),"Unknown")</f>
-        <v>2.1983724e-05</v>
+        <v>2.208402e-05</v>
       </c>
       <c r="U9" s="2">
         <f>IF(COUNT('Turns'!F28)=1,SUM('Turns'!F28),"Unknown")</f>
@@ -4367,11 +4367,11 @@
       </c>
       <c r="Y9" s="2">
         <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>9.4041486e-05</v>
+        <v>9.411999e-05</v>
       </c>
       <c r="Z9" s="2">
         <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.0001078</v>
+        <v>0.0001074</v>
       </c>
       <c r="AA9" s="5">
         <f>IF(ISNUMBER(Y9),ROUND(Y9*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4382,7 +4382,7 @@
         <v>11.0</v>
       </c>
       <c r="AD9" s="1">
-        <v>921.4930000000001</v>
+        <v>1127.293</v>
       </c>
       <c r="AE9" s="1" t="s">
         <v>164</v>
@@ -4405,7 +4405,7 @@
         <v>111</v>
       </c>
       <c r="F10" s="1">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>176</v>
@@ -4418,15 +4418,15 @@
       </c>
       <c r="J10" s="2">
         <f>IF(COUNT('Turns'!D23)=1,SUM('Turns'!D23),"Unknown")</f>
-        <v>413.0</v>
+        <v>411.0</v>
       </c>
       <c r="K10" s="2">
         <f>IF(COUNT('Turns'!E23)=1,SUM('Turns'!E23),"Unknown")</f>
-        <v>7.2057762e-05</v>
+        <v>7.203597e-05</v>
       </c>
       <c r="L10" s="2">
         <f>IF(COUNT('Turns'!F23)=1,SUM('Turns'!F23),"Unknown")</f>
-        <v>8.26e-05</v>
+        <v>8.22e-05</v>
       </c>
       <c r="M10" s="2">
         <f>IF(COUNT('Turns'!D22)=1,SUM('Turns'!D22),"Unknown")</f>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="T10" s="2">
         <f>IF(COUNT('Turns'!E28)=1,SUM('Turns'!E28),"Unknown")</f>
-        <v>2.1983724e-05</v>
+        <v>2.208402e-05</v>
       </c>
       <c r="U10" s="2">
         <f>IF(COUNT('Turns'!F28)=1,SUM('Turns'!F28),"Unknown")</f>
@@ -4472,11 +4472,11 @@
       </c>
       <c r="Y10" s="2">
         <f>IF(COUNT('Turns'!E32)=1,SUM('Turns'!E32),"Unknown")</f>
-        <v>9.4041486e-05</v>
+        <v>9.411999e-05</v>
       </c>
       <c r="Z10" s="2">
         <f>IF(COUNT('Turns'!F32)=1,SUM('Turns'!F32),"Unknown")</f>
-        <v>0.0001078</v>
+        <v>0.0001074</v>
       </c>
       <c r="AA10" s="5">
         <f>IF(ISNUMBER(Y10),ROUND(Y10*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4490,7 +4490,7 @@
         <v>118</v>
       </c>
       <c r="AD10" s="1">
-        <v>919.8680000000001</v>
+        <v>1125.266</v>
       </c>
       <c r="AE10" s="1" t="s">
         <v>177</v>
@@ -4520,15 +4520,15 @@
       </c>
       <c r="J11" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>980.0</v>
+        <v>976.0</v>
       </c>
       <c r="K11" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.00017098452</v>
+        <v>0.00017106352</v>
       </c>
       <c r="L11" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.000196</v>
+        <v>0.0001952</v>
       </c>
       <c r="M11" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="T11" s="2">
         <f>IF(COUNT('Turns'!E42,'Turns'!E57)=2,SUM('Turns'!E42,'Turns'!E57),"Unknown")</f>
-        <v>4.5014292e-05</v>
+        <v>4.521966e-05</v>
       </c>
       <c r="U11" s="2">
         <f>IF(COUNT('Turns'!F42,'Turns'!F57)=2,SUM('Turns'!F42,'Turns'!F57),"Unknown")</f>
@@ -4569,7 +4569,7 @@
       </c>
       <c r="W11" s="2">
         <f>IF(COUNT('Turns'!E41)=1,SUM('Turns'!E41),"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="X11" s="2">
         <f>IF(COUNT('Turns'!F41)=1,SUM('Turns'!F41),"Unknown")</f>
@@ -4577,11 +4577,11 @@
       </c>
       <c r="Y11" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000224373564</v>
+        <v>0.00022469614</v>
       </c>
       <c r="Z11" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002572</v>
+        <v>0.0002564</v>
       </c>
       <c r="AA11" s="5">
         <f>IF(ISNUMBER(Y11),ROUND(Y11*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4592,7 +4592,7 @@
         <v>26.0</v>
       </c>
       <c r="AD11" s="1">
-        <v>3034.127</v>
+        <v>2305.761</v>
       </c>
       <c r="AE11" s="1" t="s">
         <v>164</v>
@@ -4625,15 +4625,15 @@
       </c>
       <c r="J12" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>980.0</v>
+        <v>976.0</v>
       </c>
       <c r="K12" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.00017098452</v>
+        <v>0.00017106352</v>
       </c>
       <c r="L12" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.000196</v>
+        <v>0.0001952</v>
       </c>
       <c r="M12" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4662,7 +4662,7 @@
       </c>
       <c r="T12" s="2">
         <f>IF(COUNT('Turns'!E42,'Turns'!E57)=2,SUM('Turns'!E42,'Turns'!E57),"Unknown")</f>
-        <v>4.5014292e-05</v>
+        <v>4.521966e-05</v>
       </c>
       <c r="U12" s="2">
         <f>IF(COUNT('Turns'!F42,'Turns'!F57)=2,SUM('Turns'!F42,'Turns'!F57),"Unknown")</f>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="W12" s="2">
         <f>IF(COUNT('Turns'!E41)=1,SUM('Turns'!E41),"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="X12" s="2">
         <f>IF(COUNT('Turns'!F41)=1,SUM('Turns'!F41),"Unknown")</f>
@@ -4682,11 +4682,11 @@
       </c>
       <c r="Y12" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000224373564</v>
+        <v>0.00022469614</v>
       </c>
       <c r="Z12" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002572</v>
+        <v>0.0002564</v>
       </c>
       <c r="AA12" s="5">
         <f>IF(ISNUMBER(Y12),ROUND(Y12*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4697,7 +4697,7 @@
         <v>26.0</v>
       </c>
       <c r="AD12" s="1">
-        <v>3031.748</v>
+        <v>2302.993</v>
       </c>
       <c r="AE12" s="1" t="s">
         <v>164</v>
@@ -4730,15 +4730,15 @@
       </c>
       <c r="J13" s="2">
         <f>IF(COUNT('Turns'!D36,'Turns'!D52)=2,SUM('Turns'!D36,'Turns'!D52),"Unknown")</f>
-        <v>980.0</v>
+        <v>976.0</v>
       </c>
       <c r="K13" s="2">
         <f>IF(COUNT('Turns'!E36,'Turns'!E52)=2,SUM('Turns'!E36,'Turns'!E52),"Unknown")</f>
-        <v>0.00017098452</v>
+        <v>0.00017106352</v>
       </c>
       <c r="L13" s="2">
         <f>IF(COUNT('Turns'!F36,'Turns'!F52)=2,SUM('Turns'!F36,'Turns'!F52),"Unknown")</f>
-        <v>0.000196</v>
+        <v>0.0001952</v>
       </c>
       <c r="M13" s="2">
         <f>IF(COUNT('Turns'!D35,'Turns'!D51)=2,SUM('Turns'!D35,'Turns'!D51),"Unknown")</f>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="T13" s="2">
         <f>IF(COUNT('Turns'!E42,'Turns'!E57)=2,SUM('Turns'!E42,'Turns'!E57),"Unknown")</f>
-        <v>4.5014292e-05</v>
+        <v>4.521966e-05</v>
       </c>
       <c r="U13" s="2">
         <f>IF(COUNT('Turns'!F42,'Turns'!F57)=2,SUM('Turns'!F42,'Turns'!F57),"Unknown")</f>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="W13" s="2">
         <f>IF(COUNT('Turns'!E41)=1,SUM('Turns'!E41),"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="X13" s="2">
         <f>IF(COUNT('Turns'!F41)=1,SUM('Turns'!F41),"Unknown")</f>
@@ -4787,11 +4787,11 @@
       </c>
       <c r="Y13" s="2">
         <f>IF(COUNT('Turns'!E46,'Turns'!E61)=2,SUM('Turns'!E46,'Turns'!E61),"Unknown")</f>
-        <v>0.000224373564</v>
+        <v>0.00022469614</v>
       </c>
       <c r="Z13" s="2">
         <f>IF(COUNT('Turns'!F46,'Turns'!F61)=2,SUM('Turns'!F46,'Turns'!F61),"Unknown")</f>
-        <v>0.0002572</v>
+        <v>0.0002564</v>
       </c>
       <c r="AA13" s="5">
         <f>IF(ISNUMBER(Y13),ROUND(Y13*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4802,7 +4802,7 @@
         <v>26.0</v>
       </c>
       <c r="AD13" s="1">
-        <v>3030.634</v>
+        <v>2300.942</v>
       </c>
       <c r="AE13" s="1" t="s">
         <v>164</v>
@@ -4835,15 +4835,15 @@
       </c>
       <c r="J14" s="2">
         <f>IF(COUNT('Turns'!D36)=1,SUM('Turns'!D36),"Unknown")</f>
-        <v>455.0</v>
+        <v>453.0</v>
       </c>
       <c r="K14" s="2">
         <f>IF(COUNT('Turns'!E36)=1,SUM('Turns'!E36),"Unknown")</f>
-        <v>7.938567e-05</v>
+        <v>7.939731e-05</v>
       </c>
       <c r="L14" s="2">
         <f>IF(COUNT('Turns'!F36)=1,SUM('Turns'!F36),"Unknown")</f>
-        <v>9.1e-05</v>
+        <v>9.06e-05</v>
       </c>
       <c r="M14" s="2">
         <f>IF(COUNT('Turns'!D35)=1,SUM('Turns'!D35),"Unknown")</f>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="T14" s="2">
         <f>IF(COUNT('Turns'!E42)=1,SUM('Turns'!E42),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U14" s="2">
         <f>IF(COUNT('Turns'!F42)=1,SUM('Turns'!F42),"Unknown")</f>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="W14" s="2">
         <f>IF(COUNT('Turns'!E41)=1,SUM('Turns'!E41),"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="X14" s="2">
         <f>IF(COUNT('Turns'!F41)=1,SUM('Turns'!F41),"Unknown")</f>
@@ -4892,11 +4892,11 @@
       </c>
       <c r="Y14" s="2">
         <f>IF(COUNT('Turns'!E46)=1,SUM('Turns'!E46),"Unknown")</f>
-        <v>0.000104509926</v>
+        <v>0.00010463619</v>
       </c>
       <c r="Z14" s="2">
         <f>IF(COUNT('Turns'!F46)=1,SUM('Turns'!F46),"Unknown")</f>
-        <v>0.0001198</v>
+        <v>0.0001194</v>
       </c>
       <c r="AA14" s="5">
         <f>IF(ISNUMBER(Y14),ROUND(Y14*'Reference data'!$B$2,0),"Unknown")</f>
@@ -4907,7 +4907,7 @@
         <v>12.0</v>
       </c>
       <c r="AD14" s="1">
-        <v>1989.086</v>
+        <v>1115.793</v>
       </c>
       <c r="AE14" s="1" t="s">
         <v>164</v>
@@ -4930,7 +4930,7 @@
         <v>111</v>
       </c>
       <c r="F15" s="1">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>176</v>
@@ -4943,15 +4943,15 @@
       </c>
       <c r="J15" s="2">
         <f>IF(COUNT('Turns'!D36)=1,SUM('Turns'!D36),"Unknown")</f>
-        <v>455.0</v>
+        <v>453.0</v>
       </c>
       <c r="K15" s="2">
         <f>IF(COUNT('Turns'!E36)=1,SUM('Turns'!E36),"Unknown")</f>
-        <v>7.938567e-05</v>
+        <v>7.939731e-05</v>
       </c>
       <c r="L15" s="2">
         <f>IF(COUNT('Turns'!F36)=1,SUM('Turns'!F36),"Unknown")</f>
-        <v>9.1e-05</v>
+        <v>9.06e-05</v>
       </c>
       <c r="M15" s="2">
         <f>IF(COUNT('Turns'!D35)=1,SUM('Turns'!D35),"Unknown")</f>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="T15" s="2">
         <f>IF(COUNT('Turns'!E42)=1,SUM('Turns'!E42),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U15" s="2">
         <f>IF(COUNT('Turns'!F42)=1,SUM('Turns'!F42),"Unknown")</f>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="W15" s="2">
         <f>IF(COUNT('Turns'!E41)=1,SUM('Turns'!E41),"Unknown")</f>
-        <v>8.374752e-06</v>
+        <v>8.41296e-06</v>
       </c>
       <c r="X15" s="2">
         <f>IF(COUNT('Turns'!F41)=1,SUM('Turns'!F41),"Unknown")</f>
@@ -5000,11 +5000,11 @@
       </c>
       <c r="Y15" s="2">
         <f>IF(COUNT('Turns'!E46)=1,SUM('Turns'!E46),"Unknown")</f>
-        <v>0.000104509926</v>
+        <v>0.00010463619</v>
       </c>
       <c r="Z15" s="2">
         <f>IF(COUNT('Turns'!F46)=1,SUM('Turns'!F46),"Unknown")</f>
-        <v>0.0001198</v>
+        <v>0.0001194</v>
       </c>
       <c r="AA15" s="5">
         <f>IF(ISNUMBER(Y15),ROUND(Y15*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5018,7 +5018,7 @@
         <v>124</v>
       </c>
       <c r="AD15" s="1">
-        <v>1986.238</v>
+        <v>1113.748</v>
       </c>
       <c r="AE15" s="1" t="s">
         <v>177</v>
@@ -5050,7 +5050,7 @@
         <v>188</v>
       </c>
       <c r="AD16" s="1">
-        <v>3.446</v>
+        <v>2.554</v>
       </c>
       <c r="AE16" s="1" t="s">
         <v>181</v>
@@ -5082,7 +5082,7 @@
         <v>190</v>
       </c>
       <c r="AD17" s="1">
-        <v>0.825</v>
+        <v>0.634</v>
       </c>
       <c r="AE17" s="1" t="s">
         <v>181</v>
@@ -5115,15 +5115,15 @@
       </c>
       <c r="J18" s="2">
         <f>IF(COUNT('Turns'!D52)=1,SUM('Turns'!D52),"Unknown")</f>
-        <v>525.0</v>
+        <v>523.0</v>
       </c>
       <c r="K18" s="2">
         <f>IF(COUNT('Turns'!E52)=1,SUM('Turns'!E52),"Unknown")</f>
-        <v>9.159885e-05</v>
+        <v>9.166621e-05</v>
       </c>
       <c r="L18" s="2">
         <f>IF(COUNT('Turns'!F52)=1,SUM('Turns'!F52),"Unknown")</f>
-        <v>0.000105</v>
+        <v>0.0001046</v>
       </c>
       <c r="M18" s="2">
         <f>IF(COUNT('Turns'!D51)=1,SUM('Turns'!D51),"Unknown")</f>
@@ -5152,7 +5152,7 @@
       </c>
       <c r="T18" s="2">
         <f>IF(COUNT('Turns'!E57)=1,SUM('Turns'!E57),"Unknown")</f>
-        <v>2.8264788e-05</v>
+        <v>2.839374e-05</v>
       </c>
       <c r="U18" s="2">
         <f>IF(COUNT('Turns'!F57)=1,SUM('Turns'!F57),"Unknown")</f>
@@ -5169,11 +5169,11 @@
       </c>
       <c r="Y18" s="2">
         <f>IF(COUNT('Turns'!E61)=1,SUM('Turns'!E61),"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00012005995</v>
       </c>
       <c r="Z18" s="2">
         <f>IF(COUNT('Turns'!F61)=1,SUM('Turns'!F61),"Unknown")</f>
-        <v>0.0001374</v>
+        <v>0.000137</v>
       </c>
       <c r="AA18" s="5">
         <f>IF(ISNUMBER(Y18),ROUND(Y18*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5184,7 +5184,7 @@
         <v>14.0</v>
       </c>
       <c r="AD18" s="1">
-        <v>1032.616</v>
+        <v>1177.623</v>
       </c>
       <c r="AE18" s="1" t="s">
         <v>164</v>
@@ -5207,7 +5207,7 @@
         <v>111</v>
       </c>
       <c r="F19" s="1">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>176</v>
@@ -5220,15 +5220,15 @@
       </c>
       <c r="J19" s="2">
         <f>IF(COUNT('Turns'!D52)=1,SUM('Turns'!D52),"Unknown")</f>
-        <v>525.0</v>
+        <v>523.0</v>
       </c>
       <c r="K19" s="2">
         <f>IF(COUNT('Turns'!E52)=1,SUM('Turns'!E52),"Unknown")</f>
-        <v>9.159885e-05</v>
+        <v>9.166621e-05</v>
       </c>
       <c r="L19" s="2">
         <f>IF(COUNT('Turns'!F52)=1,SUM('Turns'!F52),"Unknown")</f>
-        <v>0.000105</v>
+        <v>0.0001046</v>
       </c>
       <c r="M19" s="2">
         <f>IF(COUNT('Turns'!D51)=1,SUM('Turns'!D51),"Unknown")</f>
@@ -5257,7 +5257,7 @@
       </c>
       <c r="T19" s="2">
         <f>IF(COUNT('Turns'!E57)=1,SUM('Turns'!E57),"Unknown")</f>
-        <v>2.8264788e-05</v>
+        <v>2.839374e-05</v>
       </c>
       <c r="U19" s="2">
         <f>IF(COUNT('Turns'!F57)=1,SUM('Turns'!F57),"Unknown")</f>
@@ -5274,11 +5274,11 @@
       </c>
       <c r="Y19" s="2">
         <f>IF(COUNT('Turns'!E61)=1,SUM('Turns'!E61),"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00012005995</v>
       </c>
       <c r="Z19" s="2">
         <f>IF(COUNT('Turns'!F61)=1,SUM('Turns'!F61),"Unknown")</f>
-        <v>0.0001374</v>
+        <v>0.000137</v>
       </c>
       <c r="AA19" s="5">
         <f>IF(ISNUMBER(Y19),ROUND(Y19*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5292,7 +5292,7 @@
         <v>131</v>
       </c>
       <c r="AD19" s="1">
-        <v>1031.15</v>
+        <v>1175.359</v>
       </c>
       <c r="AE19" s="1" t="s">
         <v>177</v>
@@ -5322,15 +5322,15 @@
       </c>
       <c r="J20" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1292.0</v>
+        <v>1287.0</v>
       </c>
       <c r="K20" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.000225420408</v>
+        <v>0.00022557249</v>
       </c>
       <c r="L20" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.0002584</v>
+        <v>0.0002574</v>
       </c>
       <c r="M20" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5355,35 +5355,35 @@
       </c>
       <c r="S20" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>75.0</v>
+        <v>74.0</v>
       </c>
       <c r="T20" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.85133e-05</v>
+        <v>7.781988e-05</v>
       </c>
       <c r="U20" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>9e-05</v>
+        <v>8.88e-05</v>
       </c>
       <c r="V20" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="W20" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="X20" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="Y20" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000324870588</v>
+        <v>0.00032337315</v>
       </c>
       <c r="Z20" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003724</v>
+        <v>0.000369</v>
       </c>
       <c r="AA20" s="5">
         <f>IF(ISNUMBER(Y20),ROUND(Y20*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5394,7 +5394,7 @@
         <v>37.0</v>
       </c>
       <c r="AD20" s="1">
-        <v>3736.47</v>
+        <v>2707.735</v>
       </c>
       <c r="AE20" s="1" t="s">
         <v>164</v>
@@ -5427,15 +5427,15 @@
       </c>
       <c r="J21" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1292.0</v>
+        <v>1287.0</v>
       </c>
       <c r="K21" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.000225420408</v>
+        <v>0.00022557249</v>
       </c>
       <c r="L21" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.0002584</v>
+        <v>0.0002574</v>
       </c>
       <c r="M21" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5460,35 +5460,35 @@
       </c>
       <c r="S21" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>75.0</v>
+        <v>74.0</v>
       </c>
       <c r="T21" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.85133e-05</v>
+        <v>7.781988e-05</v>
       </c>
       <c r="U21" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>9e-05</v>
+        <v>8.88e-05</v>
       </c>
       <c r="V21" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="W21" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="X21" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="Y21" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000324870588</v>
+        <v>0.00032337315</v>
       </c>
       <c r="Z21" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003724</v>
+        <v>0.000369</v>
       </c>
       <c r="AA21" s="5">
         <f>IF(ISNUMBER(Y21),ROUND(Y21*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5499,7 +5499,7 @@
         <v>37.0</v>
       </c>
       <c r="AD21" s="1">
-        <v>3734.538</v>
+        <v>2705.636</v>
       </c>
       <c r="AE21" s="1" t="s">
         <v>164</v>
@@ -5532,15 +5532,15 @@
       </c>
       <c r="J22" s="2">
         <f>IF(COUNT('Turns'!D65,'Turns'!D81)=2,SUM('Turns'!D65,'Turns'!D81),"Unknown")</f>
-        <v>1292.0</v>
+        <v>1287.0</v>
       </c>
       <c r="K22" s="2">
         <f>IF(COUNT('Turns'!E65,'Turns'!E81)=2,SUM('Turns'!E65,'Turns'!E81),"Unknown")</f>
-        <v>0.000225420408</v>
+        <v>0.00022557249</v>
       </c>
       <c r="L22" s="2">
         <f>IF(COUNT('Turns'!F65,'Turns'!F81)=2,SUM('Turns'!F65,'Turns'!F81),"Unknown")</f>
-        <v>0.0002584</v>
+        <v>0.0002574</v>
       </c>
       <c r="M22" s="2">
         <f>IF(COUNT('Turns'!D64,'Turns'!D80)=2,SUM('Turns'!D64,'Turns'!D80),"Unknown")</f>
@@ -5565,35 +5565,35 @@
       </c>
       <c r="S22" s="2">
         <f>IF(COUNT('Turns'!D71,'Turns'!D86)=2,SUM('Turns'!D71,'Turns'!D86),"Unknown")</f>
-        <v>75.0</v>
+        <v>74.0</v>
       </c>
       <c r="T22" s="2">
         <f>IF(COUNT('Turns'!E71,'Turns'!E86)=2,SUM('Turns'!E71,'Turns'!E86),"Unknown")</f>
-        <v>7.85133e-05</v>
+        <v>7.781988e-05</v>
       </c>
       <c r="U22" s="2">
         <f>IF(COUNT('Turns'!F71,'Turns'!F86)=2,SUM('Turns'!F71,'Turns'!F86),"Unknown")</f>
-        <v>9e-05</v>
+        <v>8.88e-05</v>
       </c>
       <c r="V22" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="W22" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="X22" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="Y22" s="2">
         <f>IF(COUNT('Turns'!E75,'Turns'!E90)=2,SUM('Turns'!E75,'Turns'!E90),"Unknown")</f>
-        <v>0.000324870588</v>
+        <v>0.00032337315</v>
       </c>
       <c r="Z22" s="2">
         <f>IF(COUNT('Turns'!F75,'Turns'!F90)=2,SUM('Turns'!F75,'Turns'!F90),"Unknown")</f>
-        <v>0.0003724</v>
+        <v>0.000369</v>
       </c>
       <c r="AA22" s="5">
         <f>IF(ISNUMBER(Y22),ROUND(Y22*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5604,7 +5604,7 @@
         <v>37.0</v>
       </c>
       <c r="AD22" s="1">
-        <v>3732.928</v>
+        <v>2704.491</v>
       </c>
       <c r="AE22" s="1" t="s">
         <v>164</v>
@@ -5637,15 +5637,15 @@
       </c>
       <c r="J23" s="2">
         <f>IF(COUNT('Turns'!D65)=1,SUM('Turns'!D65),"Unknown")</f>
-        <v>605.0</v>
+        <v>603.0</v>
       </c>
       <c r="K23" s="2">
         <f>IF(COUNT('Turns'!E65)=1,SUM('Turns'!E65),"Unknown")</f>
-        <v>0.00010555677</v>
+        <v>0.00010568781</v>
       </c>
       <c r="L23" s="2">
         <f>IF(COUNT('Turns'!F65)=1,SUM('Turns'!F65),"Unknown")</f>
-        <v>0.000121</v>
+        <v>0.0001206</v>
       </c>
       <c r="M23" s="2">
         <f>IF(COUNT('Turns'!D64)=1,SUM('Turns'!D64),"Unknown")</f>
@@ -5674,7 +5674,7 @@
       </c>
       <c r="T23" s="2">
         <f>IF(COUNT('Turns'!E71)=1,SUM('Turns'!E71),"Unknown")</f>
-        <v>4.187376e-05</v>
+        <v>4.20648e-05</v>
       </c>
       <c r="U23" s="2">
         <f>IF(COUNT('Turns'!F71)=1,SUM('Turns'!F71),"Unknown")</f>
@@ -5682,23 +5682,23 @@
       </c>
       <c r="V23" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="W23" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="X23" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="Y23" s="2">
         <f>IF(COUNT('Turns'!E75)=1,SUM('Turns'!E75),"Unknown")</f>
-        <v>0.00016836741</v>
+        <v>0.00016773339</v>
       </c>
       <c r="Z23" s="2">
         <f>IF(COUNT('Turns'!F75)=1,SUM('Turns'!F75),"Unknown")</f>
-        <v>0.000193</v>
+        <v>0.0001914</v>
       </c>
       <c r="AA23" s="5">
         <f>IF(ISNUMBER(Y23),ROUND(Y23*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5709,7 +5709,7 @@
         <v>19.0</v>
       </c>
       <c r="AD23" s="1">
-        <v>1865.263</v>
+        <v>1509.143</v>
       </c>
       <c r="AE23" s="1" t="s">
         <v>164</v>
@@ -5732,7 +5732,7 @@
         <v>111</v>
       </c>
       <c r="F24" s="1">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>176</v>
@@ -5745,15 +5745,15 @@
       </c>
       <c r="J24" s="2">
         <f>IF(COUNT('Turns'!D65)=1,SUM('Turns'!D65),"Unknown")</f>
-        <v>605.0</v>
+        <v>603.0</v>
       </c>
       <c r="K24" s="2">
         <f>IF(COUNT('Turns'!E65)=1,SUM('Turns'!E65),"Unknown")</f>
-        <v>0.00010555677</v>
+        <v>0.00010568781</v>
       </c>
       <c r="L24" s="2">
         <f>IF(COUNT('Turns'!F65)=1,SUM('Turns'!F65),"Unknown")</f>
-        <v>0.000121</v>
+        <v>0.0001206</v>
       </c>
       <c r="M24" s="2">
         <f>IF(COUNT('Turns'!D64)=1,SUM('Turns'!D64),"Unknown")</f>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="T24" s="2">
         <f>IF(COUNT('Turns'!E71)=1,SUM('Turns'!E71),"Unknown")</f>
-        <v>4.187376e-05</v>
+        <v>4.20648e-05</v>
       </c>
       <c r="U24" s="2">
         <f>IF(COUNT('Turns'!F71)=1,SUM('Turns'!F71),"Unknown")</f>
@@ -5790,23 +5790,23 @@
       </c>
       <c r="V24" s="2">
         <f>IF(COUNT('Turns'!D70)=1,SUM('Turns'!D70),"Unknown")</f>
-        <v>20.0</v>
+        <v>19.0</v>
       </c>
       <c r="W24" s="2">
         <f>IF(COUNT('Turns'!E70)=1,SUM('Turns'!E70),"Unknown")</f>
-        <v>2.093688e-05</v>
+        <v>1.998078e-05</v>
       </c>
       <c r="X24" s="2">
         <f>IF(COUNT('Turns'!F70)=1,SUM('Turns'!F70),"Unknown")</f>
-        <v>2.4e-05</v>
+        <v>2.28e-05</v>
       </c>
       <c r="Y24" s="2">
         <f>IF(COUNT('Turns'!E75)=1,SUM('Turns'!E75),"Unknown")</f>
-        <v>0.00016836741</v>
+        <v>0.00016773339</v>
       </c>
       <c r="Z24" s="2">
         <f>IF(COUNT('Turns'!F75)=1,SUM('Turns'!F75),"Unknown")</f>
-        <v>0.000193</v>
+        <v>0.0001914</v>
       </c>
       <c r="AA24" s="5">
         <f>IF(ISNUMBER(Y24),ROUND(Y24*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5820,7 +5820,7 @@
         <v>135</v>
       </c>
       <c r="AD24" s="1">
-        <v>1863.739</v>
+        <v>1506.63</v>
       </c>
       <c r="AE24" s="1" t="s">
         <v>177</v>
@@ -5852,7 +5852,7 @@
         <v>196</v>
       </c>
       <c r="AD25" s="1">
-        <v>1.923</v>
+        <v>3.986</v>
       </c>
       <c r="AE25" s="1" t="s">
         <v>181</v>
@@ -5884,7 +5884,7 @@
         <v>198</v>
       </c>
       <c r="AD26" s="1">
-        <v>0.491</v>
+        <v>1</v>
       </c>
       <c r="AE26" s="1" t="s">
         <v>181</v>
@@ -5917,15 +5917,15 @@
       </c>
       <c r="J27" s="2">
         <f>IF(COUNT('Turns'!D81)=1,SUM('Turns'!D81),"Unknown")</f>
-        <v>687.0</v>
+        <v>684.0</v>
       </c>
       <c r="K27" s="2">
         <f>IF(COUNT('Turns'!E81)=1,SUM('Turns'!E81),"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00011988468</v>
       </c>
       <c r="L27" s="2">
         <f>IF(COUNT('Turns'!F81)=1,SUM('Turns'!F81),"Unknown")</f>
-        <v>0.0001374</v>
+        <v>0.0001368</v>
       </c>
       <c r="M27" s="2">
         <f>IF(COUNT('Turns'!D80)=1,SUM('Turns'!D80),"Unknown")</f>
@@ -5950,15 +5950,15 @@
       </c>
       <c r="S27" s="2">
         <f>IF(COUNT('Turns'!D86)=1,SUM('Turns'!D86),"Unknown")</f>
-        <v>35.0</v>
+        <v>34.0</v>
       </c>
       <c r="T27" s="2">
         <f>IF(COUNT('Turns'!E86)=1,SUM('Turns'!E86),"Unknown")</f>
-        <v>3.663954e-05</v>
+        <v>3.575508e-05</v>
       </c>
       <c r="U27" s="2">
         <f>IF(COUNT('Turns'!F86)=1,SUM('Turns'!F86),"Unknown")</f>
-        <v>4.2e-05</v>
+        <v>4.08e-05</v>
       </c>
       <c r="V27" s="2">
         <v>0</v>
@@ -5971,11 +5971,11 @@
       </c>
       <c r="Y27" s="2">
         <f>IF(COUNT('Turns'!E90)=1,SUM('Turns'!E90),"Unknown")</f>
-        <v>0.000156503178</v>
+        <v>0.00015563976</v>
       </c>
       <c r="Z27" s="2">
         <f>IF(COUNT('Turns'!F90)=1,SUM('Turns'!F90),"Unknown")</f>
-        <v>0.0001794</v>
+        <v>0.0001776</v>
       </c>
       <c r="AA27" s="5">
         <f>IF(ISNUMBER(Y27),ROUND(Y27*'Reference data'!$B$2,0),"Unknown")</f>
@@ -5986,7 +5986,7 @@
         <v>18.0</v>
       </c>
       <c r="AD27" s="1">
-        <v>1854.326</v>
+        <v>1186.002</v>
       </c>
       <c r="AE27" s="1" t="s">
         <v>164</v>
@@ -6009,7 +6009,7 @@
         <v>111</v>
       </c>
       <c r="F28" s="1">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="G28" s="6" t="s">
         <v>176</v>
@@ -6022,15 +6022,15 @@
       </c>
       <c r="J28" s="2">
         <f>IF(COUNT('Turns'!D81)=1,SUM('Turns'!D81),"Unknown")</f>
-        <v>687.0</v>
+        <v>684.0</v>
       </c>
       <c r="K28" s="2">
         <f>IF(COUNT('Turns'!E81)=1,SUM('Turns'!E81),"Unknown")</f>
-        <v>0.000119863638</v>
+        <v>0.00011988468</v>
       </c>
       <c r="L28" s="2">
         <f>IF(COUNT('Turns'!F81)=1,SUM('Turns'!F81),"Unknown")</f>
-        <v>0.0001374</v>
+        <v>0.0001368</v>
       </c>
       <c r="M28" s="2">
         <f>IF(COUNT('Turns'!D80)=1,SUM('Turns'!D80),"Unknown")</f>
@@ -6055,15 +6055,15 @@
       </c>
       <c r="S28" s="2">
         <f>IF(COUNT('Turns'!D86)=1,SUM('Turns'!D86),"Unknown")</f>
-        <v>35.0</v>
+        <v>34.0</v>
       </c>
       <c r="T28" s="2">
         <f>IF(COUNT('Turns'!E86)=1,SUM('Turns'!E86),"Unknown")</f>
-        <v>3.663954e-05</v>
+        <v>3.575508e-05</v>
       </c>
       <c r="U28" s="2">
         <f>IF(COUNT('Turns'!F86)=1,SUM('Turns'!F86),"Unknown")</f>
-        <v>4.2e-05</v>
+        <v>4.08e-05</v>
       </c>
       <c r="V28" s="2">
         <v>0</v>
@@ -6076,11 +6076,11 @@
       </c>
       <c r="Y28" s="2">
         <f>IF(COUNT('Turns'!E90)=1,SUM('Turns'!E90),"Unknown")</f>
-        <v>0.000156503178</v>
+        <v>0.00015563976</v>
       </c>
       <c r="Z28" s="2">
         <f>IF(COUNT('Turns'!F90)=1,SUM('Turns'!F90),"Unknown")</f>
-        <v>0.0001794</v>
+        <v>0.0001776</v>
       </c>
       <c r="AA28" s="5">
         <f>IF(ISNUMBER(Y28),ROUND(Y28*'Reference data'!$B$2,0),"Unknown")</f>
@@ -6094,7 +6094,7 @@
         <v>143</v>
       </c>
       <c r="AD28" s="1">
-        <v>1840.509</v>
+        <v>1183.058</v>
       </c>
       <c r="AE28" s="1" t="s">
         <v>177</v>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="K29" s="2">
         <f>IF(COUNT('Turns'!E94)=1,SUM('Turns'!E94),"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="L29" s="2">
         <f>IF(COUNT('Turns'!F94)=1,SUM('Turns'!F94),"Unknown")</f>
@@ -6161,7 +6161,7 @@
       </c>
       <c r="T29" s="2">
         <f>IF(COUNT('Turns'!E100)=1,SUM('Turns'!E100),"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="U29" s="2">
         <f>IF(COUNT('Turns'!F100)=1,SUM('Turns'!F100),"Unknown")</f>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="Y29" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="Z29" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -6193,7 +6193,7 @@
         <v>11.0</v>
       </c>
       <c r="AD29" s="1">
-        <v>990.8049999999999</v>
+        <v>908.564</v>
       </c>
       <c r="AE29" s="1" t="s">
         <v>164</v>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="K30" s="2">
         <f>IF(COUNT('Turns'!E94)=1,SUM('Turns'!E94),"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="L30" s="2">
         <f>IF(COUNT('Turns'!F94)=1,SUM('Turns'!F94),"Unknown")</f>
@@ -6263,7 +6263,7 @@
       </c>
       <c r="T30" s="2">
         <f>IF(COUNT('Turns'!E100)=1,SUM('Turns'!E100),"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="U30" s="2">
         <f>IF(COUNT('Turns'!F100)=1,SUM('Turns'!F100),"Unknown")</f>
@@ -6280,7 +6280,7 @@
       </c>
       <c r="Y30" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="Z30" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -6295,7 +6295,7 @@
         <v>11.0</v>
       </c>
       <c r="AD30" s="1">
-        <v>988.484</v>
+        <v>906.515</v>
       </c>
       <c r="AE30" s="1" t="s">
         <v>164</v>
@@ -6332,7 +6332,7 @@
       </c>
       <c r="K31" s="2">
         <f>IF(COUNT('Turns'!E94)=1,SUM('Turns'!E94),"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="L31" s="2">
         <f>IF(COUNT('Turns'!F94)=1,SUM('Turns'!F94),"Unknown")</f>
@@ -6365,7 +6365,7 @@
       </c>
       <c r="T31" s="2">
         <f>IF(COUNT('Turns'!E100)=1,SUM('Turns'!E100),"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="U31" s="2">
         <f>IF(COUNT('Turns'!F100)=1,SUM('Turns'!F100),"Unknown")</f>
@@ -6382,7 +6382,7 @@
       </c>
       <c r="Y31" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="Z31" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -6397,7 +6397,7 @@
         <v>11.0</v>
       </c>
       <c r="AD31" s="1">
-        <v>987.3869999999999</v>
+        <v>905.61</v>
       </c>
       <c r="AE31" s="1" t="s">
         <v>164</v>
@@ -6434,7 +6434,7 @@
       </c>
       <c r="K32" s="2">
         <f>IF(COUNT('Turns'!E94)=1,SUM('Turns'!E94),"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="L32" s="2">
         <f>IF(COUNT('Turns'!F94)=1,SUM('Turns'!F94),"Unknown")</f>
@@ -6467,7 +6467,7 @@
       </c>
       <c r="T32" s="2">
         <f>IF(COUNT('Turns'!E100)=1,SUM('Turns'!E100),"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="U32" s="2">
         <f>IF(COUNT('Turns'!F100)=1,SUM('Turns'!F100),"Unknown")</f>
@@ -6484,7 +6484,7 @@
       </c>
       <c r="Y32" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="Z32" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -6499,7 +6499,7 @@
         <v>11.0</v>
       </c>
       <c r="AD32" s="1">
-        <v>985.467</v>
+        <v>903.63</v>
       </c>
       <c r="AE32" s="1" t="s">
         <v>164</v>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="K33" s="2">
         <f>IF(COUNT('Turns'!E94)=1,SUM('Turns'!E94),"Unknown")</f>
-        <v>7.502382e-05</v>
+        <v>7.53661e-05</v>
       </c>
       <c r="L33" s="2">
         <f>IF(COUNT('Turns'!F94)=1,SUM('Turns'!F94),"Unknown")</f>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="T33" s="2">
         <f>IF(COUNT('Turns'!E100)=1,SUM('Turns'!E100),"Unknown")</f>
-        <v>1.8843192e-05</v>
+        <v>1.892916e-05</v>
       </c>
       <c r="U33" s="2">
         <f>IF(COUNT('Turns'!F100)=1,SUM('Turns'!F100),"Unknown")</f>
@@ -6589,7 +6589,7 @@
       </c>
       <c r="Y33" s="2">
         <f>IF(COUNT('Turns'!E104)=1,SUM('Turns'!E104),"Unknown")</f>
-        <v>9.3867012e-05</v>
+        <v>9.429526e-05</v>
       </c>
       <c r="Z33" s="2">
         <f>IF(COUNT('Turns'!F104)=1,SUM('Turns'!F104),"Unknown")</f>
@@ -6607,7 +6607,7 @@
         <v>147</v>
       </c>
       <c r="AD33" s="1">
-        <v>983.5170000000001</v>
+        <v>901.8049999999999</v>
       </c>
       <c r="AE33" s="1" t="s">
         <v>177</v>
@@ -6637,15 +6637,15 @@
       </c>
       <c r="J34" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1026.0</v>
+        <v>1022.0</v>
       </c>
       <c r="K34" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000179010324</v>
+        <v>0.00017912594</v>
       </c>
       <c r="L34" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002052</v>
+        <v>0.0002044</v>
       </c>
       <c r="M34" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6670,35 +6670,35 @@
       </c>
       <c r="S34" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>45.0</v>
+        <v>47.0</v>
       </c>
       <c r="T34" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.710798e-05</v>
+        <v>4.942614e-05</v>
       </c>
       <c r="U34" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.4e-05</v>
+        <v>5.64e-05</v>
       </c>
       <c r="V34" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="W34" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X34" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y34" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00024077412</v>
+        <v>0.00023906828</v>
       </c>
       <c r="Z34" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.000276</v>
+        <v>0.0002728</v>
       </c>
       <c r="AA34" s="5">
         <f>IF(ISNUMBER(Y34),ROUND(Y34*'Reference data'!$B$2,0),"Unknown")</f>
@@ -6706,10 +6706,10 @@
       </c>
       <c r="AB34" s="5">
         <f>IF(ISNUMBER(Z34),ROUND(Z34*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
       <c r="AD34" s="1">
-        <v>2761.857</v>
+        <v>2089.984</v>
       </c>
       <c r="AE34" s="1" t="s">
         <v>164</v>
@@ -6742,15 +6742,15 @@
       </c>
       <c r="J35" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1026.0</v>
+        <v>1022.0</v>
       </c>
       <c r="K35" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000179010324</v>
+        <v>0.00017912594</v>
       </c>
       <c r="L35" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002052</v>
+        <v>0.0002044</v>
       </c>
       <c r="M35" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6775,35 +6775,35 @@
       </c>
       <c r="S35" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>45.0</v>
+        <v>47.0</v>
       </c>
       <c r="T35" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.710798e-05</v>
+        <v>4.942614e-05</v>
       </c>
       <c r="U35" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.4e-05</v>
+        <v>5.64e-05</v>
       </c>
       <c r="V35" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="W35" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X35" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y35" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00024077412</v>
+        <v>0.00023906828</v>
       </c>
       <c r="Z35" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.000276</v>
+        <v>0.0002728</v>
       </c>
       <c r="AA35" s="5">
         <f>IF(ISNUMBER(Y35),ROUND(Y35*'Reference data'!$B$2,0),"Unknown")</f>
@@ -6811,10 +6811,10 @@
       </c>
       <c r="AB35" s="5">
         <f>IF(ISNUMBER(Z35),ROUND(Z35*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
       <c r="AD35" s="1">
-        <v>2758.871</v>
+        <v>2088.28</v>
       </c>
       <c r="AE35" s="1" t="s">
         <v>164</v>
@@ -6847,15 +6847,15 @@
       </c>
       <c r="J36" s="2">
         <f>IF(COUNT('Turns'!D108,'Turns'!D124)=2,SUM('Turns'!D108,'Turns'!D124),"Unknown")</f>
-        <v>1026.0</v>
+        <v>1022.0</v>
       </c>
       <c r="K36" s="2">
         <f>IF(COUNT('Turns'!E108,'Turns'!E124)=2,SUM('Turns'!E108,'Turns'!E124),"Unknown")</f>
-        <v>0.000179010324</v>
+        <v>0.00017912594</v>
       </c>
       <c r="L36" s="2">
         <f>IF(COUNT('Turns'!F108,'Turns'!F124)=2,SUM('Turns'!F108,'Turns'!F124),"Unknown")</f>
-        <v>0.0002052</v>
+        <v>0.0002044</v>
       </c>
       <c r="M36" s="2">
         <f>IF(COUNT('Turns'!D107,'Turns'!D123)=2,SUM('Turns'!D107,'Turns'!D123),"Unknown")</f>
@@ -6880,35 +6880,35 @@
       </c>
       <c r="S36" s="2">
         <f>IF(COUNT('Turns'!D114,'Turns'!D129)=2,SUM('Turns'!D114,'Turns'!D129),"Unknown")</f>
-        <v>45.0</v>
+        <v>47.0</v>
       </c>
       <c r="T36" s="2">
         <f>IF(COUNT('Turns'!E114,'Turns'!E129)=2,SUM('Turns'!E114,'Turns'!E129),"Unknown")</f>
-        <v>4.710798e-05</v>
+        <v>4.942614e-05</v>
       </c>
       <c r="U36" s="2">
         <f>IF(COUNT('Turns'!F114,'Turns'!F129)=2,SUM('Turns'!F114,'Turns'!F129),"Unknown")</f>
-        <v>5.4e-05</v>
+        <v>5.64e-05</v>
       </c>
       <c r="V36" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="W36" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X36" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y36" s="2">
         <f>IF(COUNT('Turns'!E118,'Turns'!E133)=2,SUM('Turns'!E118,'Turns'!E133),"Unknown")</f>
-        <v>0.00024077412</v>
+        <v>0.00023906828</v>
       </c>
       <c r="Z36" s="2">
         <f>IF(COUNT('Turns'!F118,'Turns'!F133)=2,SUM('Turns'!F118,'Turns'!F133),"Unknown")</f>
-        <v>0.000276</v>
+        <v>0.0002728</v>
       </c>
       <c r="AA36" s="5">
         <f>IF(ISNUMBER(Y36),ROUND(Y36*'Reference data'!$B$2,0),"Unknown")</f>
@@ -6916,10 +6916,10 @@
       </c>
       <c r="AB36" s="5">
         <f>IF(ISNUMBER(Z36),ROUND(Z36*'Reference data'!$B$2,0),"Unknown")</f>
-        <v>28.0</v>
+        <v>27.0</v>
       </c>
       <c r="AD36" s="1">
-        <v>2757.654</v>
+        <v>2087.515</v>
       </c>
       <c r="AE36" s="1" t="s">
         <v>164</v>
@@ -6956,7 +6956,7 @@
       </c>
       <c r="K37" s="2">
         <f>IF(COUNT('Turns'!E108)=1,SUM('Turns'!E108),"Unknown")</f>
-        <v>8.2526202e-05</v>
+        <v>8.290271e-05</v>
       </c>
       <c r="L37" s="2">
         <f>IF(COUNT('Turns'!F108)=1,SUM('Turns'!F108),"Unknown")</f>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="T37" s="2">
         <f>IF(COUNT('Turns'!E114)=1,SUM('Turns'!E114),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U37" s="2">
         <f>IF(COUNT('Turns'!F114)=1,SUM('Turns'!F114),"Unknown")</f>
@@ -6997,23 +6997,23 @@
       </c>
       <c r="V37" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="W37" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X37" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y37" s="2">
         <f>IF(COUNT('Turns'!E118)=1,SUM('Turns'!E118),"Unknown")</f>
-        <v>0.000113931522</v>
+        <v>0.00011024483</v>
       </c>
       <c r="Z37" s="2">
         <f>IF(COUNT('Turns'!F118)=1,SUM('Turns'!F118),"Unknown")</f>
-        <v>0.0001306</v>
+        <v>0.0001258</v>
       </c>
       <c r="AA37" s="5">
         <f>IF(ISNUMBER(Y37),ROUND(Y37*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7024,7 +7024,7 @@
         <v>13.0</v>
       </c>
       <c r="AD37" s="1">
-        <v>1506.315</v>
+        <v>1009.675</v>
       </c>
       <c r="AE37" s="1" t="s">
         <v>164</v>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="K38" s="2">
         <f>IF(COUNT('Turns'!E108)=1,SUM('Turns'!E108),"Unknown")</f>
-        <v>8.2526202e-05</v>
+        <v>8.290271e-05</v>
       </c>
       <c r="L38" s="2">
         <f>IF(COUNT('Turns'!F108)=1,SUM('Turns'!F108),"Unknown")</f>
@@ -7097,7 +7097,7 @@
       </c>
       <c r="T38" s="2">
         <f>IF(COUNT('Turns'!E114)=1,SUM('Turns'!E114),"Unknown")</f>
-        <v>1.6749504e-05</v>
+        <v>1.682592e-05</v>
       </c>
       <c r="U38" s="2">
         <f>IF(COUNT('Turns'!F114)=1,SUM('Turns'!F114),"Unknown")</f>
@@ -7105,23 +7105,23 @@
       </c>
       <c r="V38" s="2">
         <f>IF(COUNT('Turns'!D113)=1,SUM('Turns'!D113),"Unknown")</f>
-        <v>14.0</v>
+        <v>10.0</v>
       </c>
       <c r="W38" s="2">
         <f>IF(COUNT('Turns'!E113)=1,SUM('Turns'!E113),"Unknown")</f>
-        <v>1.4655816e-05</v>
+        <v>1.05162e-05</v>
       </c>
       <c r="X38" s="2">
         <f>IF(COUNT('Turns'!F113)=1,SUM('Turns'!F113),"Unknown")</f>
-        <v>1.68e-05</v>
+        <v>1.2e-05</v>
       </c>
       <c r="Y38" s="2">
         <f>IF(COUNT('Turns'!E118)=1,SUM('Turns'!E118),"Unknown")</f>
-        <v>0.000113931522</v>
+        <v>0.00011024483</v>
       </c>
       <c r="Z38" s="2">
         <f>IF(COUNT('Turns'!F118)=1,SUM('Turns'!F118),"Unknown")</f>
-        <v>0.0001306</v>
+        <v>0.0001258</v>
       </c>
       <c r="AA38" s="5">
         <f>IF(ISNUMBER(Y38),ROUND(Y38*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7135,7 +7135,7 @@
         <v>152</v>
       </c>
       <c r="AD38" s="1">
-        <v>1504.393</v>
+        <v>1007.747</v>
       </c>
       <c r="AE38" s="1" t="s">
         <v>177</v>
@@ -7167,7 +7167,7 @@
         <v>208</v>
       </c>
       <c r="AD39" s="1">
-        <v>2.889</v>
+        <v>1.457</v>
       </c>
       <c r="AE39" s="1" t="s">
         <v>181</v>
@@ -7199,7 +7199,7 @@
         <v>210</v>
       </c>
       <c r="AD40" s="1">
-        <v>0.5620000000000001</v>
+        <v>0.403</v>
       </c>
       <c r="AE40" s="1" t="s">
         <v>181</v>
@@ -7232,15 +7232,15 @@
       </c>
       <c r="J41" s="2">
         <f>IF(COUNT('Turns'!D124)=1,SUM('Turns'!D124),"Unknown")</f>
-        <v>553.0</v>
+        <v>549.0</v>
       </c>
       <c r="K41" s="2">
         <f>IF(COUNT('Turns'!E124)=1,SUM('Turns'!E124),"Unknown")</f>
-        <v>9.6484122e-05</v>
+        <v>9.622323e-05</v>
       </c>
       <c r="L41" s="2">
         <f>IF(COUNT('Turns'!F124)=1,SUM('Turns'!F124),"Unknown")</f>
-        <v>0.0001106</v>
+        <v>0.0001098</v>
       </c>
       <c r="M41" s="2">
         <f>IF(COUNT('Turns'!D123)=1,SUM('Turns'!D123),"Unknown")</f>
@@ -7265,15 +7265,15 @@
       </c>
       <c r="S41" s="2">
         <f>IF(COUNT('Turns'!D129)=1,SUM('Turns'!D129),"Unknown")</f>
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
       <c r="T41" s="2">
         <f>IF(COUNT('Turns'!E129)=1,SUM('Turns'!E129),"Unknown")</f>
-        <v>3.0358476e-05</v>
+        <v>3.260022e-05</v>
       </c>
       <c r="U41" s="2">
         <f>IF(COUNT('Turns'!F129)=1,SUM('Turns'!F129),"Unknown")</f>
-        <v>3.48e-05</v>
+        <v>3.72e-05</v>
       </c>
       <c r="V41" s="2">
         <v>0</v>
@@ -7286,11 +7286,11 @@
       </c>
       <c r="Y41" s="2">
         <f>IF(COUNT('Turns'!E133)=1,SUM('Turns'!E133),"Unknown")</f>
-        <v>0.000126842598</v>
+        <v>0.00012882345</v>
       </c>
       <c r="Z41" s="2">
         <f>IF(COUNT('Turns'!F133)=1,SUM('Turns'!F133),"Unknown")</f>
-        <v>0.0001454</v>
+        <v>0.000147</v>
       </c>
       <c r="AA41" s="5">
         <f>IF(ISNUMBER(Y41),ROUND(Y41*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7301,7 +7301,7 @@
         <v>15.0</v>
       </c>
       <c r="AD41" s="1">
-        <v>1244.071</v>
+        <v>1073.735</v>
       </c>
       <c r="AE41" s="1" t="s">
         <v>164</v>
@@ -7324,7 +7324,7 @@
         <v>111</v>
       </c>
       <c r="F42" s="1">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>176</v>
@@ -7337,15 +7337,15 @@
       </c>
       <c r="J42" s="2">
         <f>IF(COUNT('Turns'!D124)=1,SUM('Turns'!D124),"Unknown")</f>
-        <v>553.0</v>
+        <v>549.0</v>
       </c>
       <c r="K42" s="2">
         <f>IF(COUNT('Turns'!E124)=1,SUM('Turns'!E124),"Unknown")</f>
-        <v>9.6484122e-05</v>
+        <v>9.622323e-05</v>
       </c>
       <c r="L42" s="2">
         <f>IF(COUNT('Turns'!F124)=1,SUM('Turns'!F124),"Unknown")</f>
-        <v>0.0001106</v>
+        <v>0.0001098</v>
       </c>
       <c r="M42" s="2">
         <f>IF(COUNT('Turns'!D123)=1,SUM('Turns'!D123),"Unknown")</f>
@@ -7370,15 +7370,15 @@
       </c>
       <c r="S42" s="2">
         <f>IF(COUNT('Turns'!D129)=1,SUM('Turns'!D129),"Unknown")</f>
-        <v>29.0</v>
+        <v>31.0</v>
       </c>
       <c r="T42" s="2">
         <f>IF(COUNT('Turns'!E129)=1,SUM('Turns'!E129),"Unknown")</f>
-        <v>3.0358476e-05</v>
+        <v>3.260022e-05</v>
       </c>
       <c r="U42" s="2">
         <f>IF(COUNT('Turns'!F129)=1,SUM('Turns'!F129),"Unknown")</f>
-        <v>3.48e-05</v>
+        <v>3.72e-05</v>
       </c>
       <c r="V42" s="2">
         <v>0</v>
@@ -7391,11 +7391,11 @@
       </c>
       <c r="Y42" s="2">
         <f>IF(COUNT('Turns'!E133)=1,SUM('Turns'!E133),"Unknown")</f>
-        <v>0.000126842598</v>
+        <v>0.00012882345</v>
       </c>
       <c r="Z42" s="2">
         <f>IF(COUNT('Turns'!F133)=1,SUM('Turns'!F133),"Unknown")</f>
-        <v>0.0001454</v>
+        <v>0.000147</v>
       </c>
       <c r="AA42" s="5">
         <f>IF(ISNUMBER(Y42),ROUND(Y42*'Reference data'!$B$2,0),"Unknown")</f>
@@ -7409,7 +7409,7 @@
         <v>158</v>
       </c>
       <c r="AD42" s="1">
-        <v>1242.056</v>
+        <v>1072.587</v>
       </c>
       <c r="AE42" s="1" t="s">
         <v>177</v>
@@ -7467,7 +7467,7 @@
         <v>43</v>
       </c>
       <c r="B3" s="2">
-        <v>0.87237</v>
+        <v>0.87635</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>44</v>

</xml_diff>